<commit_message>
Release 1.0.11: templates update and updater/spellchecker fixes
</commit_message>
<xml_diff>
--- a/templates/contratacion_incluyente.xlsx
+++ b/templates/contratacion_incluyente.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aaron\Desktop\RECA_INCLUSION_LABORAL\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED902101-9E51-4D9A-971A-5FE56C184C79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28DCAD81-B6FD-413F-97CF-3461C2DAD74C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1652,49 +1652,134 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1713,17 +1798,23 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1731,13 +1822,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1751,106 +1835,22 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3512,48 +3512,48 @@
       <c r="P1" s="4"/>
       <c r="Q1" s="4"/>
       <c r="R1" s="4"/>
-      <c r="S1" s="53" t="s">
+      <c r="S1" s="131" t="s">
         <v>3</v>
       </c>
-      <c r="T1" s="54"/>
-      <c r="U1" s="54"/>
-      <c r="V1" s="54"/>
-      <c r="W1" s="53" t="s">
+      <c r="T1" s="58"/>
+      <c r="U1" s="58"/>
+      <c r="V1" s="58"/>
+      <c r="W1" s="131" t="s">
         <v>4</v>
       </c>
-      <c r="X1" s="54"/>
-      <c r="Y1" s="54"/>
-      <c r="Z1" s="54"/>
-      <c r="AA1" s="53" t="s">
+      <c r="X1" s="58"/>
+      <c r="Y1" s="58"/>
+      <c r="Z1" s="58"/>
+      <c r="AA1" s="131" t="s">
         <v>5</v>
       </c>
-      <c r="AB1" s="54"/>
-      <c r="AC1" s="54"/>
-      <c r="AD1" s="54"/>
-      <c r="AE1" s="53" t="s">
+      <c r="AB1" s="58"/>
+      <c r="AC1" s="58"/>
+      <c r="AD1" s="58"/>
+      <c r="AE1" s="131" t="s">
         <v>6</v>
       </c>
-      <c r="AF1" s="54"/>
-      <c r="AG1" s="54"/>
-      <c r="AH1" s="54"/>
-      <c r="AI1" s="53" t="s">
+      <c r="AF1" s="58"/>
+      <c r="AG1" s="58"/>
+      <c r="AH1" s="58"/>
+      <c r="AI1" s="131" t="s">
         <v>7</v>
       </c>
-      <c r="AJ1" s="54"/>
-      <c r="AK1" s="54"/>
-      <c r="AL1" s="54"/>
-      <c r="AM1" s="53" t="s">
+      <c r="AJ1" s="58"/>
+      <c r="AK1" s="58"/>
+      <c r="AL1" s="58"/>
+      <c r="AM1" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="AN1" s="54"/>
-      <c r="AO1" s="54"/>
-      <c r="AP1" s="54"/>
+      <c r="AN1" s="58"/>
+      <c r="AO1" s="58"/>
+      <c r="AP1" s="58"/>
       <c r="AQ1" s="4"/>
-      <c r="AR1" s="53" t="s">
+      <c r="AR1" s="131" t="s">
         <v>9</v>
       </c>
-      <c r="AS1" s="54"/>
-      <c r="AT1" s="54"/>
+      <c r="AS1" s="58"/>
+      <c r="AT1" s="58"/>
       <c r="AU1" s="4"/>
       <c r="AV1" s="4"/>
       <c r="AW1" s="4"/>
@@ -3634,11 +3634,11 @@
       <c r="AO2" s="7"/>
       <c r="AP2" s="7"/>
       <c r="AQ2" s="7"/>
-      <c r="AR2" s="53" t="s">
+      <c r="AR2" s="131" t="s">
         <v>18</v>
       </c>
-      <c r="AS2" s="54"/>
-      <c r="AT2" s="54"/>
+      <c r="AS2" s="58"/>
+      <c r="AT2" s="58"/>
       <c r="AU2" s="7"/>
       <c r="AV2" s="7"/>
       <c r="AW2" s="7"/>
@@ -3718,11 +3718,11 @@
       <c r="AO3" s="7"/>
       <c r="AP3" s="7"/>
       <c r="AQ3" s="7"/>
-      <c r="AR3" s="53" t="s">
+      <c r="AR3" s="131" t="s">
         <v>25</v>
       </c>
-      <c r="AS3" s="54"/>
-      <c r="AT3" s="54"/>
+      <c r="AS3" s="58"/>
+      <c r="AT3" s="58"/>
       <c r="AU3" s="7"/>
       <c r="AV3" s="7"/>
       <c r="AW3" s="7"/>
@@ -3802,11 +3802,11 @@
       <c r="AO4" s="7"/>
       <c r="AP4" s="7"/>
       <c r="AQ4" s="7"/>
-      <c r="AR4" s="53" t="s">
+      <c r="AR4" s="131" t="s">
         <v>29</v>
       </c>
-      <c r="AS4" s="54"/>
-      <c r="AT4" s="54"/>
+      <c r="AS4" s="58"/>
+      <c r="AT4" s="58"/>
       <c r="AU4" s="7"/>
       <c r="AV4" s="7"/>
       <c r="AW4" s="7"/>
@@ -3886,11 +3886,11 @@
       <c r="AO5" s="7"/>
       <c r="AP5" s="7"/>
       <c r="AQ5" s="7"/>
-      <c r="AR5" s="53" t="s">
+      <c r="AR5" s="131" t="s">
         <v>34</v>
       </c>
-      <c r="AS5" s="54"/>
-      <c r="AT5" s="54"/>
+      <c r="AS5" s="58"/>
+      <c r="AT5" s="58"/>
       <c r="AU5" s="7"/>
       <c r="AV5" s="7"/>
       <c r="AW5" s="7"/>
@@ -3964,11 +3964,11 @@
       <c r="AO6" s="7"/>
       <c r="AP6" s="7"/>
       <c r="AQ6" s="7"/>
-      <c r="AR6" s="53" t="s">
+      <c r="AR6" s="131" t="s">
         <v>37</v>
       </c>
-      <c r="AS6" s="54"/>
-      <c r="AT6" s="54"/>
+      <c r="AS6" s="58"/>
+      <c r="AT6" s="58"/>
       <c r="AU6" s="7"/>
       <c r="AV6" s="7"/>
       <c r="AW6" s="7"/>
@@ -5920,31 +5920,31 @@
       <c r="A75" s="34" t="s">
         <v>134</v>
       </c>
-      <c r="B75" s="55" t="s">
+      <c r="B75" s="132" t="s">
         <v>135</v>
       </c>
-      <c r="C75" s="56"/>
-      <c r="D75" s="57"/>
+      <c r="C75" s="54"/>
+      <c r="D75" s="72"/>
     </row>
     <row r="76" spans="1:4" ht="25.5">
       <c r="A76" s="35" t="s">
         <v>136</v>
       </c>
-      <c r="B76" s="55" t="s">
+      <c r="B76" s="132" t="s">
         <v>137</v>
       </c>
-      <c r="C76" s="56"/>
-      <c r="D76" s="57"/>
+      <c r="C76" s="54"/>
+      <c r="D76" s="72"/>
     </row>
     <row r="77" spans="1:4" ht="12.75">
       <c r="A77" s="36" t="s">
         <v>138</v>
       </c>
-      <c r="B77" s="55" t="s">
+      <c r="B77" s="132" t="s">
         <v>139</v>
       </c>
-      <c r="C77" s="56"/>
-      <c r="D77" s="57"/>
+      <c r="C77" s="54"/>
+      <c r="D77" s="72"/>
     </row>
     <row r="82" spans="1:5" ht="17.25">
       <c r="A82" s="3" t="str">
@@ -12704,21 +12704,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="AR2:AT2"/>
+    <mergeCell ref="AR3:AT3"/>
+    <mergeCell ref="AR4:AT4"/>
+    <mergeCell ref="AR5:AT5"/>
+    <mergeCell ref="AR6:AT6"/>
+    <mergeCell ref="B75:D75"/>
+    <mergeCell ref="B76:D76"/>
+    <mergeCell ref="B77:D77"/>
+    <mergeCell ref="S1:V1"/>
+    <mergeCell ref="W1:Z1"/>
     <mergeCell ref="AA1:AD1"/>
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="AM1:AP1"/>
     <mergeCell ref="AR1:AT1"/>
-    <mergeCell ref="B75:D75"/>
-    <mergeCell ref="B76:D76"/>
-    <mergeCell ref="B77:D77"/>
-    <mergeCell ref="S1:V1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="AR2:AT2"/>
-    <mergeCell ref="AR3:AT3"/>
-    <mergeCell ref="AR4:AT4"/>
-    <mergeCell ref="AR5:AT5"/>
-    <mergeCell ref="AR6:AT6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A156" r:id="rId1" display="http://falabella.com/" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -12756,25 +12756,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12.75">
-      <c r="A1" s="85" t="e" vm="1">
+      <c r="A1" s="122" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="87"/>
-      <c r="F1" s="93" t="s">
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="123" t="s">
         <v>172</v>
       </c>
-      <c r="G1" s="86"/>
-      <c r="H1" s="86"/>
-      <c r="I1" s="86"/>
-      <c r="J1" s="86"/>
-      <c r="K1" s="86"/>
-      <c r="L1" s="86"/>
-      <c r="M1" s="86"/>
-      <c r="N1" s="86"/>
-      <c r="O1" s="87"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="79"/>
       <c r="P1" s="41" t="s">
         <v>141</v>
       </c>
@@ -12783,21 +12783,21 @@
       </c>
     </row>
     <row r="2" spans="1:17" ht="12.75">
-      <c r="A2" s="88"/>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="89"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="M2" s="54"/>
-      <c r="N2" s="54"/>
-      <c r="O2" s="89"/>
+      <c r="A2" s="57"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="80"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="80"/>
       <c r="P2" s="43" t="s">
         <v>174</v>
       </c>
@@ -12806,21 +12806,21 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="12.75">
-      <c r="A3" s="88"/>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="88"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="54"/>
-      <c r="L3" s="54"/>
-      <c r="M3" s="54"/>
-      <c r="N3" s="54"/>
-      <c r="O3" s="89"/>
+      <c r="A3" s="57"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="58"/>
+      <c r="L3" s="58"/>
+      <c r="M3" s="58"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="80"/>
       <c r="P3" s="43" t="s">
         <v>175</v>
       </c>
@@ -12829,1601 +12829,1741 @@
       </c>
     </row>
     <row r="4" spans="1:17" ht="12.75">
-      <c r="A4" s="90"/>
-      <c r="B4" s="91"/>
-      <c r="C4" s="91"/>
-      <c r="D4" s="91"/>
-      <c r="E4" s="92"/>
-      <c r="F4" s="90"/>
-      <c r="G4" s="91"/>
-      <c r="H4" s="91"/>
-      <c r="I4" s="91"/>
-      <c r="J4" s="91"/>
-      <c r="K4" s="91"/>
-      <c r="L4" s="91"/>
-      <c r="M4" s="91"/>
-      <c r="N4" s="91"/>
-      <c r="O4" s="92"/>
-      <c r="P4" s="94" t="s">
+      <c r="A4" s="81"/>
+      <c r="B4" s="82"/>
+      <c r="C4" s="82"/>
+      <c r="D4" s="82"/>
+      <c r="E4" s="83"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="82"/>
+      <c r="H4" s="82"/>
+      <c r="I4" s="82"/>
+      <c r="J4" s="82"/>
+      <c r="K4" s="82"/>
+      <c r="L4" s="82"/>
+      <c r="M4" s="82"/>
+      <c r="N4" s="82"/>
+      <c r="O4" s="83"/>
+      <c r="P4" s="124" t="s">
         <v>143</v>
       </c>
-      <c r="Q4" s="57"/>
+      <c r="Q4" s="72"/>
     </row>
     <row r="5" spans="1:17" ht="43.5" customHeight="1">
-      <c r="A5" s="95" t="s">
+      <c r="A5" s="125" t="s">
         <v>176</v>
       </c>
-      <c r="B5" s="56"/>
-      <c r="C5" s="56"/>
-      <c r="D5" s="56"/>
-      <c r="E5" s="56"/>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
-      <c r="H5" s="56"/>
-      <c r="I5" s="56"/>
-      <c r="J5" s="56"/>
-      <c r="K5" s="56"/>
-      <c r="L5" s="56"/>
-      <c r="M5" s="56"/>
-      <c r="N5" s="56"/>
-      <c r="O5" s="56"/>
-      <c r="P5" s="56"/>
-      <c r="Q5" s="57"/>
+      <c r="B5" s="54"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="54"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="54"/>
+      <c r="K5" s="54"/>
+      <c r="L5" s="54"/>
+      <c r="M5" s="54"/>
+      <c r="N5" s="54"/>
+      <c r="O5" s="54"/>
+      <c r="P5" s="54"/>
+      <c r="Q5" s="72"/>
     </row>
     <row r="6" spans="1:17">
-      <c r="A6" s="61" t="s">
+      <c r="A6" s="87" t="s">
         <v>161</v>
       </c>
-      <c r="B6" s="56"/>
-      <c r="C6" s="56"/>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="56"/>
-      <c r="I6" s="56"/>
-      <c r="J6" s="56"/>
-      <c r="K6" s="56"/>
-      <c r="L6" s="56"/>
-      <c r="M6" s="56"/>
-      <c r="N6" s="56"/>
-      <c r="O6" s="56"/>
-      <c r="P6" s="56"/>
-      <c r="Q6" s="57"/>
+      <c r="B6" s="54"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="54"/>
+      <c r="K6" s="54"/>
+      <c r="L6" s="54"/>
+      <c r="M6" s="54"/>
+      <c r="N6" s="54"/>
+      <c r="O6" s="54"/>
+      <c r="P6" s="54"/>
+      <c r="Q6" s="72"/>
     </row>
     <row r="7" spans="1:17" ht="30" customHeight="1">
-      <c r="A7" s="74" t="s">
+      <c r="A7" s="109" t="s">
         <v>144</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="76"/>
-      <c r="D7" s="96"/>
-      <c r="E7" s="78"/>
-      <c r="F7" s="78"/>
-      <c r="G7" s="78"/>
-      <c r="H7" s="78"/>
-      <c r="I7" s="79"/>
-      <c r="J7" s="58" t="s">
+      <c r="B7" s="110"/>
+      <c r="C7" s="111"/>
+      <c r="D7" s="126"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
+      <c r="H7" s="113"/>
+      <c r="I7" s="114"/>
+      <c r="J7" s="115" t="s">
         <v>145</v>
       </c>
-      <c r="K7" s="80"/>
-      <c r="L7" s="58"/>
-      <c r="M7" s="59"/>
-      <c r="N7" s="59"/>
-      <c r="O7" s="59"/>
-      <c r="P7" s="59"/>
-      <c r="Q7" s="60"/>
+      <c r="K7" s="116"/>
+      <c r="L7" s="115"/>
+      <c r="M7" s="117"/>
+      <c r="N7" s="117"/>
+      <c r="O7" s="117"/>
+      <c r="P7" s="117"/>
+      <c r="Q7" s="118"/>
     </row>
     <row r="8" spans="1:17" ht="30" customHeight="1">
-      <c r="A8" s="74" t="s">
+      <c r="A8" s="109" t="s">
         <v>146</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="76"/>
-      <c r="D8" s="77"/>
-      <c r="E8" s="78"/>
-      <c r="F8" s="78"/>
-      <c r="G8" s="78"/>
-      <c r="H8" s="78"/>
-      <c r="I8" s="79"/>
-      <c r="J8" s="58" t="s">
+      <c r="B8" s="110"/>
+      <c r="C8" s="111"/>
+      <c r="D8" s="112"/>
+      <c r="E8" s="113"/>
+      <c r="F8" s="113"/>
+      <c r="G8" s="113"/>
+      <c r="H8" s="113"/>
+      <c r="I8" s="114"/>
+      <c r="J8" s="115" t="s">
         <v>147</v>
       </c>
-      <c r="K8" s="80"/>
-      <c r="L8" s="58"/>
-      <c r="M8" s="59"/>
-      <c r="N8" s="59"/>
-      <c r="O8" s="59"/>
-      <c r="P8" s="59"/>
-      <c r="Q8" s="60"/>
+      <c r="K8" s="116"/>
+      <c r="L8" s="115"/>
+      <c r="M8" s="117"/>
+      <c r="N8" s="117"/>
+      <c r="O8" s="117"/>
+      <c r="P8" s="117"/>
+      <c r="Q8" s="118"/>
     </row>
     <row r="9" spans="1:17" ht="30" customHeight="1">
-      <c r="A9" s="74" t="s">
+      <c r="A9" s="109" t="s">
         <v>148</v>
       </c>
-      <c r="B9" s="75"/>
-      <c r="C9" s="76"/>
-      <c r="D9" s="77"/>
-      <c r="E9" s="78"/>
-      <c r="F9" s="78"/>
-      <c r="G9" s="78"/>
-      <c r="H9" s="78"/>
-      <c r="I9" s="79"/>
-      <c r="J9" s="58" t="s">
+      <c r="B9" s="110"/>
+      <c r="C9" s="111"/>
+      <c r="D9" s="112"/>
+      <c r="E9" s="113"/>
+      <c r="F9" s="113"/>
+      <c r="G9" s="113"/>
+      <c r="H9" s="113"/>
+      <c r="I9" s="114"/>
+      <c r="J9" s="115" t="s">
         <v>149</v>
       </c>
-      <c r="K9" s="80"/>
-      <c r="L9" s="58"/>
-      <c r="M9" s="59"/>
-      <c r="N9" s="59"/>
-      <c r="O9" s="59"/>
-      <c r="P9" s="59"/>
-      <c r="Q9" s="60"/>
+      <c r="K9" s="116"/>
+      <c r="L9" s="115"/>
+      <c r="M9" s="117"/>
+      <c r="N9" s="117"/>
+      <c r="O9" s="117"/>
+      <c r="P9" s="117"/>
+      <c r="Q9" s="118"/>
     </row>
     <row r="10" spans="1:17" ht="30" customHeight="1">
-      <c r="A10" s="74" t="s">
+      <c r="A10" s="109" t="s">
         <v>150</v>
       </c>
-      <c r="B10" s="75"/>
-      <c r="C10" s="76"/>
-      <c r="D10" s="77"/>
-      <c r="E10" s="78"/>
-      <c r="F10" s="78"/>
-      <c r="G10" s="78"/>
-      <c r="H10" s="78"/>
-      <c r="I10" s="79"/>
-      <c r="J10" s="58" t="s">
+      <c r="B10" s="110"/>
+      <c r="C10" s="111"/>
+      <c r="D10" s="112"/>
+      <c r="E10" s="113"/>
+      <c r="F10" s="113"/>
+      <c r="G10" s="113"/>
+      <c r="H10" s="113"/>
+      <c r="I10" s="114"/>
+      <c r="J10" s="115" t="s">
         <v>151</v>
       </c>
-      <c r="K10" s="80"/>
-      <c r="L10" s="58"/>
-      <c r="M10" s="59"/>
-      <c r="N10" s="59"/>
-      <c r="O10" s="59"/>
-      <c r="P10" s="59"/>
-      <c r="Q10" s="60"/>
+      <c r="K10" s="116"/>
+      <c r="L10" s="115"/>
+      <c r="M10" s="117"/>
+      <c r="N10" s="117"/>
+      <c r="O10" s="117"/>
+      <c r="P10" s="117"/>
+      <c r="Q10" s="118"/>
     </row>
     <row r="11" spans="1:17" ht="30" customHeight="1">
-      <c r="A11" s="74" t="s">
+      <c r="A11" s="109" t="s">
         <v>160</v>
       </c>
-      <c r="B11" s="75"/>
-      <c r="C11" s="76"/>
-      <c r="D11" s="77"/>
-      <c r="E11" s="78"/>
-      <c r="F11" s="78"/>
-      <c r="G11" s="78"/>
-      <c r="H11" s="78"/>
-      <c r="I11" s="79"/>
-      <c r="J11" s="58" t="s">
+      <c r="B11" s="110"/>
+      <c r="C11" s="111"/>
+      <c r="D11" s="112"/>
+      <c r="E11" s="113"/>
+      <c r="F11" s="113"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="114"/>
+      <c r="J11" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="K11" s="80"/>
-      <c r="L11" s="58"/>
-      <c r="M11" s="59"/>
-      <c r="N11" s="59"/>
-      <c r="O11" s="59"/>
-      <c r="P11" s="59"/>
-      <c r="Q11" s="60"/>
+      <c r="K11" s="116"/>
+      <c r="L11" s="115"/>
+      <c r="M11" s="117"/>
+      <c r="N11" s="117"/>
+      <c r="O11" s="117"/>
+      <c r="P11" s="117"/>
+      <c r="Q11" s="118"/>
     </row>
     <row r="12" spans="1:17" ht="30" customHeight="1">
-      <c r="A12" s="97" t="s">
+      <c r="A12" s="119" t="s">
         <v>153</v>
       </c>
-      <c r="B12" s="75"/>
-      <c r="C12" s="75"/>
-      <c r="D12" s="98"/>
-      <c r="E12" s="78"/>
-      <c r="F12" s="78"/>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="79"/>
-      <c r="J12" s="58" t="s">
+      <c r="B12" s="110"/>
+      <c r="C12" s="110"/>
+      <c r="D12" s="120"/>
+      <c r="E12" s="113"/>
+      <c r="F12" s="113"/>
+      <c r="G12" s="113"/>
+      <c r="H12" s="113"/>
+      <c r="I12" s="114"/>
+      <c r="J12" s="115" t="s">
         <v>154</v>
       </c>
-      <c r="K12" s="80"/>
-      <c r="L12" s="58"/>
-      <c r="M12" s="59"/>
-      <c r="N12" s="59"/>
-      <c r="O12" s="59"/>
-      <c r="P12" s="59"/>
-      <c r="Q12" s="60"/>
+      <c r="K12" s="116"/>
+      <c r="L12" s="115"/>
+      <c r="M12" s="117"/>
+      <c r="N12" s="117"/>
+      <c r="O12" s="117"/>
+      <c r="P12" s="117"/>
+      <c r="Q12" s="118"/>
     </row>
     <row r="13" spans="1:17" ht="30" customHeight="1">
-      <c r="A13" s="74" t="s">
+      <c r="A13" s="109" t="s">
         <v>158</v>
       </c>
-      <c r="B13" s="75"/>
-      <c r="C13" s="76"/>
-      <c r="D13" s="77"/>
-      <c r="E13" s="78"/>
-      <c r="F13" s="78"/>
-      <c r="G13" s="78"/>
-      <c r="H13" s="78"/>
-      <c r="I13" s="79"/>
-      <c r="J13" s="58" t="s">
+      <c r="B13" s="110"/>
+      <c r="C13" s="111"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="113"/>
+      <c r="F13" s="113"/>
+      <c r="G13" s="113"/>
+      <c r="H13" s="113"/>
+      <c r="I13" s="114"/>
+      <c r="J13" s="115" t="s">
         <v>155</v>
       </c>
-      <c r="K13" s="80"/>
-      <c r="L13" s="58"/>
-      <c r="M13" s="59"/>
-      <c r="N13" s="59"/>
-      <c r="O13" s="59"/>
-      <c r="P13" s="59"/>
-      <c r="Q13" s="60"/>
+      <c r="K13" s="116"/>
+      <c r="L13" s="115"/>
+      <c r="M13" s="117"/>
+      <c r="N13" s="117"/>
+      <c r="O13" s="117"/>
+      <c r="P13" s="117"/>
+      <c r="Q13" s="118"/>
     </row>
     <row r="14" spans="1:17">
-      <c r="A14" s="61" t="s">
+      <c r="A14" s="87" t="s">
         <v>177</v>
       </c>
-      <c r="B14" s="56"/>
-      <c r="C14" s="56"/>
-      <c r="D14" s="56"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56"/>
-      <c r="G14" s="56"/>
-      <c r="H14" s="56"/>
-      <c r="I14" s="56"/>
-      <c r="J14" s="56"/>
-      <c r="K14" s="56"/>
-      <c r="L14" s="56"/>
-      <c r="M14" s="56"/>
-      <c r="N14" s="56"/>
-      <c r="O14" s="56"/>
-      <c r="P14" s="56"/>
-      <c r="Q14" s="57"/>
+      <c r="B14" s="54"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="54"/>
+      <c r="J14" s="54"/>
+      <c r="K14" s="54"/>
+      <c r="L14" s="54"/>
+      <c r="M14" s="54"/>
+      <c r="N14" s="54"/>
+      <c r="O14" s="54"/>
+      <c r="P14" s="54"/>
+      <c r="Q14" s="72"/>
     </row>
     <row r="15" spans="1:17" ht="39.75" customHeight="1">
-      <c r="A15" s="62" t="s">
+      <c r="A15" s="127" t="s">
         <v>178</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63"/>
-      <c r="E15" s="63"/>
-      <c r="F15" s="63"/>
-      <c r="G15" s="63"/>
-      <c r="H15" s="63"/>
-      <c r="I15" s="63"/>
-      <c r="J15" s="63"/>
-      <c r="K15" s="63"/>
-      <c r="L15" s="63"/>
-      <c r="M15" s="63"/>
-      <c r="N15" s="63"/>
-      <c r="O15" s="63"/>
-      <c r="P15" s="63"/>
-      <c r="Q15" s="64"/>
+      <c r="B15" s="128"/>
+      <c r="C15" s="128"/>
+      <c r="D15" s="128"/>
+      <c r="E15" s="128"/>
+      <c r="F15" s="128"/>
+      <c r="G15" s="128"/>
+      <c r="H15" s="128"/>
+      <c r="I15" s="128"/>
+      <c r="J15" s="128"/>
+      <c r="K15" s="128"/>
+      <c r="L15" s="128"/>
+      <c r="M15" s="128"/>
+      <c r="N15" s="128"/>
+      <c r="O15" s="128"/>
+      <c r="P15" s="128"/>
+      <c r="Q15" s="129"/>
     </row>
     <row r="16" spans="1:17" ht="15">
-      <c r="A16" s="65" t="s">
+      <c r="A16" s="96" t="s">
         <v>179</v>
       </c>
-      <c r="B16" s="66"/>
-      <c r="C16" s="66"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="66"/>
-      <c r="F16" s="66"/>
-      <c r="G16" s="66"/>
-      <c r="H16" s="66"/>
-      <c r="I16" s="66"/>
-      <c r="J16" s="67"/>
-      <c r="K16" s="65" t="s">
+      <c r="B16" s="74"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="74"/>
+      <c r="I16" s="74"/>
+      <c r="J16" s="75"/>
+      <c r="K16" s="96" t="s">
         <v>162</v>
       </c>
-      <c r="L16" s="66"/>
-      <c r="M16" s="66"/>
-      <c r="N16" s="67"/>
-      <c r="O16" s="68" t="s">
+      <c r="L16" s="74"/>
+      <c r="M16" s="74"/>
+      <c r="N16" s="75"/>
+      <c r="O16" s="130" t="s">
         <v>163</v>
       </c>
-      <c r="P16" s="69"/>
-      <c r="Q16" s="70"/>
+      <c r="P16" s="60"/>
+      <c r="Q16" s="61"/>
     </row>
     <row r="17" spans="1:17">
-      <c r="A17" s="65" t="s">
+      <c r="A17" s="96" t="s">
         <v>164</v>
       </c>
-      <c r="B17" s="67"/>
-      <c r="C17" s="65" t="s">
+      <c r="B17" s="75"/>
+      <c r="C17" s="96" t="s">
         <v>165</v>
       </c>
-      <c r="D17" s="66"/>
-      <c r="E17" s="66"/>
-      <c r="F17" s="66"/>
-      <c r="G17" s="67"/>
-      <c r="H17" s="65" t="s">
+      <c r="D17" s="74"/>
+      <c r="E17" s="74"/>
+      <c r="F17" s="74"/>
+      <c r="G17" s="75"/>
+      <c r="H17" s="96" t="s">
         <v>166</v>
       </c>
-      <c r="I17" s="66"/>
-      <c r="J17" s="67"/>
+      <c r="I17" s="74"/>
+      <c r="J17" s="75"/>
       <c r="K17" s="46" t="s">
         <v>167</v>
       </c>
-      <c r="L17" s="65" t="s">
+      <c r="L17" s="96" t="s">
         <v>168</v>
       </c>
-      <c r="M17" s="66"/>
-      <c r="N17" s="67"/>
-      <c r="O17" s="71"/>
-      <c r="P17" s="72"/>
-      <c r="Q17" s="73"/>
+      <c r="M17" s="74"/>
+      <c r="N17" s="75"/>
+      <c r="O17" s="65"/>
+      <c r="P17" s="66"/>
+      <c r="Q17" s="67"/>
     </row>
     <row r="18" spans="1:17" ht="15">
-      <c r="A18" s="81"/>
-      <c r="B18" s="66"/>
-      <c r="C18" s="82"/>
-      <c r="D18" s="66"/>
-      <c r="E18" s="66"/>
-      <c r="F18" s="66"/>
-      <c r="G18" s="67"/>
-      <c r="H18" s="83"/>
-      <c r="I18" s="66"/>
-      <c r="J18" s="67"/>
+      <c r="A18" s="95"/>
+      <c r="B18" s="74"/>
+      <c r="C18" s="101"/>
+      <c r="D18" s="74"/>
+      <c r="E18" s="74"/>
+      <c r="F18" s="74"/>
+      <c r="G18" s="75"/>
+      <c r="H18" s="97"/>
+      <c r="I18" s="74"/>
+      <c r="J18" s="75"/>
       <c r="K18" s="47"/>
-      <c r="L18" s="84"/>
-      <c r="M18" s="66"/>
-      <c r="N18" s="67"/>
-      <c r="O18" s="81"/>
-      <c r="P18" s="66"/>
-      <c r="Q18" s="67"/>
+      <c r="L18" s="121"/>
+      <c r="M18" s="74"/>
+      <c r="N18" s="75"/>
+      <c r="O18" s="95"/>
+      <c r="P18" s="74"/>
+      <c r="Q18" s="75"/>
     </row>
     <row r="19" spans="1:17" ht="30" customHeight="1">
-      <c r="A19" s="65" t="s">
+      <c r="A19" s="96" t="s">
         <v>180</v>
       </c>
-      <c r="B19" s="66"/>
-      <c r="C19" s="81"/>
-      <c r="D19" s="67"/>
-      <c r="E19" s="99" t="s">
+      <c r="B19" s="74"/>
+      <c r="C19" s="95"/>
+      <c r="D19" s="75"/>
+      <c r="E19" s="104" t="s">
         <v>181</v>
       </c>
-      <c r="F19" s="66"/>
-      <c r="G19" s="81"/>
-      <c r="H19" s="66"/>
-      <c r="I19" s="67"/>
-      <c r="J19" s="99" t="s">
+      <c r="F19" s="74"/>
+      <c r="G19" s="95"/>
+      <c r="H19" s="74"/>
+      <c r="I19" s="75"/>
+      <c r="J19" s="104" t="s">
         <v>182</v>
       </c>
-      <c r="K19" s="66"/>
-      <c r="L19" s="66"/>
-      <c r="M19" s="81"/>
-      <c r="N19" s="67"/>
-      <c r="O19" s="100" t="s">
+      <c r="K19" s="74"/>
+      <c r="L19" s="74"/>
+      <c r="M19" s="95"/>
+      <c r="N19" s="75"/>
+      <c r="O19" s="102" t="s">
         <v>183</v>
       </c>
-      <c r="P19" s="66"/>
+      <c r="P19" s="74"/>
       <c r="Q19" s="49"/>
     </row>
     <row r="20" spans="1:17" ht="34.5" customHeight="1">
-      <c r="A20" s="65" t="s">
+      <c r="A20" s="96" t="s">
         <v>184</v>
       </c>
-      <c r="B20" s="66"/>
-      <c r="C20" s="66"/>
-      <c r="D20" s="67"/>
+      <c r="B20" s="74"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="75"/>
       <c r="E20" s="107"/>
-      <c r="F20" s="66"/>
-      <c r="G20" s="67"/>
+      <c r="F20" s="74"/>
+      <c r="G20" s="75"/>
       <c r="H20" s="108" t="s">
         <v>185</v>
       </c>
-      <c r="I20" s="72"/>
-      <c r="J20" s="72"/>
-      <c r="K20" s="73"/>
+      <c r="I20" s="66"/>
+      <c r="J20" s="66"/>
+      <c r="K20" s="67"/>
       <c r="L20" s="107"/>
-      <c r="M20" s="67"/>
+      <c r="M20" s="75"/>
       <c r="N20" s="50" t="s">
         <v>169</v>
       </c>
-      <c r="O20" s="81"/>
-      <c r="P20" s="66"/>
-      <c r="Q20" s="67"/>
+      <c r="O20" s="95"/>
+      <c r="P20" s="74"/>
+      <c r="Q20" s="75"/>
     </row>
     <row r="21" spans="1:17" ht="34.5" customHeight="1">
-      <c r="A21" s="65" t="s">
+      <c r="A21" s="96" t="s">
         <v>186</v>
       </c>
-      <c r="B21" s="66"/>
-      <c r="C21" s="83"/>
-      <c r="D21" s="66"/>
-      <c r="E21" s="66"/>
-      <c r="F21" s="67"/>
-      <c r="G21" s="65" t="s">
+      <c r="B21" s="74"/>
+      <c r="C21" s="97"/>
+      <c r="D21" s="74"/>
+      <c r="E21" s="74"/>
+      <c r="F21" s="75"/>
+      <c r="G21" s="96" t="s">
         <v>187</v>
       </c>
-      <c r="H21" s="67"/>
-      <c r="I21" s="105"/>
-      <c r="J21" s="66"/>
-      <c r="K21" s="67"/>
+      <c r="H21" s="75"/>
+      <c r="I21" s="85"/>
+      <c r="J21" s="74"/>
+      <c r="K21" s="75"/>
       <c r="L21" s="48" t="s">
         <v>188</v>
       </c>
-      <c r="M21" s="106"/>
-      <c r="N21" s="67"/>
-      <c r="O21" s="100" t="s">
+      <c r="M21" s="98"/>
+      <c r="N21" s="75"/>
+      <c r="O21" s="102" t="s">
         <v>189</v>
       </c>
-      <c r="P21" s="66"/>
+      <c r="P21" s="74"/>
       <c r="Q21" s="49"/>
     </row>
     <row r="22" spans="1:17" ht="39" customHeight="1">
-      <c r="A22" s="65" t="s">
+      <c r="A22" s="96" t="s">
         <v>190</v>
       </c>
-      <c r="B22" s="66"/>
-      <c r="C22" s="66"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="67"/>
-      <c r="F22" s="110"/>
-      <c r="G22" s="66"/>
-      <c r="H22" s="66"/>
-      <c r="I22" s="66"/>
-      <c r="J22" s="65" t="s">
+      <c r="B22" s="74"/>
+      <c r="C22" s="74"/>
+      <c r="D22" s="74"/>
+      <c r="E22" s="75"/>
+      <c r="F22" s="100"/>
+      <c r="G22" s="74"/>
+      <c r="H22" s="74"/>
+      <c r="I22" s="74"/>
+      <c r="J22" s="96" t="s">
         <v>191</v>
       </c>
-      <c r="K22" s="67"/>
-      <c r="L22" s="82"/>
-      <c r="M22" s="66"/>
-      <c r="N22" s="67"/>
-      <c r="O22" s="100" t="s">
+      <c r="K22" s="75"/>
+      <c r="L22" s="101"/>
+      <c r="M22" s="74"/>
+      <c r="N22" s="75"/>
+      <c r="O22" s="102" t="s">
         <v>192</v>
       </c>
-      <c r="P22" s="66"/>
+      <c r="P22" s="74"/>
       <c r="Q22" s="49"/>
     </row>
     <row r="23" spans="1:17">
-      <c r="A23" s="111" t="s">
+      <c r="A23" s="103" t="s">
         <v>193</v>
       </c>
-      <c r="B23" s="66"/>
-      <c r="C23" s="66"/>
-      <c r="D23" s="66"/>
-      <c r="E23" s="66"/>
-      <c r="F23" s="66"/>
-      <c r="G23" s="66"/>
-      <c r="H23" s="66"/>
-      <c r="I23" s="66"/>
-      <c r="J23" s="66"/>
-      <c r="K23" s="66"/>
-      <c r="L23" s="66"/>
-      <c r="M23" s="66"/>
-      <c r="N23" s="66"/>
-      <c r="O23" s="66"/>
-      <c r="P23" s="66"/>
-      <c r="Q23" s="67"/>
+      <c r="B23" s="74"/>
+      <c r="C23" s="74"/>
+      <c r="D23" s="74"/>
+      <c r="E23" s="74"/>
+      <c r="F23" s="74"/>
+      <c r="G23" s="74"/>
+      <c r="H23" s="74"/>
+      <c r="I23" s="74"/>
+      <c r="J23" s="74"/>
+      <c r="K23" s="74"/>
+      <c r="L23" s="74"/>
+      <c r="M23" s="74"/>
+      <c r="N23" s="74"/>
+      <c r="O23" s="74"/>
+      <c r="P23" s="74"/>
+      <c r="Q23" s="75"/>
     </row>
     <row r="24" spans="1:17" ht="15">
-      <c r="A24" s="109" t="s">
+      <c r="A24" s="99" t="s">
         <v>194</v>
       </c>
-      <c r="B24" s="66"/>
-      <c r="C24" s="66"/>
-      <c r="D24" s="66"/>
-      <c r="E24" s="66"/>
-      <c r="F24" s="67"/>
-      <c r="G24" s="106"/>
-      <c r="H24" s="66"/>
-      <c r="I24" s="66"/>
-      <c r="J24" s="66"/>
-      <c r="K24" s="67"/>
-      <c r="L24" s="109" t="s">
+      <c r="B24" s="74"/>
+      <c r="C24" s="74"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="74"/>
+      <c r="F24" s="75"/>
+      <c r="G24" s="98"/>
+      <c r="H24" s="74"/>
+      <c r="I24" s="74"/>
+      <c r="J24" s="74"/>
+      <c r="K24" s="75"/>
+      <c r="L24" s="99" t="s">
         <v>195</v>
       </c>
-      <c r="M24" s="67"/>
-      <c r="N24" s="81"/>
-      <c r="O24" s="66"/>
-      <c r="P24" s="66"/>
-      <c r="Q24" s="67"/>
+      <c r="M24" s="75"/>
+      <c r="N24" s="95"/>
+      <c r="O24" s="74"/>
+      <c r="P24" s="74"/>
+      <c r="Q24" s="75"/>
     </row>
     <row r="25" spans="1:17">
-      <c r="A25" s="112" t="s">
+      <c r="A25" s="93" t="s">
         <v>196</v>
       </c>
-      <c r="B25" s="91"/>
-      <c r="C25" s="91"/>
-      <c r="D25" s="91"/>
-      <c r="E25" s="91"/>
-      <c r="F25" s="91"/>
-      <c r="G25" s="91"/>
-      <c r="H25" s="91"/>
-      <c r="I25" s="91"/>
-      <c r="J25" s="91"/>
-      <c r="K25" s="91"/>
-      <c r="L25" s="91"/>
-      <c r="M25" s="91"/>
-      <c r="N25" s="91"/>
-      <c r="O25" s="91"/>
-      <c r="P25" s="91"/>
-      <c r="Q25" s="92"/>
+      <c r="B25" s="82"/>
+      <c r="C25" s="82"/>
+      <c r="D25" s="82"/>
+      <c r="E25" s="82"/>
+      <c r="F25" s="82"/>
+      <c r="G25" s="82"/>
+      <c r="H25" s="82"/>
+      <c r="I25" s="82"/>
+      <c r="J25" s="82"/>
+      <c r="K25" s="82"/>
+      <c r="L25" s="82"/>
+      <c r="M25" s="82"/>
+      <c r="N25" s="82"/>
+      <c r="O25" s="82"/>
+      <c r="P25" s="82"/>
+      <c r="Q25" s="83"/>
     </row>
     <row r="26" spans="1:17" ht="134.25" customHeight="1">
-      <c r="A26" s="113"/>
-      <c r="B26" s="72"/>
-      <c r="C26" s="72"/>
-      <c r="D26" s="72"/>
-      <c r="E26" s="72"/>
-      <c r="F26" s="72"/>
-      <c r="G26" s="72"/>
-      <c r="H26" s="72"/>
-      <c r="I26" s="72"/>
-      <c r="J26" s="72"/>
-      <c r="K26" s="72"/>
-      <c r="L26" s="72"/>
-      <c r="M26" s="72"/>
-      <c r="N26" s="72"/>
-      <c r="O26" s="72"/>
-      <c r="P26" s="72"/>
-      <c r="Q26" s="73"/>
+      <c r="A26" s="94"/>
+      <c r="B26" s="66"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="66"/>
+      <c r="E26" s="66"/>
+      <c r="F26" s="66"/>
+      <c r="G26" s="66"/>
+      <c r="H26" s="66"/>
+      <c r="I26" s="66"/>
+      <c r="J26" s="66"/>
+      <c r="K26" s="66"/>
+      <c r="L26" s="66"/>
+      <c r="M26" s="66"/>
+      <c r="N26" s="66"/>
+      <c r="O26" s="66"/>
+      <c r="P26" s="66"/>
+      <c r="Q26" s="67"/>
     </row>
     <row r="27" spans="1:17">
-      <c r="A27" s="112" t="s">
+      <c r="A27" s="93" t="s">
         <v>197</v>
       </c>
-      <c r="B27" s="91"/>
-      <c r="C27" s="91"/>
-      <c r="D27" s="91"/>
-      <c r="E27" s="91"/>
-      <c r="F27" s="91"/>
-      <c r="G27" s="91"/>
-      <c r="H27" s="91"/>
-      <c r="I27" s="91"/>
-      <c r="J27" s="91"/>
-      <c r="K27" s="91"/>
-      <c r="L27" s="91"/>
-      <c r="M27" s="91"/>
-      <c r="N27" s="91"/>
-      <c r="O27" s="91"/>
-      <c r="P27" s="91"/>
-      <c r="Q27" s="92"/>
+      <c r="B27" s="82"/>
+      <c r="C27" s="82"/>
+      <c r="D27" s="82"/>
+      <c r="E27" s="82"/>
+      <c r="F27" s="82"/>
+      <c r="G27" s="82"/>
+      <c r="H27" s="82"/>
+      <c r="I27" s="82"/>
+      <c r="J27" s="82"/>
+      <c r="K27" s="82"/>
+      <c r="L27" s="82"/>
+      <c r="M27" s="82"/>
+      <c r="N27" s="82"/>
+      <c r="O27" s="82"/>
+      <c r="P27" s="82"/>
+      <c r="Q27" s="83"/>
     </row>
     <row r="28" spans="1:17" ht="12.75">
-      <c r="A28" s="114" t="s">
+      <c r="A28" s="71" t="s">
         <v>198</v>
       </c>
-      <c r="B28" s="56"/>
-      <c r="C28" s="56"/>
-      <c r="D28" s="56"/>
-      <c r="E28" s="56"/>
-      <c r="F28" s="56"/>
-      <c r="G28" s="56"/>
-      <c r="H28" s="56"/>
-      <c r="I28" s="56"/>
-      <c r="J28" s="56"/>
-      <c r="K28" s="56"/>
-      <c r="L28" s="56"/>
-      <c r="M28" s="56"/>
-      <c r="N28" s="56"/>
-      <c r="O28" s="56"/>
-      <c r="P28" s="56"/>
-      <c r="Q28" s="57"/>
+      <c r="B28" s="54"/>
+      <c r="C28" s="54"/>
+      <c r="D28" s="54"/>
+      <c r="E28" s="54"/>
+      <c r="F28" s="54"/>
+      <c r="G28" s="54"/>
+      <c r="H28" s="54"/>
+      <c r="I28" s="54"/>
+      <c r="J28" s="54"/>
+      <c r="K28" s="54"/>
+      <c r="L28" s="54"/>
+      <c r="M28" s="54"/>
+      <c r="N28" s="54"/>
+      <c r="O28" s="54"/>
+      <c r="P28" s="54"/>
+      <c r="Q28" s="72"/>
     </row>
     <row r="29" spans="1:17" ht="36.75" customHeight="1">
-      <c r="A29" s="115" t="s">
+      <c r="A29" s="53" t="s">
         <v>199</v>
       </c>
-      <c r="B29" s="56"/>
-      <c r="C29" s="56"/>
-      <c r="D29" s="56"/>
-      <c r="E29" s="56"/>
-      <c r="F29" s="56"/>
-      <c r="G29" s="115" t="s">
+      <c r="B29" s="54"/>
+      <c r="C29" s="54"/>
+      <c r="D29" s="54"/>
+      <c r="E29" s="54"/>
+      <c r="F29" s="54"/>
+      <c r="G29" s="53" t="s">
         <v>200</v>
       </c>
-      <c r="H29" s="56"/>
-      <c r="I29" s="56"/>
-      <c r="J29" s="56"/>
-      <c r="K29" s="56"/>
-      <c r="L29" s="115" t="s">
+      <c r="H29" s="54"/>
+      <c r="I29" s="54"/>
+      <c r="J29" s="54"/>
+      <c r="K29" s="54"/>
+      <c r="L29" s="53" t="s">
         <v>201</v>
       </c>
-      <c r="M29" s="56"/>
-      <c r="N29" s="56"/>
-      <c r="O29" s="56"/>
-      <c r="P29" s="56"/>
-      <c r="Q29" s="57"/>
+      <c r="M29" s="54"/>
+      <c r="N29" s="54"/>
+      <c r="O29" s="54"/>
+      <c r="P29" s="54"/>
+      <c r="Q29" s="72"/>
     </row>
     <row r="30" spans="1:17" ht="36" customHeight="1">
-      <c r="A30" s="116" t="s">
+      <c r="A30" s="89" t="s">
         <v>202</v>
       </c>
-      <c r="B30" s="86"/>
-      <c r="C30" s="86"/>
-      <c r="D30" s="86"/>
-      <c r="E30" s="86"/>
-      <c r="F30" s="86"/>
-      <c r="G30" s="117"/>
-      <c r="H30" s="69"/>
-      <c r="I30" s="69"/>
-      <c r="J30" s="69"/>
-      <c r="K30" s="70"/>
-      <c r="L30" s="103"/>
-      <c r="M30" s="66"/>
-      <c r="N30" s="66"/>
-      <c r="O30" s="66"/>
-      <c r="P30" s="66"/>
-      <c r="Q30" s="67"/>
+      <c r="B30" s="56"/>
+      <c r="C30" s="56"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
+      <c r="G30" s="59"/>
+      <c r="H30" s="60"/>
+      <c r="I30" s="60"/>
+      <c r="J30" s="60"/>
+      <c r="K30" s="61"/>
+      <c r="L30" s="105"/>
+      <c r="M30" s="74"/>
+      <c r="N30" s="74"/>
+      <c r="O30" s="74"/>
+      <c r="P30" s="74"/>
+      <c r="Q30" s="75"/>
     </row>
     <row r="31" spans="1:17">
-      <c r="A31" s="88"/>
-      <c r="B31" s="54"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="54"/>
-      <c r="E31" s="54"/>
-      <c r="F31" s="54"/>
-      <c r="G31" s="71"/>
-      <c r="H31" s="72"/>
-      <c r="I31" s="72"/>
-      <c r="J31" s="72"/>
-      <c r="K31" s="73"/>
+      <c r="A31" s="57"/>
+      <c r="B31" s="58"/>
+      <c r="C31" s="58"/>
+      <c r="D31" s="58"/>
+      <c r="E31" s="58"/>
+      <c r="F31" s="58"/>
+      <c r="G31" s="65"/>
+      <c r="H31" s="66"/>
+      <c r="I31" s="66"/>
+      <c r="J31" s="66"/>
+      <c r="K31" s="67"/>
       <c r="L31" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M31" s="102"/>
-      <c r="N31" s="72"/>
-      <c r="O31" s="72"/>
-      <c r="P31" s="72"/>
-      <c r="Q31" s="73"/>
+      <c r="M31" s="77"/>
+      <c r="N31" s="66"/>
+      <c r="O31" s="66"/>
+      <c r="P31" s="66"/>
+      <c r="Q31" s="67"/>
     </row>
     <row r="32" spans="1:17" ht="15">
-      <c r="A32" s="116" t="s">
+      <c r="A32" s="89" t="s">
         <v>203</v>
       </c>
-      <c r="B32" s="86"/>
-      <c r="C32" s="86"/>
-      <c r="D32" s="86"/>
-      <c r="E32" s="86"/>
-      <c r="F32" s="86"/>
-      <c r="G32" s="117"/>
-      <c r="H32" s="69"/>
-      <c r="I32" s="69"/>
-      <c r="J32" s="69"/>
-      <c r="K32" s="70"/>
-      <c r="L32" s="104"/>
-      <c r="M32" s="72"/>
-      <c r="N32" s="72"/>
-      <c r="O32" s="72"/>
-      <c r="P32" s="72"/>
-      <c r="Q32" s="73"/>
+      <c r="B32" s="56"/>
+      <c r="C32" s="56"/>
+      <c r="D32" s="56"/>
+      <c r="E32" s="56"/>
+      <c r="F32" s="56"/>
+      <c r="G32" s="59"/>
+      <c r="H32" s="60"/>
+      <c r="I32" s="60"/>
+      <c r="J32" s="60"/>
+      <c r="K32" s="61"/>
+      <c r="L32" s="106"/>
+      <c r="M32" s="66"/>
+      <c r="N32" s="66"/>
+      <c r="O32" s="66"/>
+      <c r="P32" s="66"/>
+      <c r="Q32" s="67"/>
     </row>
     <row r="33" spans="1:17">
-      <c r="A33" s="88"/>
-      <c r="B33" s="54"/>
-      <c r="C33" s="54"/>
-      <c r="D33" s="54"/>
-      <c r="E33" s="54"/>
-      <c r="F33" s="54"/>
-      <c r="G33" s="71"/>
-      <c r="H33" s="72"/>
-      <c r="I33" s="72"/>
-      <c r="J33" s="72"/>
-      <c r="K33" s="73"/>
+      <c r="A33" s="57"/>
+      <c r="B33" s="58"/>
+      <c r="C33" s="58"/>
+      <c r="D33" s="58"/>
+      <c r="E33" s="58"/>
+      <c r="F33" s="58"/>
+      <c r="G33" s="65"/>
+      <c r="H33" s="66"/>
+      <c r="I33" s="66"/>
+      <c r="J33" s="66"/>
+      <c r="K33" s="67"/>
       <c r="L33" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M33" s="102"/>
-      <c r="N33" s="72"/>
-      <c r="O33" s="72"/>
-      <c r="P33" s="72"/>
-      <c r="Q33" s="73"/>
+      <c r="M33" s="77"/>
+      <c r="N33" s="66"/>
+      <c r="O33" s="66"/>
+      <c r="P33" s="66"/>
+      <c r="Q33" s="67"/>
     </row>
     <row r="34" spans="1:17" ht="15">
-      <c r="A34" s="118" t="s">
+      <c r="A34" s="55" t="s">
         <v>204</v>
       </c>
-      <c r="B34" s="86"/>
-      <c r="C34" s="86"/>
-      <c r="D34" s="86"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="86"/>
-      <c r="G34" s="117"/>
-      <c r="H34" s="69"/>
-      <c r="I34" s="69"/>
-      <c r="J34" s="69"/>
-      <c r="K34" s="70"/>
-      <c r="L34" s="101"/>
-      <c r="M34" s="66"/>
-      <c r="N34" s="66"/>
-      <c r="O34" s="66"/>
-      <c r="P34" s="66"/>
-      <c r="Q34" s="67"/>
+      <c r="B34" s="56"/>
+      <c r="C34" s="56"/>
+      <c r="D34" s="56"/>
+      <c r="E34" s="56"/>
+      <c r="F34" s="56"/>
+      <c r="G34" s="59"/>
+      <c r="H34" s="60"/>
+      <c r="I34" s="60"/>
+      <c r="J34" s="60"/>
+      <c r="K34" s="61"/>
+      <c r="L34" s="76"/>
+      <c r="M34" s="74"/>
+      <c r="N34" s="74"/>
+      <c r="O34" s="74"/>
+      <c r="P34" s="74"/>
+      <c r="Q34" s="75"/>
     </row>
     <row r="35" spans="1:17" ht="15">
-      <c r="A35" s="88"/>
-      <c r="B35" s="54"/>
-      <c r="C35" s="54"/>
-      <c r="D35" s="54"/>
-      <c r="E35" s="54"/>
-      <c r="F35" s="54"/>
-      <c r="G35" s="119"/>
-      <c r="H35" s="120"/>
-      <c r="I35" s="120"/>
-      <c r="J35" s="120"/>
-      <c r="K35" s="121"/>
-      <c r="L35" s="101"/>
-      <c r="M35" s="66"/>
-      <c r="N35" s="66"/>
-      <c r="O35" s="66"/>
-      <c r="P35" s="66"/>
-      <c r="Q35" s="67"/>
+      <c r="A35" s="57"/>
+      <c r="B35" s="58"/>
+      <c r="C35" s="58"/>
+      <c r="D35" s="58"/>
+      <c r="E35" s="58"/>
+      <c r="F35" s="58"/>
+      <c r="G35" s="62"/>
+      <c r="H35" s="63"/>
+      <c r="I35" s="63"/>
+      <c r="J35" s="63"/>
+      <c r="K35" s="64"/>
+      <c r="L35" s="76"/>
+      <c r="M35" s="74"/>
+      <c r="N35" s="74"/>
+      <c r="O35" s="74"/>
+      <c r="P35" s="74"/>
+      <c r="Q35" s="75"/>
     </row>
     <row r="36" spans="1:17" ht="15">
-      <c r="A36" s="88"/>
-      <c r="B36" s="54"/>
-      <c r="C36" s="54"/>
-      <c r="D36" s="54"/>
-      <c r="E36" s="54"/>
-      <c r="F36" s="54"/>
-      <c r="G36" s="119"/>
-      <c r="H36" s="120"/>
-      <c r="I36" s="120"/>
-      <c r="J36" s="120"/>
-      <c r="K36" s="121"/>
-      <c r="L36" s="101"/>
-      <c r="M36" s="66"/>
-      <c r="N36" s="66"/>
-      <c r="O36" s="66"/>
-      <c r="P36" s="66"/>
-      <c r="Q36" s="67"/>
+      <c r="A36" s="57"/>
+      <c r="B36" s="58"/>
+      <c r="C36" s="58"/>
+      <c r="D36" s="58"/>
+      <c r="E36" s="58"/>
+      <c r="F36" s="58"/>
+      <c r="G36" s="62"/>
+      <c r="H36" s="63"/>
+      <c r="I36" s="63"/>
+      <c r="J36" s="63"/>
+      <c r="K36" s="64"/>
+      <c r="L36" s="76"/>
+      <c r="M36" s="74"/>
+      <c r="N36" s="74"/>
+      <c r="O36" s="74"/>
+      <c r="P36" s="74"/>
+      <c r="Q36" s="75"/>
     </row>
     <row r="37" spans="1:17" ht="15">
-      <c r="A37" s="88"/>
-      <c r="B37" s="54"/>
-      <c r="C37" s="54"/>
-      <c r="D37" s="54"/>
-      <c r="E37" s="54"/>
-      <c r="F37" s="54"/>
-      <c r="G37" s="119"/>
-      <c r="H37" s="120"/>
-      <c r="I37" s="120"/>
-      <c r="J37" s="120"/>
-      <c r="K37" s="121"/>
-      <c r="L37" s="101"/>
-      <c r="M37" s="66"/>
-      <c r="N37" s="66"/>
-      <c r="O37" s="66"/>
-      <c r="P37" s="66"/>
-      <c r="Q37" s="67"/>
+      <c r="A37" s="57"/>
+      <c r="B37" s="58"/>
+      <c r="C37" s="58"/>
+      <c r="D37" s="58"/>
+      <c r="E37" s="58"/>
+      <c r="F37" s="58"/>
+      <c r="G37" s="62"/>
+      <c r="H37" s="63"/>
+      <c r="I37" s="63"/>
+      <c r="J37" s="63"/>
+      <c r="K37" s="64"/>
+      <c r="L37" s="76"/>
+      <c r="M37" s="74"/>
+      <c r="N37" s="74"/>
+      <c r="O37" s="74"/>
+      <c r="P37" s="74"/>
+      <c r="Q37" s="75"/>
     </row>
     <row r="38" spans="1:17">
-      <c r="A38" s="88"/>
-      <c r="B38" s="54"/>
-      <c r="C38" s="54"/>
-      <c r="D38" s="54"/>
-      <c r="E38" s="54"/>
-      <c r="F38" s="54"/>
-      <c r="G38" s="71"/>
-      <c r="H38" s="72"/>
-      <c r="I38" s="72"/>
-      <c r="J38" s="72"/>
-      <c r="K38" s="73"/>
+      <c r="A38" s="57"/>
+      <c r="B38" s="58"/>
+      <c r="C38" s="58"/>
+      <c r="D38" s="58"/>
+      <c r="E38" s="58"/>
+      <c r="F38" s="58"/>
+      <c r="G38" s="65"/>
+      <c r="H38" s="66"/>
+      <c r="I38" s="66"/>
+      <c r="J38" s="66"/>
+      <c r="K38" s="67"/>
       <c r="L38" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M38" s="102"/>
-      <c r="N38" s="72"/>
-      <c r="O38" s="72"/>
-      <c r="P38" s="72"/>
-      <c r="Q38" s="73"/>
+      <c r="M38" s="77"/>
+      <c r="N38" s="66"/>
+      <c r="O38" s="66"/>
+      <c r="P38" s="66"/>
+      <c r="Q38" s="67"/>
     </row>
     <row r="39" spans="1:17" ht="15">
-      <c r="A39" s="118" t="s">
+      <c r="A39" s="55" t="s">
         <v>205</v>
       </c>
-      <c r="B39" s="86"/>
-      <c r="C39" s="86"/>
-      <c r="D39" s="86"/>
-      <c r="E39" s="86"/>
-      <c r="F39" s="87"/>
-      <c r="G39" s="117"/>
-      <c r="H39" s="69"/>
-      <c r="I39" s="69"/>
-      <c r="J39" s="69"/>
-      <c r="K39" s="70"/>
-      <c r="L39" s="101"/>
-      <c r="M39" s="66"/>
-      <c r="N39" s="66"/>
-      <c r="O39" s="66"/>
-      <c r="P39" s="66"/>
-      <c r="Q39" s="67"/>
+      <c r="B39" s="56"/>
+      <c r="C39" s="56"/>
+      <c r="D39" s="56"/>
+      <c r="E39" s="56"/>
+      <c r="F39" s="79"/>
+      <c r="G39" s="59"/>
+      <c r="H39" s="60"/>
+      <c r="I39" s="60"/>
+      <c r="J39" s="60"/>
+      <c r="K39" s="61"/>
+      <c r="L39" s="76"/>
+      <c r="M39" s="74"/>
+      <c r="N39" s="74"/>
+      <c r="O39" s="74"/>
+      <c r="P39" s="74"/>
+      <c r="Q39" s="75"/>
     </row>
     <row r="40" spans="1:17" ht="15">
-      <c r="A40" s="88"/>
-      <c r="B40" s="54"/>
-      <c r="C40" s="54"/>
-      <c r="D40" s="54"/>
-      <c r="E40" s="54"/>
-      <c r="F40" s="89"/>
-      <c r="G40" s="119"/>
-      <c r="H40" s="120"/>
-      <c r="I40" s="120"/>
-      <c r="J40" s="120"/>
-      <c r="K40" s="121"/>
-      <c r="L40" s="101"/>
-      <c r="M40" s="66"/>
-      <c r="N40" s="66"/>
-      <c r="O40" s="66"/>
-      <c r="P40" s="66"/>
-      <c r="Q40" s="67"/>
+      <c r="A40" s="57"/>
+      <c r="B40" s="58"/>
+      <c r="C40" s="58"/>
+      <c r="D40" s="58"/>
+      <c r="E40" s="58"/>
+      <c r="F40" s="80"/>
+      <c r="G40" s="62"/>
+      <c r="H40" s="63"/>
+      <c r="I40" s="63"/>
+      <c r="J40" s="63"/>
+      <c r="K40" s="64"/>
+      <c r="L40" s="76"/>
+      <c r="M40" s="74"/>
+      <c r="N40" s="74"/>
+      <c r="O40" s="74"/>
+      <c r="P40" s="74"/>
+      <c r="Q40" s="75"/>
     </row>
     <row r="41" spans="1:17" ht="15">
-      <c r="A41" s="88"/>
-      <c r="B41" s="54"/>
-      <c r="C41" s="54"/>
-      <c r="D41" s="54"/>
-      <c r="E41" s="54"/>
-      <c r="F41" s="89"/>
-      <c r="G41" s="119"/>
-      <c r="H41" s="120"/>
-      <c r="I41" s="120"/>
-      <c r="J41" s="120"/>
-      <c r="K41" s="121"/>
-      <c r="L41" s="101"/>
-      <c r="M41" s="66"/>
-      <c r="N41" s="66"/>
-      <c r="O41" s="66"/>
-      <c r="P41" s="66"/>
-      <c r="Q41" s="67"/>
+      <c r="A41" s="57"/>
+      <c r="B41" s="58"/>
+      <c r="C41" s="58"/>
+      <c r="D41" s="58"/>
+      <c r="E41" s="58"/>
+      <c r="F41" s="80"/>
+      <c r="G41" s="62"/>
+      <c r="H41" s="63"/>
+      <c r="I41" s="63"/>
+      <c r="J41" s="63"/>
+      <c r="K41" s="64"/>
+      <c r="L41" s="76"/>
+      <c r="M41" s="74"/>
+      <c r="N41" s="74"/>
+      <c r="O41" s="74"/>
+      <c r="P41" s="74"/>
+      <c r="Q41" s="75"/>
     </row>
     <row r="42" spans="1:17">
-      <c r="A42" s="90"/>
-      <c r="B42" s="91"/>
-      <c r="C42" s="91"/>
-      <c r="D42" s="91"/>
-      <c r="E42" s="91"/>
-      <c r="F42" s="92"/>
-      <c r="G42" s="71"/>
-      <c r="H42" s="72"/>
-      <c r="I42" s="72"/>
-      <c r="J42" s="72"/>
-      <c r="K42" s="73"/>
+      <c r="A42" s="81"/>
+      <c r="B42" s="82"/>
+      <c r="C42" s="82"/>
+      <c r="D42" s="82"/>
+      <c r="E42" s="82"/>
+      <c r="F42" s="83"/>
+      <c r="G42" s="65"/>
+      <c r="H42" s="66"/>
+      <c r="I42" s="66"/>
+      <c r="J42" s="66"/>
+      <c r="K42" s="67"/>
       <c r="L42" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M42" s="102"/>
-      <c r="N42" s="72"/>
-      <c r="O42" s="72"/>
-      <c r="P42" s="72"/>
-      <c r="Q42" s="73"/>
+      <c r="M42" s="77"/>
+      <c r="N42" s="66"/>
+      <c r="O42" s="66"/>
+      <c r="P42" s="66"/>
+      <c r="Q42" s="67"/>
     </row>
     <row r="43" spans="1:17" ht="12.75">
-      <c r="A43" s="114" t="s">
+      <c r="A43" s="71" t="s">
         <v>206</v>
       </c>
-      <c r="B43" s="56"/>
-      <c r="C43" s="56"/>
-      <c r="D43" s="56"/>
-      <c r="E43" s="56"/>
-      <c r="F43" s="56"/>
-      <c r="G43" s="56"/>
-      <c r="H43" s="56"/>
-      <c r="I43" s="56"/>
-      <c r="J43" s="56"/>
-      <c r="K43" s="56"/>
-      <c r="L43" s="56"/>
-      <c r="M43" s="56"/>
-      <c r="N43" s="56"/>
-      <c r="O43" s="56"/>
-      <c r="P43" s="56"/>
-      <c r="Q43" s="57"/>
+      <c r="B43" s="54"/>
+      <c r="C43" s="54"/>
+      <c r="D43" s="54"/>
+      <c r="E43" s="54"/>
+      <c r="F43" s="54"/>
+      <c r="G43" s="54"/>
+      <c r="H43" s="54"/>
+      <c r="I43" s="54"/>
+      <c r="J43" s="54"/>
+      <c r="K43" s="54"/>
+      <c r="L43" s="54"/>
+      <c r="M43" s="54"/>
+      <c r="N43" s="54"/>
+      <c r="O43" s="54"/>
+      <c r="P43" s="54"/>
+      <c r="Q43" s="72"/>
     </row>
     <row r="44" spans="1:17" ht="30.75" customHeight="1">
-      <c r="A44" s="115" t="s">
+      <c r="A44" s="53" t="s">
         <v>170</v>
       </c>
-      <c r="B44" s="56"/>
-      <c r="C44" s="56"/>
-      <c r="D44" s="56"/>
-      <c r="E44" s="56"/>
-      <c r="F44" s="56"/>
-      <c r="G44" s="115" t="s">
+      <c r="B44" s="54"/>
+      <c r="C44" s="54"/>
+      <c r="D44" s="54"/>
+      <c r="E44" s="54"/>
+      <c r="F44" s="54"/>
+      <c r="G44" s="53" t="s">
         <v>200</v>
       </c>
-      <c r="H44" s="56"/>
-      <c r="I44" s="56"/>
-      <c r="J44" s="56"/>
-      <c r="K44" s="56"/>
-      <c r="L44" s="115" t="s">
+      <c r="H44" s="54"/>
+      <c r="I44" s="54"/>
+      <c r="J44" s="54"/>
+      <c r="K44" s="54"/>
+      <c r="L44" s="53" t="s">
         <v>171</v>
       </c>
-      <c r="M44" s="56"/>
-      <c r="N44" s="56"/>
-      <c r="O44" s="56"/>
-      <c r="P44" s="56"/>
-      <c r="Q44" s="57"/>
+      <c r="M44" s="54"/>
+      <c r="N44" s="54"/>
+      <c r="O44" s="54"/>
+      <c r="P44" s="54"/>
+      <c r="Q44" s="72"/>
     </row>
     <row r="45" spans="1:17" ht="15">
-      <c r="A45" s="125" t="s">
+      <c r="A45" s="70" t="s">
         <v>207</v>
       </c>
-      <c r="B45" s="86"/>
-      <c r="C45" s="86"/>
-      <c r="D45" s="86"/>
-      <c r="E45" s="86"/>
-      <c r="F45" s="86"/>
-      <c r="G45" s="117"/>
-      <c r="H45" s="69"/>
-      <c r="I45" s="69"/>
-      <c r="J45" s="69"/>
-      <c r="K45" s="70"/>
-      <c r="L45" s="101"/>
-      <c r="M45" s="66"/>
-      <c r="N45" s="66"/>
-      <c r="O45" s="66"/>
-      <c r="P45" s="66"/>
-      <c r="Q45" s="67"/>
+      <c r="B45" s="56"/>
+      <c r="C45" s="56"/>
+      <c r="D45" s="56"/>
+      <c r="E45" s="56"/>
+      <c r="F45" s="56"/>
+      <c r="G45" s="59"/>
+      <c r="H45" s="60"/>
+      <c r="I45" s="60"/>
+      <c r="J45" s="60"/>
+      <c r="K45" s="61"/>
+      <c r="L45" s="76"/>
+      <c r="M45" s="74"/>
+      <c r="N45" s="74"/>
+      <c r="O45" s="74"/>
+      <c r="P45" s="74"/>
+      <c r="Q45" s="75"/>
     </row>
     <row r="46" spans="1:17">
-      <c r="A46" s="88"/>
-      <c r="B46" s="54"/>
-      <c r="C46" s="54"/>
-      <c r="D46" s="54"/>
-      <c r="E46" s="54"/>
-      <c r="F46" s="54"/>
-      <c r="G46" s="71"/>
-      <c r="H46" s="72"/>
-      <c r="I46" s="72"/>
-      <c r="J46" s="72"/>
-      <c r="K46" s="73"/>
+      <c r="A46" s="57"/>
+      <c r="B46" s="58"/>
+      <c r="C46" s="58"/>
+      <c r="D46" s="58"/>
+      <c r="E46" s="58"/>
+      <c r="F46" s="58"/>
+      <c r="G46" s="65"/>
+      <c r="H46" s="66"/>
+      <c r="I46" s="66"/>
+      <c r="J46" s="66"/>
+      <c r="K46" s="67"/>
       <c r="L46" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M46" s="102"/>
-      <c r="N46" s="72"/>
-      <c r="O46" s="72"/>
-      <c r="P46" s="72"/>
-      <c r="Q46" s="73"/>
+      <c r="M46" s="77"/>
+      <c r="N46" s="66"/>
+      <c r="O46" s="66"/>
+      <c r="P46" s="66"/>
+      <c r="Q46" s="67"/>
     </row>
     <row r="47" spans="1:17" ht="15">
-      <c r="A47" s="125" t="s">
+      <c r="A47" s="70" t="s">
         <v>208</v>
       </c>
-      <c r="B47" s="86"/>
-      <c r="C47" s="86"/>
-      <c r="D47" s="86"/>
-      <c r="E47" s="86"/>
-      <c r="F47" s="86"/>
-      <c r="G47" s="117"/>
-      <c r="H47" s="69"/>
-      <c r="I47" s="69"/>
-      <c r="J47" s="69"/>
-      <c r="K47" s="70"/>
-      <c r="L47" s="101"/>
-      <c r="M47" s="66"/>
-      <c r="N47" s="66"/>
-      <c r="O47" s="66"/>
-      <c r="P47" s="66"/>
-      <c r="Q47" s="67"/>
+      <c r="B47" s="56"/>
+      <c r="C47" s="56"/>
+      <c r="D47" s="56"/>
+      <c r="E47" s="56"/>
+      <c r="F47" s="56"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="60"/>
+      <c r="I47" s="60"/>
+      <c r="J47" s="60"/>
+      <c r="K47" s="61"/>
+      <c r="L47" s="76"/>
+      <c r="M47" s="74"/>
+      <c r="N47" s="74"/>
+      <c r="O47" s="74"/>
+      <c r="P47" s="74"/>
+      <c r="Q47" s="75"/>
     </row>
     <row r="48" spans="1:17">
-      <c r="A48" s="88"/>
-      <c r="B48" s="54"/>
-      <c r="C48" s="54"/>
-      <c r="D48" s="54"/>
-      <c r="E48" s="54"/>
-      <c r="F48" s="54"/>
-      <c r="G48" s="71"/>
-      <c r="H48" s="72"/>
-      <c r="I48" s="72"/>
-      <c r="J48" s="72"/>
-      <c r="K48" s="73"/>
+      <c r="A48" s="57"/>
+      <c r="B48" s="58"/>
+      <c r="C48" s="58"/>
+      <c r="D48" s="58"/>
+      <c r="E48" s="58"/>
+      <c r="F48" s="58"/>
+      <c r="G48" s="65"/>
+      <c r="H48" s="66"/>
+      <c r="I48" s="66"/>
+      <c r="J48" s="66"/>
+      <c r="K48" s="67"/>
       <c r="L48" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M48" s="102"/>
-      <c r="N48" s="72"/>
-      <c r="O48" s="72"/>
-      <c r="P48" s="72"/>
-      <c r="Q48" s="73"/>
+      <c r="M48" s="77"/>
+      <c r="N48" s="66"/>
+      <c r="O48" s="66"/>
+      <c r="P48" s="66"/>
+      <c r="Q48" s="67"/>
     </row>
     <row r="49" spans="1:17" ht="15">
-      <c r="A49" s="125" t="s">
+      <c r="A49" s="70" t="s">
         <v>209</v>
       </c>
-      <c r="B49" s="86"/>
-      <c r="C49" s="86"/>
-      <c r="D49" s="86"/>
-      <c r="E49" s="86"/>
-      <c r="F49" s="86"/>
-      <c r="G49" s="117"/>
-      <c r="H49" s="69"/>
-      <c r="I49" s="69"/>
-      <c r="J49" s="69"/>
-      <c r="K49" s="70"/>
-      <c r="L49" s="101"/>
-      <c r="M49" s="66"/>
-      <c r="N49" s="66"/>
-      <c r="O49" s="66"/>
-      <c r="P49" s="66"/>
-      <c r="Q49" s="67"/>
+      <c r="B49" s="56"/>
+      <c r="C49" s="56"/>
+      <c r="D49" s="56"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="59"/>
+      <c r="H49" s="60"/>
+      <c r="I49" s="60"/>
+      <c r="J49" s="60"/>
+      <c r="K49" s="61"/>
+      <c r="L49" s="76"/>
+      <c r="M49" s="74"/>
+      <c r="N49" s="74"/>
+      <c r="O49" s="74"/>
+      <c r="P49" s="74"/>
+      <c r="Q49" s="75"/>
     </row>
     <row r="50" spans="1:17">
-      <c r="A50" s="88"/>
-      <c r="B50" s="54"/>
-      <c r="C50" s="54"/>
-      <c r="D50" s="54"/>
-      <c r="E50" s="54"/>
-      <c r="F50" s="54"/>
-      <c r="G50" s="71"/>
-      <c r="H50" s="72"/>
-      <c r="I50" s="72"/>
-      <c r="J50" s="72"/>
-      <c r="K50" s="73"/>
+      <c r="A50" s="57"/>
+      <c r="B50" s="58"/>
+      <c r="C50" s="58"/>
+      <c r="D50" s="58"/>
+      <c r="E50" s="58"/>
+      <c r="F50" s="58"/>
+      <c r="G50" s="65"/>
+      <c r="H50" s="66"/>
+      <c r="I50" s="66"/>
+      <c r="J50" s="66"/>
+      <c r="K50" s="67"/>
       <c r="L50" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M50" s="102"/>
-      <c r="N50" s="72"/>
-      <c r="O50" s="72"/>
-      <c r="P50" s="72"/>
-      <c r="Q50" s="73"/>
+      <c r="M50" s="77"/>
+      <c r="N50" s="66"/>
+      <c r="O50" s="66"/>
+      <c r="P50" s="66"/>
+      <c r="Q50" s="67"/>
     </row>
     <row r="51" spans="1:17" ht="15">
-      <c r="A51" s="118" t="s">
+      <c r="A51" s="55" t="s">
         <v>210</v>
       </c>
-      <c r="B51" s="86"/>
-      <c r="C51" s="86"/>
-      <c r="D51" s="86"/>
-      <c r="E51" s="86"/>
-      <c r="F51" s="86"/>
-      <c r="G51" s="117"/>
-      <c r="H51" s="69"/>
-      <c r="I51" s="69"/>
-      <c r="J51" s="69"/>
-      <c r="K51" s="70"/>
-      <c r="L51" s="101"/>
-      <c r="M51" s="66"/>
-      <c r="N51" s="66"/>
-      <c r="O51" s="66"/>
-      <c r="P51" s="66"/>
-      <c r="Q51" s="67"/>
+      <c r="B51" s="56"/>
+      <c r="C51" s="56"/>
+      <c r="D51" s="56"/>
+      <c r="E51" s="56"/>
+      <c r="F51" s="56"/>
+      <c r="G51" s="59"/>
+      <c r="H51" s="60"/>
+      <c r="I51" s="60"/>
+      <c r="J51" s="60"/>
+      <c r="K51" s="61"/>
+      <c r="L51" s="76"/>
+      <c r="M51" s="74"/>
+      <c r="N51" s="74"/>
+      <c r="O51" s="74"/>
+      <c r="P51" s="74"/>
+      <c r="Q51" s="75"/>
     </row>
     <row r="52" spans="1:17">
-      <c r="A52" s="88"/>
-      <c r="B52" s="54"/>
-      <c r="C52" s="54"/>
-      <c r="D52" s="54"/>
-      <c r="E52" s="54"/>
-      <c r="F52" s="54"/>
-      <c r="G52" s="71"/>
-      <c r="H52" s="72"/>
-      <c r="I52" s="72"/>
-      <c r="J52" s="72"/>
-      <c r="K52" s="73"/>
+      <c r="A52" s="57"/>
+      <c r="B52" s="58"/>
+      <c r="C52" s="58"/>
+      <c r="D52" s="58"/>
+      <c r="E52" s="58"/>
+      <c r="F52" s="58"/>
+      <c r="G52" s="65"/>
+      <c r="H52" s="66"/>
+      <c r="I52" s="66"/>
+      <c r="J52" s="66"/>
+      <c r="K52" s="67"/>
       <c r="L52" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M52" s="102"/>
-      <c r="N52" s="72"/>
-      <c r="O52" s="72"/>
-      <c r="P52" s="72"/>
-      <c r="Q52" s="73"/>
+      <c r="M52" s="77"/>
+      <c r="N52" s="66"/>
+      <c r="O52" s="66"/>
+      <c r="P52" s="66"/>
+      <c r="Q52" s="67"/>
     </row>
     <row r="53" spans="1:17" ht="15">
-      <c r="A53" s="125" t="s">
+      <c r="A53" s="70" t="s">
         <v>211</v>
       </c>
-      <c r="B53" s="86"/>
-      <c r="C53" s="86"/>
-      <c r="D53" s="86"/>
-      <c r="E53" s="86"/>
-      <c r="F53" s="86"/>
-      <c r="G53" s="117"/>
-      <c r="H53" s="69"/>
-      <c r="I53" s="69"/>
-      <c r="J53" s="69"/>
-      <c r="K53" s="70"/>
-      <c r="L53" s="101"/>
-      <c r="M53" s="66"/>
-      <c r="N53" s="66"/>
-      <c r="O53" s="66"/>
-      <c r="P53" s="66"/>
-      <c r="Q53" s="67"/>
+      <c r="B53" s="56"/>
+      <c r="C53" s="56"/>
+      <c r="D53" s="56"/>
+      <c r="E53" s="56"/>
+      <c r="F53" s="56"/>
+      <c r="G53" s="59"/>
+      <c r="H53" s="60"/>
+      <c r="I53" s="60"/>
+      <c r="J53" s="60"/>
+      <c r="K53" s="61"/>
+      <c r="L53" s="76"/>
+      <c r="M53" s="74"/>
+      <c r="N53" s="74"/>
+      <c r="O53" s="74"/>
+      <c r="P53" s="74"/>
+      <c r="Q53" s="75"/>
     </row>
     <row r="54" spans="1:17">
-      <c r="A54" s="88"/>
-      <c r="B54" s="54"/>
-      <c r="C54" s="54"/>
-      <c r="D54" s="54"/>
-      <c r="E54" s="54"/>
-      <c r="F54" s="54"/>
-      <c r="G54" s="71"/>
-      <c r="H54" s="72"/>
-      <c r="I54" s="72"/>
-      <c r="J54" s="72"/>
-      <c r="K54" s="73"/>
+      <c r="A54" s="57"/>
+      <c r="B54" s="58"/>
+      <c r="C54" s="58"/>
+      <c r="D54" s="58"/>
+      <c r="E54" s="58"/>
+      <c r="F54" s="58"/>
+      <c r="G54" s="65"/>
+      <c r="H54" s="66"/>
+      <c r="I54" s="66"/>
+      <c r="J54" s="66"/>
+      <c r="K54" s="67"/>
       <c r="L54" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M54" s="102"/>
-      <c r="N54" s="72"/>
-      <c r="O54" s="72"/>
-      <c r="P54" s="72"/>
-      <c r="Q54" s="73"/>
+      <c r="M54" s="77"/>
+      <c r="N54" s="66"/>
+      <c r="O54" s="66"/>
+      <c r="P54" s="66"/>
+      <c r="Q54" s="67"/>
     </row>
     <row r="55" spans="1:17" ht="15">
-      <c r="A55" s="125" t="s">
+      <c r="A55" s="70" t="s">
         <v>212</v>
       </c>
-      <c r="B55" s="86"/>
-      <c r="C55" s="86"/>
-      <c r="D55" s="86"/>
-      <c r="E55" s="86"/>
-      <c r="F55" s="86"/>
-      <c r="G55" s="117"/>
-      <c r="H55" s="69"/>
-      <c r="I55" s="69"/>
-      <c r="J55" s="69"/>
-      <c r="K55" s="70"/>
-      <c r="L55" s="101"/>
-      <c r="M55" s="66"/>
-      <c r="N55" s="66"/>
-      <c r="O55" s="66"/>
-      <c r="P55" s="66"/>
-      <c r="Q55" s="67"/>
+      <c r="B55" s="56"/>
+      <c r="C55" s="56"/>
+      <c r="D55" s="56"/>
+      <c r="E55" s="56"/>
+      <c r="F55" s="56"/>
+      <c r="G55" s="59"/>
+      <c r="H55" s="60"/>
+      <c r="I55" s="60"/>
+      <c r="J55" s="60"/>
+      <c r="K55" s="61"/>
+      <c r="L55" s="76"/>
+      <c r="M55" s="74"/>
+      <c r="N55" s="74"/>
+      <c r="O55" s="74"/>
+      <c r="P55" s="74"/>
+      <c r="Q55" s="75"/>
     </row>
     <row r="56" spans="1:17">
-      <c r="A56" s="88"/>
-      <c r="B56" s="54"/>
-      <c r="C56" s="54"/>
-      <c r="D56" s="54"/>
-      <c r="E56" s="54"/>
-      <c r="F56" s="54"/>
-      <c r="G56" s="71"/>
-      <c r="H56" s="72"/>
-      <c r="I56" s="72"/>
-      <c r="J56" s="72"/>
-      <c r="K56" s="73"/>
+      <c r="A56" s="57"/>
+      <c r="B56" s="58"/>
+      <c r="C56" s="58"/>
+      <c r="D56" s="58"/>
+      <c r="E56" s="58"/>
+      <c r="F56" s="58"/>
+      <c r="G56" s="65"/>
+      <c r="H56" s="66"/>
+      <c r="I56" s="66"/>
+      <c r="J56" s="66"/>
+      <c r="K56" s="67"/>
       <c r="L56" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M56" s="102"/>
-      <c r="N56" s="72"/>
-      <c r="O56" s="72"/>
-      <c r="P56" s="72"/>
-      <c r="Q56" s="73"/>
+      <c r="M56" s="77"/>
+      <c r="N56" s="66"/>
+      <c r="O56" s="66"/>
+      <c r="P56" s="66"/>
+      <c r="Q56" s="67"/>
     </row>
     <row r="57" spans="1:17" ht="12.75">
-      <c r="A57" s="114" t="s">
+      <c r="A57" s="71" t="s">
         <v>213</v>
       </c>
-      <c r="B57" s="56"/>
-      <c r="C57" s="56"/>
-      <c r="D57" s="56"/>
-      <c r="E57" s="56"/>
-      <c r="F57" s="56"/>
-      <c r="G57" s="56"/>
-      <c r="H57" s="56"/>
-      <c r="I57" s="56"/>
-      <c r="J57" s="56"/>
-      <c r="K57" s="56"/>
-      <c r="L57" s="56"/>
-      <c r="M57" s="56"/>
-      <c r="N57" s="56"/>
-      <c r="O57" s="56"/>
-      <c r="P57" s="56"/>
-      <c r="Q57" s="57"/>
+      <c r="B57" s="54"/>
+      <c r="C57" s="54"/>
+      <c r="D57" s="54"/>
+      <c r="E57" s="54"/>
+      <c r="F57" s="54"/>
+      <c r="G57" s="54"/>
+      <c r="H57" s="54"/>
+      <c r="I57" s="54"/>
+      <c r="J57" s="54"/>
+      <c r="K57" s="54"/>
+      <c r="L57" s="54"/>
+      <c r="M57" s="54"/>
+      <c r="N57" s="54"/>
+      <c r="O57" s="54"/>
+      <c r="P57" s="54"/>
+      <c r="Q57" s="72"/>
     </row>
     <row r="58" spans="1:17" ht="27.75" customHeight="1">
-      <c r="A58" s="115" t="s">
+      <c r="A58" s="53" t="s">
         <v>170</v>
       </c>
-      <c r="B58" s="56"/>
-      <c r="C58" s="56"/>
-      <c r="D58" s="56"/>
-      <c r="E58" s="56"/>
-      <c r="F58" s="56"/>
-      <c r="G58" s="130" t="s">
+      <c r="B58" s="54"/>
+      <c r="C58" s="54"/>
+      <c r="D58" s="54"/>
+      <c r="E58" s="54"/>
+      <c r="F58" s="54"/>
+      <c r="G58" s="73" t="s">
         <v>200</v>
       </c>
-      <c r="H58" s="66"/>
-      <c r="I58" s="66"/>
-      <c r="J58" s="66"/>
-      <c r="K58" s="66"/>
-      <c r="L58" s="130" t="s">
+      <c r="H58" s="74"/>
+      <c r="I58" s="74"/>
+      <c r="J58" s="74"/>
+      <c r="K58" s="74"/>
+      <c r="L58" s="73" t="s">
         <v>171</v>
       </c>
-      <c r="M58" s="66"/>
-      <c r="N58" s="66"/>
-      <c r="O58" s="66"/>
-      <c r="P58" s="66"/>
-      <c r="Q58" s="67"/>
+      <c r="M58" s="74"/>
+      <c r="N58" s="74"/>
+      <c r="O58" s="74"/>
+      <c r="P58" s="74"/>
+      <c r="Q58" s="75"/>
     </row>
     <row r="59" spans="1:17" ht="15">
-      <c r="A59" s="118" t="s">
+      <c r="A59" s="55" t="s">
         <v>214</v>
       </c>
-      <c r="B59" s="86"/>
-      <c r="C59" s="86"/>
-      <c r="D59" s="86"/>
-      <c r="E59" s="86"/>
-      <c r="F59" s="86"/>
-      <c r="G59" s="117"/>
-      <c r="H59" s="69"/>
-      <c r="I59" s="69"/>
-      <c r="J59" s="69"/>
-      <c r="K59" s="70"/>
-      <c r="L59" s="101"/>
-      <c r="M59" s="66"/>
-      <c r="N59" s="66"/>
-      <c r="O59" s="66"/>
-      <c r="P59" s="66"/>
-      <c r="Q59" s="67"/>
+      <c r="B59" s="56"/>
+      <c r="C59" s="56"/>
+      <c r="D59" s="56"/>
+      <c r="E59" s="56"/>
+      <c r="F59" s="56"/>
+      <c r="G59" s="59"/>
+      <c r="H59" s="60"/>
+      <c r="I59" s="60"/>
+      <c r="J59" s="60"/>
+      <c r="K59" s="61"/>
+      <c r="L59" s="76"/>
+      <c r="M59" s="74"/>
+      <c r="N59" s="74"/>
+      <c r="O59" s="74"/>
+      <c r="P59" s="74"/>
+      <c r="Q59" s="75"/>
     </row>
     <row r="60" spans="1:17" ht="15">
-      <c r="A60" s="88"/>
-      <c r="B60" s="54"/>
-      <c r="C60" s="54"/>
-      <c r="D60" s="54"/>
-      <c r="E60" s="54"/>
-      <c r="F60" s="54"/>
-      <c r="G60" s="119"/>
-      <c r="H60" s="120"/>
-      <c r="I60" s="120"/>
-      <c r="J60" s="120"/>
-      <c r="K60" s="121"/>
-      <c r="L60" s="101"/>
-      <c r="M60" s="66"/>
-      <c r="N60" s="66"/>
-      <c r="O60" s="66"/>
-      <c r="P60" s="66"/>
-      <c r="Q60" s="67"/>
+      <c r="A60" s="57"/>
+      <c r="B60" s="58"/>
+      <c r="C60" s="58"/>
+      <c r="D60" s="58"/>
+      <c r="E60" s="58"/>
+      <c r="F60" s="58"/>
+      <c r="G60" s="62"/>
+      <c r="H60" s="63"/>
+      <c r="I60" s="63"/>
+      <c r="J60" s="63"/>
+      <c r="K60" s="64"/>
+      <c r="L60" s="76"/>
+      <c r="M60" s="74"/>
+      <c r="N60" s="74"/>
+      <c r="O60" s="74"/>
+      <c r="P60" s="74"/>
+      <c r="Q60" s="75"/>
     </row>
     <row r="61" spans="1:17" ht="15">
-      <c r="A61" s="88"/>
-      <c r="B61" s="54"/>
-      <c r="C61" s="54"/>
-      <c r="D61" s="54"/>
-      <c r="E61" s="54"/>
-      <c r="F61" s="54"/>
-      <c r="G61" s="119"/>
-      <c r="H61" s="120"/>
-      <c r="I61" s="120"/>
-      <c r="J61" s="120"/>
-      <c r="K61" s="121"/>
-      <c r="L61" s="101"/>
-      <c r="M61" s="66"/>
-      <c r="N61" s="66"/>
-      <c r="O61" s="66"/>
-      <c r="P61" s="66"/>
-      <c r="Q61" s="67"/>
+      <c r="A61" s="57"/>
+      <c r="B61" s="58"/>
+      <c r="C61" s="58"/>
+      <c r="D61" s="58"/>
+      <c r="E61" s="58"/>
+      <c r="F61" s="58"/>
+      <c r="G61" s="62"/>
+      <c r="H61" s="63"/>
+      <c r="I61" s="63"/>
+      <c r="J61" s="63"/>
+      <c r="K61" s="64"/>
+      <c r="L61" s="76"/>
+      <c r="M61" s="74"/>
+      <c r="N61" s="74"/>
+      <c r="O61" s="74"/>
+      <c r="P61" s="74"/>
+      <c r="Q61" s="75"/>
     </row>
     <row r="62" spans="1:17" ht="15">
-      <c r="A62" s="88"/>
-      <c r="B62" s="54"/>
-      <c r="C62" s="54"/>
-      <c r="D62" s="54"/>
-      <c r="E62" s="54"/>
-      <c r="F62" s="54"/>
-      <c r="G62" s="119"/>
-      <c r="H62" s="120"/>
-      <c r="I62" s="120"/>
-      <c r="J62" s="120"/>
-      <c r="K62" s="121"/>
-      <c r="L62" s="101"/>
-      <c r="M62" s="66"/>
-      <c r="N62" s="66"/>
-      <c r="O62" s="66"/>
-      <c r="P62" s="66"/>
-      <c r="Q62" s="67"/>
+      <c r="A62" s="57"/>
+      <c r="B62" s="58"/>
+      <c r="C62" s="58"/>
+      <c r="D62" s="58"/>
+      <c r="E62" s="58"/>
+      <c r="F62" s="58"/>
+      <c r="G62" s="62"/>
+      <c r="H62" s="63"/>
+      <c r="I62" s="63"/>
+      <c r="J62" s="63"/>
+      <c r="K62" s="64"/>
+      <c r="L62" s="76"/>
+      <c r="M62" s="74"/>
+      <c r="N62" s="74"/>
+      <c r="O62" s="74"/>
+      <c r="P62" s="74"/>
+      <c r="Q62" s="75"/>
     </row>
     <row r="63" spans="1:17">
-      <c r="A63" s="88"/>
-      <c r="B63" s="54"/>
-      <c r="C63" s="54"/>
-      <c r="D63" s="54"/>
-      <c r="E63" s="54"/>
-      <c r="F63" s="54"/>
-      <c r="G63" s="71"/>
-      <c r="H63" s="72"/>
-      <c r="I63" s="72"/>
-      <c r="J63" s="72"/>
-      <c r="K63" s="73"/>
+      <c r="A63" s="57"/>
+      <c r="B63" s="58"/>
+      <c r="C63" s="58"/>
+      <c r="D63" s="58"/>
+      <c r="E63" s="58"/>
+      <c r="F63" s="58"/>
+      <c r="G63" s="65"/>
+      <c r="H63" s="66"/>
+      <c r="I63" s="66"/>
+      <c r="J63" s="66"/>
+      <c r="K63" s="67"/>
       <c r="L63" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M63" s="102"/>
-      <c r="N63" s="72"/>
-      <c r="O63" s="72"/>
-      <c r="P63" s="72"/>
-      <c r="Q63" s="73"/>
+      <c r="M63" s="77"/>
+      <c r="N63" s="66"/>
+      <c r="O63" s="66"/>
+      <c r="P63" s="66"/>
+      <c r="Q63" s="67"/>
     </row>
     <row r="64" spans="1:17" ht="15">
-      <c r="A64" s="118" t="s">
+      <c r="A64" s="55" t="s">
         <v>215</v>
       </c>
-      <c r="B64" s="86"/>
-      <c r="C64" s="86"/>
-      <c r="D64" s="86"/>
-      <c r="E64" s="86"/>
-      <c r="F64" s="86"/>
-      <c r="G64" s="117"/>
-      <c r="H64" s="69"/>
-      <c r="I64" s="69"/>
-      <c r="J64" s="69"/>
-      <c r="K64" s="70"/>
-      <c r="L64" s="101"/>
-      <c r="M64" s="66"/>
-      <c r="N64" s="66"/>
-      <c r="O64" s="66"/>
-      <c r="P64" s="66"/>
-      <c r="Q64" s="67"/>
+      <c r="B64" s="56"/>
+      <c r="C64" s="56"/>
+      <c r="D64" s="56"/>
+      <c r="E64" s="56"/>
+      <c r="F64" s="56"/>
+      <c r="G64" s="59"/>
+      <c r="H64" s="60"/>
+      <c r="I64" s="60"/>
+      <c r="J64" s="60"/>
+      <c r="K64" s="61"/>
+      <c r="L64" s="76"/>
+      <c r="M64" s="74"/>
+      <c r="N64" s="74"/>
+      <c r="O64" s="74"/>
+      <c r="P64" s="74"/>
+      <c r="Q64" s="75"/>
     </row>
     <row r="65" spans="1:17">
-      <c r="A65" s="88"/>
-      <c r="B65" s="54"/>
-      <c r="C65" s="54"/>
-      <c r="D65" s="54"/>
-      <c r="E65" s="54"/>
-      <c r="F65" s="54"/>
-      <c r="G65" s="71"/>
-      <c r="H65" s="72"/>
-      <c r="I65" s="72"/>
-      <c r="J65" s="72"/>
-      <c r="K65" s="73"/>
+      <c r="A65" s="57"/>
+      <c r="B65" s="58"/>
+      <c r="C65" s="58"/>
+      <c r="D65" s="58"/>
+      <c r="E65" s="58"/>
+      <c r="F65" s="58"/>
+      <c r="G65" s="65"/>
+      <c r="H65" s="66"/>
+      <c r="I65" s="66"/>
+      <c r="J65" s="66"/>
+      <c r="K65" s="67"/>
       <c r="L65" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="M65" s="102"/>
-      <c r="N65" s="72"/>
-      <c r="O65" s="72"/>
-      <c r="P65" s="72"/>
-      <c r="Q65" s="73"/>
+      <c r="M65" s="77"/>
+      <c r="N65" s="66"/>
+      <c r="O65" s="66"/>
+      <c r="P65" s="66"/>
+      <c r="Q65" s="67"/>
     </row>
     <row r="66" spans="1:17" ht="33.75" customHeight="1">
-      <c r="A66" s="128" t="s">
+      <c r="A66" s="68" t="s">
         <v>216</v>
       </c>
-      <c r="B66" s="86"/>
-      <c r="C66" s="86"/>
-      <c r="D66" s="86"/>
-      <c r="E66" s="86"/>
-      <c r="F66" s="86"/>
-      <c r="G66" s="129"/>
-      <c r="H66" s="69"/>
-      <c r="I66" s="69"/>
-      <c r="J66" s="69"/>
-      <c r="K66" s="70"/>
-      <c r="L66" s="122"/>
-      <c r="M66" s="66"/>
-      <c r="N66" s="66"/>
-      <c r="O66" s="66"/>
-      <c r="P66" s="66"/>
-      <c r="Q66" s="67"/>
+      <c r="B66" s="56"/>
+      <c r="C66" s="56"/>
+      <c r="D66" s="56"/>
+      <c r="E66" s="56"/>
+      <c r="F66" s="56"/>
+      <c r="G66" s="69"/>
+      <c r="H66" s="60"/>
+      <c r="I66" s="60"/>
+      <c r="J66" s="60"/>
+      <c r="K66" s="61"/>
+      <c r="L66" s="90"/>
+      <c r="M66" s="74"/>
+      <c r="N66" s="74"/>
+      <c r="O66" s="74"/>
+      <c r="P66" s="74"/>
+      <c r="Q66" s="75"/>
     </row>
     <row r="67" spans="1:17" ht="33.75" customHeight="1">
-      <c r="A67" s="88"/>
-      <c r="B67" s="54"/>
-      <c r="C67" s="54"/>
-      <c r="D67" s="54"/>
-      <c r="E67" s="54"/>
-      <c r="F67" s="54"/>
-      <c r="G67" s="71"/>
-      <c r="H67" s="72"/>
-      <c r="I67" s="72"/>
-      <c r="J67" s="72"/>
-      <c r="K67" s="73"/>
+      <c r="A67" s="57"/>
+      <c r="B67" s="58"/>
+      <c r="C67" s="58"/>
+      <c r="D67" s="58"/>
+      <c r="E67" s="58"/>
+      <c r="F67" s="58"/>
+      <c r="G67" s="65"/>
+      <c r="H67" s="66"/>
+      <c r="I67" s="66"/>
+      <c r="J67" s="66"/>
+      <c r="K67" s="67"/>
       <c r="L67" s="52" t="s">
         <v>159</v>
       </c>
-      <c r="M67" s="123"/>
-      <c r="N67" s="72"/>
-      <c r="O67" s="72"/>
-      <c r="P67" s="72"/>
-      <c r="Q67" s="73"/>
+      <c r="M67" s="91"/>
+      <c r="N67" s="66"/>
+      <c r="O67" s="66"/>
+      <c r="P67" s="66"/>
+      <c r="Q67" s="67"/>
     </row>
     <row r="68" spans="1:17" ht="12.75">
-      <c r="A68" s="124" t="s">
+      <c r="A68" s="92" t="s">
         <v>219</v>
       </c>
-      <c r="B68" s="56"/>
-      <c r="C68" s="56"/>
-      <c r="D68" s="56"/>
-      <c r="E68" s="56"/>
-      <c r="F68" s="56"/>
-      <c r="G68" s="56"/>
-      <c r="H68" s="56"/>
-      <c r="I68" s="56"/>
-      <c r="J68" s="56"/>
-      <c r="K68" s="56"/>
-      <c r="L68" s="56"/>
-      <c r="M68" s="56"/>
-      <c r="N68" s="56"/>
-      <c r="O68" s="56"/>
-      <c r="P68" s="56"/>
-      <c r="Q68" s="57"/>
+      <c r="B68" s="54"/>
+      <c r="C68" s="54"/>
+      <c r="D68" s="54"/>
+      <c r="E68" s="54"/>
+      <c r="F68" s="54"/>
+      <c r="G68" s="54"/>
+      <c r="H68" s="54"/>
+      <c r="I68" s="54"/>
+      <c r="J68" s="54"/>
+      <c r="K68" s="54"/>
+      <c r="L68" s="54"/>
+      <c r="M68" s="54"/>
+      <c r="N68" s="54"/>
+      <c r="O68" s="54"/>
+      <c r="P68" s="54"/>
+      <c r="Q68" s="72"/>
     </row>
     <row r="69" spans="1:17" ht="90" customHeight="1">
-      <c r="A69" s="131"/>
-      <c r="B69" s="66"/>
-      <c r="C69" s="66"/>
-      <c r="D69" s="66"/>
-      <c r="E69" s="66"/>
-      <c r="F69" s="66"/>
-      <c r="G69" s="66"/>
-      <c r="H69" s="66"/>
-      <c r="I69" s="66"/>
-      <c r="J69" s="66"/>
-      <c r="K69" s="66"/>
-      <c r="L69" s="66"/>
-      <c r="M69" s="66"/>
-      <c r="N69" s="66"/>
-      <c r="O69" s="66"/>
-      <c r="P69" s="66"/>
-      <c r="Q69" s="67"/>
+      <c r="A69" s="78"/>
+      <c r="B69" s="74"/>
+      <c r="C69" s="74"/>
+      <c r="D69" s="74"/>
+      <c r="E69" s="74"/>
+      <c r="F69" s="74"/>
+      <c r="G69" s="74"/>
+      <c r="H69" s="74"/>
+      <c r="I69" s="74"/>
+      <c r="J69" s="74"/>
+      <c r="K69" s="74"/>
+      <c r="L69" s="74"/>
+      <c r="M69" s="74"/>
+      <c r="N69" s="74"/>
+      <c r="O69" s="74"/>
+      <c r="P69" s="74"/>
+      <c r="Q69" s="75"/>
     </row>
     <row r="70" spans="1:17" ht="18" customHeight="1">
-      <c r="A70" s="118" t="s">
+      <c r="A70" s="55" t="s">
         <v>217</v>
       </c>
-      <c r="B70" s="86"/>
-      <c r="C70" s="86"/>
-      <c r="D70" s="86"/>
-      <c r="E70" s="86"/>
-      <c r="F70" s="86"/>
-      <c r="G70" s="86"/>
-      <c r="H70" s="86"/>
-      <c r="I70" s="86"/>
-      <c r="J70" s="86"/>
-      <c r="K70" s="86"/>
-      <c r="L70" s="86"/>
-      <c r="M70" s="86"/>
-      <c r="N70" s="86"/>
-      <c r="O70" s="86"/>
-      <c r="P70" s="86"/>
-      <c r="Q70" s="87"/>
+      <c r="B70" s="56"/>
+      <c r="C70" s="56"/>
+      <c r="D70" s="56"/>
+      <c r="E70" s="56"/>
+      <c r="F70" s="56"/>
+      <c r="G70" s="56"/>
+      <c r="H70" s="56"/>
+      <c r="I70" s="56"/>
+      <c r="J70" s="56"/>
+      <c r="K70" s="56"/>
+      <c r="L70" s="56"/>
+      <c r="M70" s="56"/>
+      <c r="N70" s="56"/>
+      <c r="O70" s="56"/>
+      <c r="P70" s="56"/>
+      <c r="Q70" s="79"/>
     </row>
     <row r="71" spans="1:17" ht="18" customHeight="1">
-      <c r="A71" s="88"/>
-      <c r="B71" s="54"/>
-      <c r="C71" s="54"/>
-      <c r="D71" s="54"/>
-      <c r="E71" s="54"/>
-      <c r="F71" s="54"/>
-      <c r="G71" s="54"/>
-      <c r="H71" s="54"/>
-      <c r="I71" s="54"/>
-      <c r="J71" s="54"/>
-      <c r="K71" s="54"/>
-      <c r="L71" s="54"/>
-      <c r="M71" s="54"/>
-      <c r="N71" s="54"/>
-      <c r="O71" s="54"/>
-      <c r="P71" s="54"/>
-      <c r="Q71" s="89"/>
+      <c r="A71" s="57"/>
+      <c r="B71" s="58"/>
+      <c r="C71" s="58"/>
+      <c r="D71" s="58"/>
+      <c r="E71" s="58"/>
+      <c r="F71" s="58"/>
+      <c r="G71" s="58"/>
+      <c r="H71" s="58"/>
+      <c r="I71" s="58"/>
+      <c r="J71" s="58"/>
+      <c r="K71" s="58"/>
+      <c r="L71" s="58"/>
+      <c r="M71" s="58"/>
+      <c r="N71" s="58"/>
+      <c r="O71" s="58"/>
+      <c r="P71" s="58"/>
+      <c r="Q71" s="80"/>
     </row>
     <row r="72" spans="1:17" ht="18" customHeight="1">
-      <c r="A72" s="90"/>
-      <c r="B72" s="91"/>
-      <c r="C72" s="91"/>
-      <c r="D72" s="91"/>
-      <c r="E72" s="91"/>
-      <c r="F72" s="91"/>
-      <c r="G72" s="91"/>
-      <c r="H72" s="91"/>
-      <c r="I72" s="91"/>
-      <c r="J72" s="91"/>
-      <c r="K72" s="91"/>
-      <c r="L72" s="91"/>
-      <c r="M72" s="91"/>
-      <c r="N72" s="91"/>
-      <c r="O72" s="91"/>
-      <c r="P72" s="91"/>
-      <c r="Q72" s="92"/>
+      <c r="A72" s="81"/>
+      <c r="B72" s="82"/>
+      <c r="C72" s="82"/>
+      <c r="D72" s="82"/>
+      <c r="E72" s="82"/>
+      <c r="F72" s="82"/>
+      <c r="G72" s="82"/>
+      <c r="H72" s="82"/>
+      <c r="I72" s="82"/>
+      <c r="J72" s="82"/>
+      <c r="K72" s="82"/>
+      <c r="L72" s="82"/>
+      <c r="M72" s="82"/>
+      <c r="N72" s="82"/>
+      <c r="O72" s="82"/>
+      <c r="P72" s="82"/>
+      <c r="Q72" s="83"/>
     </row>
     <row r="73" spans="1:17">
-      <c r="A73" s="61" t="s">
+      <c r="A73" s="87" t="s">
         <v>218</v>
       </c>
-      <c r="B73" s="56"/>
-      <c r="C73" s="56"/>
-      <c r="D73" s="56"/>
-      <c r="E73" s="56"/>
-      <c r="F73" s="56"/>
-      <c r="G73" s="56"/>
-      <c r="H73" s="56"/>
-      <c r="I73" s="56"/>
-      <c r="J73" s="56"/>
-      <c r="K73" s="56"/>
-      <c r="L73" s="56"/>
-      <c r="M73" s="56"/>
-      <c r="N73" s="56"/>
-      <c r="O73" s="56"/>
-      <c r="P73" s="56"/>
-      <c r="Q73" s="57"/>
+      <c r="B73" s="54"/>
+      <c r="C73" s="54"/>
+      <c r="D73" s="54"/>
+      <c r="E73" s="54"/>
+      <c r="F73" s="54"/>
+      <c r="G73" s="54"/>
+      <c r="H73" s="54"/>
+      <c r="I73" s="54"/>
+      <c r="J73" s="54"/>
+      <c r="K73" s="54"/>
+      <c r="L73" s="54"/>
+      <c r="M73" s="54"/>
+      <c r="N73" s="54"/>
+      <c r="O73" s="54"/>
+      <c r="P73" s="54"/>
+      <c r="Q73" s="72"/>
     </row>
     <row r="74" spans="1:17" ht="15">
-      <c r="A74" s="126" t="s">
+      <c r="A74" s="84" t="s">
         <v>156</v>
       </c>
-      <c r="B74" s="57"/>
-      <c r="C74" s="132"/>
-      <c r="D74" s="66"/>
-      <c r="E74" s="66"/>
-      <c r="F74" s="66"/>
-      <c r="G74" s="66"/>
-      <c r="H74" s="66"/>
-      <c r="I74" s="67"/>
+      <c r="B74" s="72"/>
+      <c r="C74" s="88"/>
+      <c r="D74" s="74"/>
+      <c r="E74" s="74"/>
+      <c r="F74" s="74"/>
+      <c r="G74" s="74"/>
+      <c r="H74" s="74"/>
+      <c r="I74" s="75"/>
       <c r="J74" s="40" t="s">
         <v>152</v>
       </c>
-      <c r="K74" s="105"/>
-      <c r="L74" s="66"/>
-      <c r="M74" s="66"/>
-      <c r="N74" s="66"/>
-      <c r="O74" s="66"/>
-      <c r="P74" s="66"/>
-      <c r="Q74" s="67"/>
+      <c r="K74" s="85"/>
+      <c r="L74" s="74"/>
+      <c r="M74" s="74"/>
+      <c r="N74" s="74"/>
+      <c r="O74" s="74"/>
+      <c r="P74" s="74"/>
+      <c r="Q74" s="75"/>
     </row>
     <row r="75" spans="1:17" ht="15">
-      <c r="A75" s="126" t="s">
+      <c r="A75" s="84" t="s">
         <v>156</v>
       </c>
-      <c r="B75" s="57"/>
-      <c r="C75" s="105"/>
-      <c r="D75" s="66"/>
-      <c r="E75" s="66"/>
-      <c r="F75" s="66"/>
-      <c r="G75" s="66"/>
-      <c r="H75" s="66"/>
-      <c r="I75" s="67"/>
+      <c r="B75" s="72"/>
+      <c r="C75" s="85"/>
+      <c r="D75" s="74"/>
+      <c r="E75" s="74"/>
+      <c r="F75" s="74"/>
+      <c r="G75" s="74"/>
+      <c r="H75" s="74"/>
+      <c r="I75" s="75"/>
       <c r="J75" s="40" t="s">
         <v>152</v>
       </c>
-      <c r="K75" s="105"/>
-      <c r="L75" s="66"/>
-      <c r="M75" s="66"/>
-      <c r="N75" s="66"/>
-      <c r="O75" s="66"/>
-      <c r="P75" s="66"/>
-      <c r="Q75" s="67"/>
+      <c r="K75" s="85"/>
+      <c r="L75" s="74"/>
+      <c r="M75" s="74"/>
+      <c r="N75" s="74"/>
+      <c r="O75" s="74"/>
+      <c r="P75" s="74"/>
+      <c r="Q75" s="75"/>
     </row>
     <row r="76" spans="1:17" ht="15">
-      <c r="A76" s="126" t="s">
+      <c r="A76" s="84" t="s">
         <v>156</v>
       </c>
-      <c r="B76" s="57"/>
-      <c r="C76" s="105"/>
-      <c r="D76" s="66"/>
-      <c r="E76" s="66"/>
-      <c r="F76" s="66"/>
-      <c r="G76" s="66"/>
-      <c r="H76" s="66"/>
-      <c r="I76" s="67"/>
+      <c r="B76" s="72"/>
+      <c r="C76" s="85"/>
+      <c r="D76" s="74"/>
+      <c r="E76" s="74"/>
+      <c r="F76" s="74"/>
+      <c r="G76" s="74"/>
+      <c r="H76" s="74"/>
+      <c r="I76" s="75"/>
       <c r="J76" s="40" t="s">
         <v>152</v>
       </c>
-      <c r="K76" s="105"/>
-      <c r="L76" s="66"/>
-      <c r="M76" s="66"/>
-      <c r="N76" s="66"/>
-      <c r="O76" s="66"/>
-      <c r="P76" s="66"/>
-      <c r="Q76" s="67"/>
+      <c r="K76" s="85"/>
+      <c r="L76" s="74"/>
+      <c r="M76" s="74"/>
+      <c r="N76" s="74"/>
+      <c r="O76" s="74"/>
+      <c r="P76" s="74"/>
+      <c r="Q76" s="75"/>
     </row>
     <row r="77" spans="1:17" ht="12.75">
-      <c r="A77" s="127" t="s">
+      <c r="A77" s="86" t="s">
         <v>157</v>
       </c>
-      <c r="B77" s="56"/>
-      <c r="C77" s="56"/>
-      <c r="D77" s="56"/>
-      <c r="E77" s="56"/>
-      <c r="F77" s="56"/>
-      <c r="G77" s="56"/>
-      <c r="H77" s="56"/>
-      <c r="I77" s="56"/>
-      <c r="J77" s="56"/>
-      <c r="K77" s="56"/>
-      <c r="L77" s="56"/>
-      <c r="M77" s="56"/>
-      <c r="N77" s="56"/>
-      <c r="O77" s="56"/>
-      <c r="P77" s="56"/>
-      <c r="Q77" s="57"/>
+      <c r="B77" s="54"/>
+      <c r="C77" s="54"/>
+      <c r="D77" s="54"/>
+      <c r="E77" s="54"/>
+      <c r="F77" s="54"/>
+      <c r="G77" s="54"/>
+      <c r="H77" s="54"/>
+      <c r="I77" s="54"/>
+      <c r="J77" s="54"/>
+      <c r="K77" s="54"/>
+      <c r="L77" s="54"/>
+      <c r="M77" s="54"/>
+      <c r="N77" s="54"/>
+      <c r="O77" s="54"/>
+      <c r="P77" s="54"/>
+      <c r="Q77" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="164">
+    <mergeCell ref="L13:Q13"/>
+    <mergeCell ref="A14:Q14"/>
+    <mergeCell ref="A15:Q15"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="K16:N16"/>
+    <mergeCell ref="O16:Q17"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:I13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="L18:N18"/>
+    <mergeCell ref="O18:Q18"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L7:Q7"/>
+    <mergeCell ref="A1:E4"/>
+    <mergeCell ref="F1:O4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A5:Q5"/>
+    <mergeCell ref="A6:Q6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="D7:I7"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="D8:I8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:Q8"/>
+    <mergeCell ref="D9:I9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:Q9"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="L11:Q11"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="L10:Q10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:I11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="L12:Q12"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="L37:Q37"/>
+    <mergeCell ref="M38:Q38"/>
+    <mergeCell ref="L30:Q30"/>
+    <mergeCell ref="M31:Q31"/>
+    <mergeCell ref="L32:Q32"/>
+    <mergeCell ref="M33:Q33"/>
+    <mergeCell ref="L34:Q34"/>
+    <mergeCell ref="L35:Q35"/>
+    <mergeCell ref="L36:Q36"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="O20:Q20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="L22:N22"/>
+    <mergeCell ref="O22:P22"/>
+    <mergeCell ref="A23:Q23"/>
+    <mergeCell ref="N24:Q24"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A25:Q25"/>
+    <mergeCell ref="A26:Q26"/>
+    <mergeCell ref="A27:Q27"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="L29:Q29"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:F31"/>
+    <mergeCell ref="G30:K31"/>
+    <mergeCell ref="A32:F33"/>
+    <mergeCell ref="G32:K33"/>
+    <mergeCell ref="A34:F38"/>
+    <mergeCell ref="G34:K38"/>
+    <mergeCell ref="L64:Q64"/>
+    <mergeCell ref="M65:Q65"/>
+    <mergeCell ref="L66:Q66"/>
+    <mergeCell ref="M67:Q67"/>
+    <mergeCell ref="A68:Q68"/>
+    <mergeCell ref="A39:F42"/>
+    <mergeCell ref="G39:K42"/>
+    <mergeCell ref="L39:Q39"/>
+    <mergeCell ref="L40:Q40"/>
+    <mergeCell ref="L41:Q41"/>
+    <mergeCell ref="M42:Q42"/>
+    <mergeCell ref="A43:Q43"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="L44:Q44"/>
+    <mergeCell ref="A45:F46"/>
+    <mergeCell ref="G45:K46"/>
+    <mergeCell ref="L45:Q45"/>
+    <mergeCell ref="M46:Q46"/>
+    <mergeCell ref="L51:Q51"/>
+    <mergeCell ref="A69:Q69"/>
+    <mergeCell ref="A70:Q72"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="C76:I76"/>
+    <mergeCell ref="K76:Q76"/>
+    <mergeCell ref="A77:Q77"/>
+    <mergeCell ref="A73:Q73"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="C74:I74"/>
+    <mergeCell ref="K74:Q74"/>
+    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="C75:I75"/>
+    <mergeCell ref="K75:Q75"/>
+    <mergeCell ref="L55:Q55"/>
+    <mergeCell ref="M56:Q56"/>
+    <mergeCell ref="A47:F48"/>
+    <mergeCell ref="G47:K48"/>
+    <mergeCell ref="L47:Q47"/>
+    <mergeCell ref="M48:Q48"/>
+    <mergeCell ref="G49:K50"/>
+    <mergeCell ref="L49:Q49"/>
+    <mergeCell ref="M50:Q50"/>
+    <mergeCell ref="A55:F56"/>
     <mergeCell ref="A58:F58"/>
     <mergeCell ref="A59:F63"/>
     <mergeCell ref="G59:K63"/>
@@ -14448,146 +14588,6 @@
     <mergeCell ref="M52:Q52"/>
     <mergeCell ref="L53:Q53"/>
     <mergeCell ref="M54:Q54"/>
-    <mergeCell ref="L55:Q55"/>
-    <mergeCell ref="M56:Q56"/>
-    <mergeCell ref="A47:F48"/>
-    <mergeCell ref="G47:K48"/>
-    <mergeCell ref="L47:Q47"/>
-    <mergeCell ref="M48:Q48"/>
-    <mergeCell ref="G49:K50"/>
-    <mergeCell ref="L49:Q49"/>
-    <mergeCell ref="M50:Q50"/>
-    <mergeCell ref="A55:F56"/>
-    <mergeCell ref="A69:Q69"/>
-    <mergeCell ref="A70:Q72"/>
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="C76:I76"/>
-    <mergeCell ref="K76:Q76"/>
-    <mergeCell ref="A77:Q77"/>
-    <mergeCell ref="A73:Q73"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="C74:I74"/>
-    <mergeCell ref="K74:Q74"/>
-    <mergeCell ref="A75:B75"/>
-    <mergeCell ref="C75:I75"/>
-    <mergeCell ref="K75:Q75"/>
-    <mergeCell ref="A32:F33"/>
-    <mergeCell ref="G32:K33"/>
-    <mergeCell ref="A34:F38"/>
-    <mergeCell ref="G34:K38"/>
-    <mergeCell ref="L64:Q64"/>
-    <mergeCell ref="M65:Q65"/>
-    <mergeCell ref="L66:Q66"/>
-    <mergeCell ref="M67:Q67"/>
-    <mergeCell ref="A68:Q68"/>
-    <mergeCell ref="A39:F42"/>
-    <mergeCell ref="G39:K42"/>
-    <mergeCell ref="L39:Q39"/>
-    <mergeCell ref="L40:Q40"/>
-    <mergeCell ref="L41:Q41"/>
-    <mergeCell ref="M42:Q42"/>
-    <mergeCell ref="A43:Q43"/>
-    <mergeCell ref="A44:F44"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="L44:Q44"/>
-    <mergeCell ref="A45:F46"/>
-    <mergeCell ref="G45:K46"/>
-    <mergeCell ref="L45:Q45"/>
-    <mergeCell ref="M46:Q46"/>
-    <mergeCell ref="L51:Q51"/>
-    <mergeCell ref="A25:Q25"/>
-    <mergeCell ref="A26:Q26"/>
-    <mergeCell ref="A27:Q27"/>
-    <mergeCell ref="A28:Q28"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="L29:Q29"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A30:F31"/>
-    <mergeCell ref="G30:K31"/>
-    <mergeCell ref="O20:Q20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="G24:K24"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="F22:I22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="L22:N22"/>
-    <mergeCell ref="O22:P22"/>
-    <mergeCell ref="A23:Q23"/>
-    <mergeCell ref="N24:Q24"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="L37:Q37"/>
-    <mergeCell ref="M38:Q38"/>
-    <mergeCell ref="L30:Q30"/>
-    <mergeCell ref="M31:Q31"/>
-    <mergeCell ref="L32:Q32"/>
-    <mergeCell ref="M33:Q33"/>
-    <mergeCell ref="L34:Q34"/>
-    <mergeCell ref="L35:Q35"/>
-    <mergeCell ref="L36:Q36"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:I10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="L10:Q10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:I11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D12:I12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="L12:Q12"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="H18:J18"/>
-    <mergeCell ref="L18:N18"/>
-    <mergeCell ref="O18:Q18"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="L7:Q7"/>
-    <mergeCell ref="A1:E4"/>
-    <mergeCell ref="F1:O4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A5:Q5"/>
-    <mergeCell ref="A6:Q6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="D7:I7"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="D8:I8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L8:Q8"/>
-    <mergeCell ref="D9:I9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:Q9"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="L11:Q11"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="L13:Q13"/>
-    <mergeCell ref="A14:Q14"/>
-    <mergeCell ref="A15:Q15"/>
-    <mergeCell ref="A16:J16"/>
-    <mergeCell ref="K16:N16"/>
-    <mergeCell ref="O16:Q17"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="L17:N17"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="D13:I13"/>
-    <mergeCell ref="J13:K13"/>
   </mergeCells>
   <dataValidations count="25">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L39" xr:uid="{00000000-0002-0000-0800-000000000000}">

</xml_diff>

<commit_message>
Release v1.0.17: include updated templates and form/export fixes
</commit_message>
<xml_diff>
--- a/templates/contratacion_incluyente.xlsx
+++ b/templates/contratacion_incluyente.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aaron\Desktop\RECA_INCLUSION_LABORAL\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28DCAD81-B6FD-413F-97CF-3461C2DAD74C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EE3FEC2-84AC-4FEC-9979-997A711D0E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,28 +35,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </valueMetadata>
-</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1518,7 +1496,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1613,24 +1591,6 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1652,132 +1612,18 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1792,23 +1638,24 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1816,34 +1663,64 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1851,6 +1728,126 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3200,68 +3197,53 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-</richValueRels>
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>152770</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9ABA5B9A-0C44-61DB-3159-B80C6D74A8E8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="1"/>
+          <a:ext cx="2886075" cy="638544"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3512,48 +3494,48 @@
       <c r="P1" s="4"/>
       <c r="Q1" s="4"/>
       <c r="R1" s="4"/>
-      <c r="S1" s="131" t="s">
+      <c r="S1" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="T1" s="58"/>
-      <c r="U1" s="58"/>
-      <c r="V1" s="58"/>
-      <c r="W1" s="131" t="s">
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="86" t="s">
         <v>4</v>
       </c>
-      <c r="X1" s="58"/>
-      <c r="Y1" s="58"/>
-      <c r="Z1" s="58"/>
-      <c r="AA1" s="131" t="s">
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="86" t="s">
         <v>5</v>
       </c>
-      <c r="AB1" s="58"/>
-      <c r="AC1" s="58"/>
-      <c r="AD1" s="58"/>
-      <c r="AE1" s="131" t="s">
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+      <c r="AE1" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="AF1" s="58"/>
-      <c r="AG1" s="58"/>
-      <c r="AH1" s="58"/>
-      <c r="AI1" s="131" t="s">
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="AJ1" s="58"/>
-      <c r="AK1" s="58"/>
-      <c r="AL1" s="58"/>
-      <c r="AM1" s="131" t="s">
+      <c r="AJ1" s="62"/>
+      <c r="AK1" s="62"/>
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="86" t="s">
         <v>8</v>
       </c>
-      <c r="AN1" s="58"/>
-      <c r="AO1" s="58"/>
-      <c r="AP1" s="58"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
       <c r="AQ1" s="4"/>
-      <c r="AR1" s="131" t="s">
+      <c r="AR1" s="86" t="s">
         <v>9</v>
       </c>
-      <c r="AS1" s="58"/>
-      <c r="AT1" s="58"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
       <c r="AU1" s="4"/>
       <c r="AV1" s="4"/>
       <c r="AW1" s="4"/>
@@ -3634,11 +3616,11 @@
       <c r="AO2" s="7"/>
       <c r="AP2" s="7"/>
       <c r="AQ2" s="7"/>
-      <c r="AR2" s="131" t="s">
+      <c r="AR2" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="AS2" s="58"/>
-      <c r="AT2" s="58"/>
+      <c r="AS2" s="62"/>
+      <c r="AT2" s="62"/>
       <c r="AU2" s="7"/>
       <c r="AV2" s="7"/>
       <c r="AW2" s="7"/>
@@ -3718,11 +3700,11 @@
       <c r="AO3" s="7"/>
       <c r="AP3" s="7"/>
       <c r="AQ3" s="7"/>
-      <c r="AR3" s="131" t="s">
+      <c r="AR3" s="86" t="s">
         <v>25</v>
       </c>
-      <c r="AS3" s="58"/>
-      <c r="AT3" s="58"/>
+      <c r="AS3" s="62"/>
+      <c r="AT3" s="62"/>
       <c r="AU3" s="7"/>
       <c r="AV3" s="7"/>
       <c r="AW3" s="7"/>
@@ -3802,11 +3784,11 @@
       <c r="AO4" s="7"/>
       <c r="AP4" s="7"/>
       <c r="AQ4" s="7"/>
-      <c r="AR4" s="131" t="s">
+      <c r="AR4" s="86" t="s">
         <v>29</v>
       </c>
-      <c r="AS4" s="58"/>
-      <c r="AT4" s="58"/>
+      <c r="AS4" s="62"/>
+      <c r="AT4" s="62"/>
       <c r="AU4" s="7"/>
       <c r="AV4" s="7"/>
       <c r="AW4" s="7"/>
@@ -3886,11 +3868,11 @@
       <c r="AO5" s="7"/>
       <c r="AP5" s="7"/>
       <c r="AQ5" s="7"/>
-      <c r="AR5" s="131" t="s">
+      <c r="AR5" s="86" t="s">
         <v>34</v>
       </c>
-      <c r="AS5" s="58"/>
-      <c r="AT5" s="58"/>
+      <c r="AS5" s="62"/>
+      <c r="AT5" s="62"/>
       <c r="AU5" s="7"/>
       <c r="AV5" s="7"/>
       <c r="AW5" s="7"/>
@@ -3964,11 +3946,11 @@
       <c r="AO6" s="7"/>
       <c r="AP6" s="7"/>
       <c r="AQ6" s="7"/>
-      <c r="AR6" s="131" t="s">
+      <c r="AR6" s="86" t="s">
         <v>37</v>
       </c>
-      <c r="AS6" s="58"/>
-      <c r="AT6" s="58"/>
+      <c r="AS6" s="62"/>
+      <c r="AT6" s="62"/>
       <c r="AU6" s="7"/>
       <c r="AV6" s="7"/>
       <c r="AW6" s="7"/>
@@ -5920,31 +5902,31 @@
       <c r="A75" s="34" t="s">
         <v>134</v>
       </c>
-      <c r="B75" s="132" t="s">
+      <c r="B75" s="87" t="s">
         <v>135</v>
       </c>
-      <c r="C75" s="54"/>
-      <c r="D75" s="72"/>
+      <c r="C75" s="48"/>
+      <c r="D75" s="49"/>
     </row>
     <row r="76" spans="1:4" ht="25.5">
       <c r="A76" s="35" t="s">
         <v>136</v>
       </c>
-      <c r="B76" s="132" t="s">
+      <c r="B76" s="87" t="s">
         <v>137</v>
       </c>
-      <c r="C76" s="54"/>
-      <c r="D76" s="72"/>
+      <c r="C76" s="48"/>
+      <c r="D76" s="49"/>
     </row>
     <row r="77" spans="1:4" ht="12.75">
       <c r="A77" s="36" t="s">
         <v>138</v>
       </c>
-      <c r="B77" s="132" t="s">
+      <c r="B77" s="87" t="s">
         <v>139</v>
       </c>
-      <c r="C77" s="54"/>
-      <c r="D77" s="72"/>
+      <c r="C77" s="48"/>
+      <c r="D77" s="49"/>
     </row>
     <row r="82" spans="1:5" ht="17.25">
       <c r="A82" s="3" t="str">
@@ -12704,21 +12686,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="AA1:AD1"/>
+    <mergeCell ref="AE1:AH1"/>
+    <mergeCell ref="AI1:AL1"/>
+    <mergeCell ref="AM1:AP1"/>
+    <mergeCell ref="AR1:AT1"/>
+    <mergeCell ref="B75:D75"/>
+    <mergeCell ref="B76:D76"/>
+    <mergeCell ref="B77:D77"/>
+    <mergeCell ref="S1:V1"/>
+    <mergeCell ref="W1:Z1"/>
     <mergeCell ref="AR2:AT2"/>
     <mergeCell ref="AR3:AT3"/>
     <mergeCell ref="AR4:AT4"/>
     <mergeCell ref="AR5:AT5"/>
     <mergeCell ref="AR6:AT6"/>
-    <mergeCell ref="B75:D75"/>
-    <mergeCell ref="B76:D76"/>
-    <mergeCell ref="B77:D77"/>
-    <mergeCell ref="S1:V1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="AA1:AD1"/>
-    <mergeCell ref="AE1:AH1"/>
-    <mergeCell ref="AI1:AL1"/>
-    <mergeCell ref="AM1:AP1"/>
-    <mergeCell ref="AR1:AT1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A156" r:id="rId1" display="http://falabella.com/" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -12756,1687 +12738,1799 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="12.75">
-      <c r="A1" s="122" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="123" t="s">
+      <c r="A1" s="88"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="91" t="s">
         <v>172</v>
       </c>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="79"/>
-      <c r="P1" s="41" t="s">
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="89"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="92" t="s">
         <v>141</v>
       </c>
-      <c r="Q1" s="42" t="s">
+      <c r="Q1" s="93" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="12.75">
-      <c r="A2" s="57"/>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="58"/>
-      <c r="O2" s="80"/>
-      <c r="P2" s="43" t="s">
+      <c r="A2" s="94"/>
+      <c r="B2" s="95"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="95"/>
+      <c r="L2" s="95"/>
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="96"/>
+      <c r="P2" s="97" t="s">
         <v>174</v>
       </c>
-      <c r="Q2" s="44" t="s">
+      <c r="Q2" s="98" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="12.75">
-      <c r="A3" s="57"/>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="58"/>
-      <c r="L3" s="58"/>
-      <c r="M3" s="58"/>
-      <c r="N3" s="58"/>
-      <c r="O3" s="80"/>
-      <c r="P3" s="43" t="s">
+      <c r="A3" s="94"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="95"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="94"/>
+      <c r="G3" s="95"/>
+      <c r="H3" s="95"/>
+      <c r="I3" s="95"/>
+      <c r="J3" s="95"/>
+      <c r="K3" s="95"/>
+      <c r="L3" s="95"/>
+      <c r="M3" s="95"/>
+      <c r="N3" s="95"/>
+      <c r="O3" s="96"/>
+      <c r="P3" s="97" t="s">
         <v>175</v>
       </c>
-      <c r="Q3" s="45">
+      <c r="Q3" s="99">
         <v>45324</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="12.75">
-      <c r="A4" s="81"/>
-      <c r="B4" s="82"/>
-      <c r="C4" s="82"/>
-      <c r="D4" s="82"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="81"/>
-      <c r="G4" s="82"/>
-      <c r="H4" s="82"/>
-      <c r="I4" s="82"/>
-      <c r="J4" s="82"/>
-      <c r="K4" s="82"/>
-      <c r="L4" s="82"/>
-      <c r="M4" s="82"/>
-      <c r="N4" s="82"/>
-      <c r="O4" s="83"/>
-      <c r="P4" s="124" t="s">
+      <c r="A4" s="100"/>
+      <c r="B4" s="101"/>
+      <c r="C4" s="101"/>
+      <c r="D4" s="101"/>
+      <c r="E4" s="102"/>
+      <c r="F4" s="100"/>
+      <c r="G4" s="101"/>
+      <c r="H4" s="101"/>
+      <c r="I4" s="101"/>
+      <c r="J4" s="101"/>
+      <c r="K4" s="101"/>
+      <c r="L4" s="101"/>
+      <c r="M4" s="101"/>
+      <c r="N4" s="101"/>
+      <c r="O4" s="102"/>
+      <c r="P4" s="103" t="s">
         <v>143</v>
       </c>
-      <c r="Q4" s="72"/>
+      <c r="Q4" s="104"/>
     </row>
     <row r="5" spans="1:17" ht="43.5" customHeight="1">
-      <c r="A5" s="125" t="s">
+      <c r="A5" s="63" t="s">
         <v>176</v>
       </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="54"/>
-      <c r="I5" s="54"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="54"/>
-      <c r="L5" s="54"/>
-      <c r="M5" s="54"/>
-      <c r="N5" s="54"/>
-      <c r="O5" s="54"/>
-      <c r="P5" s="54"/>
-      <c r="Q5" s="72"/>
-    </row>
-    <row r="6" spans="1:17">
-      <c r="A6" s="87" t="s">
+      <c r="B5" s="105"/>
+      <c r="C5" s="105"/>
+      <c r="D5" s="105"/>
+      <c r="E5" s="105"/>
+      <c r="F5" s="105"/>
+      <c r="G5" s="105"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="105"/>
+      <c r="K5" s="105"/>
+      <c r="L5" s="105"/>
+      <c r="M5" s="105"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="105"/>
+      <c r="P5" s="105"/>
+      <c r="Q5" s="104"/>
+    </row>
+    <row r="6" spans="1:17" ht="12.75">
+      <c r="A6" s="76" t="s">
         <v>161</v>
       </c>
-      <c r="B6" s="54"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
-      <c r="I6" s="54"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="54"/>
-      <c r="L6" s="54"/>
-      <c r="M6" s="54"/>
-      <c r="N6" s="54"/>
-      <c r="O6" s="54"/>
-      <c r="P6" s="54"/>
-      <c r="Q6" s="72"/>
+      <c r="B6" s="105"/>
+      <c r="C6" s="105"/>
+      <c r="D6" s="105"/>
+      <c r="E6" s="105"/>
+      <c r="F6" s="105"/>
+      <c r="G6" s="105"/>
+      <c r="H6" s="105"/>
+      <c r="I6" s="105"/>
+      <c r="J6" s="105"/>
+      <c r="K6" s="105"/>
+      <c r="L6" s="105"/>
+      <c r="M6" s="105"/>
+      <c r="N6" s="105"/>
+      <c r="O6" s="105"/>
+      <c r="P6" s="105"/>
+      <c r="Q6" s="104"/>
     </row>
     <row r="7" spans="1:17" ht="30" customHeight="1">
-      <c r="A7" s="109" t="s">
+      <c r="A7" s="53" t="s">
         <v>144</v>
       </c>
-      <c r="B7" s="110"/>
-      <c r="C7" s="111"/>
-      <c r="D7" s="126"/>
-      <c r="E7" s="113"/>
-      <c r="F7" s="113"/>
-      <c r="G7" s="113"/>
-      <c r="H7" s="113"/>
-      <c r="I7" s="114"/>
-      <c r="J7" s="115" t="s">
+      <c r="B7" s="54"/>
+      <c r="C7" s="55"/>
+      <c r="D7" s="83"/>
+      <c r="E7" s="106"/>
+      <c r="F7" s="106"/>
+      <c r="G7" s="106"/>
+      <c r="H7" s="106"/>
+      <c r="I7" s="107"/>
+      <c r="J7" s="47" t="s">
         <v>145</v>
       </c>
-      <c r="K7" s="116"/>
-      <c r="L7" s="115"/>
-      <c r="M7" s="117"/>
-      <c r="N7" s="117"/>
-      <c r="O7" s="117"/>
-      <c r="P7" s="117"/>
-      <c r="Q7" s="118"/>
+      <c r="K7" s="57"/>
+      <c r="L7" s="47"/>
+      <c r="M7" s="108"/>
+      <c r="N7" s="108"/>
+      <c r="O7" s="108"/>
+      <c r="P7" s="108"/>
+      <c r="Q7" s="57"/>
     </row>
     <row r="8" spans="1:17" ht="30" customHeight="1">
-      <c r="A8" s="109" t="s">
+      <c r="A8" s="53" t="s">
         <v>146</v>
       </c>
-      <c r="B8" s="110"/>
-      <c r="C8" s="111"/>
-      <c r="D8" s="112"/>
-      <c r="E8" s="113"/>
-      <c r="F8" s="113"/>
-      <c r="G8" s="113"/>
-      <c r="H8" s="113"/>
-      <c r="I8" s="114"/>
-      <c r="J8" s="115" t="s">
+      <c r="B8" s="54"/>
+      <c r="C8" s="55"/>
+      <c r="D8" s="56"/>
+      <c r="E8" s="106"/>
+      <c r="F8" s="106"/>
+      <c r="G8" s="106"/>
+      <c r="H8" s="106"/>
+      <c r="I8" s="107"/>
+      <c r="J8" s="47" t="s">
         <v>147</v>
       </c>
-      <c r="K8" s="116"/>
-      <c r="L8" s="115"/>
-      <c r="M8" s="117"/>
-      <c r="N8" s="117"/>
-      <c r="O8" s="117"/>
-      <c r="P8" s="117"/>
-      <c r="Q8" s="118"/>
+      <c r="K8" s="57"/>
+      <c r="L8" s="47"/>
+      <c r="M8" s="108"/>
+      <c r="N8" s="108"/>
+      <c r="O8" s="108"/>
+      <c r="P8" s="108"/>
+      <c r="Q8" s="57"/>
     </row>
     <row r="9" spans="1:17" ht="30" customHeight="1">
-      <c r="A9" s="109" t="s">
+      <c r="A9" s="53" t="s">
         <v>148</v>
       </c>
-      <c r="B9" s="110"/>
-      <c r="C9" s="111"/>
-      <c r="D9" s="112"/>
-      <c r="E9" s="113"/>
-      <c r="F9" s="113"/>
-      <c r="G9" s="113"/>
-      <c r="H9" s="113"/>
-      <c r="I9" s="114"/>
-      <c r="J9" s="115" t="s">
+      <c r="B9" s="54"/>
+      <c r="C9" s="55"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="106"/>
+      <c r="F9" s="106"/>
+      <c r="G9" s="106"/>
+      <c r="H9" s="106"/>
+      <c r="I9" s="107"/>
+      <c r="J9" s="47" t="s">
         <v>149</v>
       </c>
-      <c r="K9" s="116"/>
-      <c r="L9" s="115"/>
-      <c r="M9" s="117"/>
-      <c r="N9" s="117"/>
-      <c r="O9" s="117"/>
-      <c r="P9" s="117"/>
-      <c r="Q9" s="118"/>
+      <c r="K9" s="57"/>
+      <c r="L9" s="47"/>
+      <c r="M9" s="108"/>
+      <c r="N9" s="108"/>
+      <c r="O9" s="108"/>
+      <c r="P9" s="108"/>
+      <c r="Q9" s="57"/>
     </row>
     <row r="10" spans="1:17" ht="30" customHeight="1">
-      <c r="A10" s="109" t="s">
+      <c r="A10" s="53" t="s">
         <v>150</v>
       </c>
-      <c r="B10" s="110"/>
-      <c r="C10" s="111"/>
-      <c r="D10" s="112"/>
-      <c r="E10" s="113"/>
-      <c r="F10" s="113"/>
-      <c r="G10" s="113"/>
-      <c r="H10" s="113"/>
-      <c r="I10" s="114"/>
-      <c r="J10" s="115" t="s">
+      <c r="B10" s="54"/>
+      <c r="C10" s="55"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="106"/>
+      <c r="F10" s="106"/>
+      <c r="G10" s="106"/>
+      <c r="H10" s="106"/>
+      <c r="I10" s="107"/>
+      <c r="J10" s="47" t="s">
         <v>151</v>
       </c>
-      <c r="K10" s="116"/>
-      <c r="L10" s="115"/>
-      <c r="M10" s="117"/>
-      <c r="N10" s="117"/>
-      <c r="O10" s="117"/>
-      <c r="P10" s="117"/>
-      <c r="Q10" s="118"/>
+      <c r="K10" s="57"/>
+      <c r="L10" s="47"/>
+      <c r="M10" s="108"/>
+      <c r="N10" s="108"/>
+      <c r="O10" s="108"/>
+      <c r="P10" s="108"/>
+      <c r="Q10" s="57"/>
     </row>
     <row r="11" spans="1:17" ht="30" customHeight="1">
-      <c r="A11" s="109" t="s">
+      <c r="A11" s="53" t="s">
         <v>160</v>
       </c>
-      <c r="B11" s="110"/>
-      <c r="C11" s="111"/>
-      <c r="D11" s="112"/>
-      <c r="E11" s="113"/>
-      <c r="F11" s="113"/>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113"/>
-      <c r="I11" s="114"/>
-      <c r="J11" s="115" t="s">
+      <c r="B11" s="54"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="56"/>
+      <c r="E11" s="106"/>
+      <c r="F11" s="106"/>
+      <c r="G11" s="106"/>
+      <c r="H11" s="106"/>
+      <c r="I11" s="107"/>
+      <c r="J11" s="47" t="s">
         <v>152</v>
       </c>
-      <c r="K11" s="116"/>
-      <c r="L11" s="115"/>
-      <c r="M11" s="117"/>
-      <c r="N11" s="117"/>
-      <c r="O11" s="117"/>
-      <c r="P11" s="117"/>
-      <c r="Q11" s="118"/>
+      <c r="K11" s="57"/>
+      <c r="L11" s="47"/>
+      <c r="M11" s="108"/>
+      <c r="N11" s="108"/>
+      <c r="O11" s="108"/>
+      <c r="P11" s="108"/>
+      <c r="Q11" s="57"/>
     </row>
     <row r="12" spans="1:17" ht="30" customHeight="1">
-      <c r="A12" s="119" t="s">
+      <c r="A12" s="64" t="s">
         <v>153</v>
       </c>
-      <c r="B12" s="110"/>
-      <c r="C12" s="110"/>
-      <c r="D12" s="120"/>
-      <c r="E12" s="113"/>
-      <c r="F12" s="113"/>
-      <c r="G12" s="113"/>
-      <c r="H12" s="113"/>
-      <c r="I12" s="114"/>
-      <c r="J12" s="115" t="s">
+      <c r="B12" s="54"/>
+      <c r="C12" s="54"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="106"/>
+      <c r="F12" s="106"/>
+      <c r="G12" s="106"/>
+      <c r="H12" s="106"/>
+      <c r="I12" s="107"/>
+      <c r="J12" s="47" t="s">
         <v>154</v>
       </c>
-      <c r="K12" s="116"/>
-      <c r="L12" s="115"/>
-      <c r="M12" s="117"/>
-      <c r="N12" s="117"/>
-      <c r="O12" s="117"/>
-      <c r="P12" s="117"/>
-      <c r="Q12" s="118"/>
+      <c r="K12" s="57"/>
+      <c r="L12" s="47"/>
+      <c r="M12" s="108"/>
+      <c r="N12" s="108"/>
+      <c r="O12" s="108"/>
+      <c r="P12" s="108"/>
+      <c r="Q12" s="57"/>
     </row>
     <row r="13" spans="1:17" ht="30" customHeight="1">
-      <c r="A13" s="109" t="s">
+      <c r="A13" s="53" t="s">
         <v>158</v>
       </c>
-      <c r="B13" s="110"/>
-      <c r="C13" s="111"/>
-      <c r="D13" s="112"/>
-      <c r="E13" s="113"/>
-      <c r="F13" s="113"/>
-      <c r="G13" s="113"/>
-      <c r="H13" s="113"/>
-      <c r="I13" s="114"/>
-      <c r="J13" s="115" t="s">
+      <c r="B13" s="54"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="56"/>
+      <c r="E13" s="106"/>
+      <c r="F13" s="106"/>
+      <c r="G13" s="106"/>
+      <c r="H13" s="106"/>
+      <c r="I13" s="107"/>
+      <c r="J13" s="47" t="s">
         <v>155</v>
       </c>
-      <c r="K13" s="116"/>
-      <c r="L13" s="115"/>
-      <c r="M13" s="117"/>
-      <c r="N13" s="117"/>
-      <c r="O13" s="117"/>
-      <c r="P13" s="117"/>
-      <c r="Q13" s="118"/>
-    </row>
-    <row r="14" spans="1:17">
-      <c r="A14" s="87" t="s">
+      <c r="K13" s="57"/>
+      <c r="L13" s="47"/>
+      <c r="M13" s="108"/>
+      <c r="N13" s="108"/>
+      <c r="O13" s="108"/>
+      <c r="P13" s="108"/>
+      <c r="Q13" s="57"/>
+    </row>
+    <row r="14" spans="1:17" ht="12.75">
+      <c r="A14" s="76" t="s">
         <v>177</v>
       </c>
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="54"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
-      <c r="J14" s="54"/>
-      <c r="K14" s="54"/>
-      <c r="L14" s="54"/>
-      <c r="M14" s="54"/>
-      <c r="N14" s="54"/>
-      <c r="O14" s="54"/>
-      <c r="P14" s="54"/>
-      <c r="Q14" s="72"/>
+      <c r="B14" s="105"/>
+      <c r="C14" s="105"/>
+      <c r="D14" s="105"/>
+      <c r="E14" s="105"/>
+      <c r="F14" s="105"/>
+      <c r="G14" s="105"/>
+      <c r="H14" s="105"/>
+      <c r="I14" s="105"/>
+      <c r="J14" s="105"/>
+      <c r="K14" s="105"/>
+      <c r="L14" s="105"/>
+      <c r="M14" s="105"/>
+      <c r="N14" s="105"/>
+      <c r="O14" s="105"/>
+      <c r="P14" s="105"/>
+      <c r="Q14" s="104"/>
     </row>
     <row r="15" spans="1:17" ht="39.75" customHeight="1">
-      <c r="A15" s="127" t="s">
+      <c r="A15" s="50" t="s">
         <v>178</v>
       </c>
-      <c r="B15" s="128"/>
-      <c r="C15" s="128"/>
-      <c r="D15" s="128"/>
-      <c r="E15" s="128"/>
-      <c r="F15" s="128"/>
-      <c r="G15" s="128"/>
-      <c r="H15" s="128"/>
-      <c r="I15" s="128"/>
-      <c r="J15" s="128"/>
-      <c r="K15" s="128"/>
-      <c r="L15" s="128"/>
-      <c r="M15" s="128"/>
-      <c r="N15" s="128"/>
-      <c r="O15" s="128"/>
-      <c r="P15" s="128"/>
-      <c r="Q15" s="129"/>
+      <c r="B15" s="109"/>
+      <c r="C15" s="109"/>
+      <c r="D15" s="109"/>
+      <c r="E15" s="109"/>
+      <c r="F15" s="109"/>
+      <c r="G15" s="109"/>
+      <c r="H15" s="109"/>
+      <c r="I15" s="109"/>
+      <c r="J15" s="109"/>
+      <c r="K15" s="109"/>
+      <c r="L15" s="109"/>
+      <c r="M15" s="109"/>
+      <c r="N15" s="109"/>
+      <c r="O15" s="109"/>
+      <c r="P15" s="109"/>
+      <c r="Q15" s="110"/>
     </row>
     <row r="16" spans="1:17" ht="15">
-      <c r="A16" s="96" t="s">
+      <c r="A16" s="51" t="s">
         <v>179</v>
       </c>
-      <c r="B16" s="74"/>
-      <c r="C16" s="74"/>
-      <c r="D16" s="74"/>
-      <c r="E16" s="74"/>
-      <c r="F16" s="74"/>
-      <c r="G16" s="74"/>
-      <c r="H16" s="74"/>
-      <c r="I16" s="74"/>
-      <c r="J16" s="75"/>
-      <c r="K16" s="96" t="s">
+      <c r="B16" s="111"/>
+      <c r="C16" s="111"/>
+      <c r="D16" s="111"/>
+      <c r="E16" s="111"/>
+      <c r="F16" s="111"/>
+      <c r="G16" s="111"/>
+      <c r="H16" s="111"/>
+      <c r="I16" s="111"/>
+      <c r="J16" s="112"/>
+      <c r="K16" s="51" t="s">
         <v>162</v>
       </c>
-      <c r="L16" s="74"/>
-      <c r="M16" s="74"/>
-      <c r="N16" s="75"/>
-      <c r="O16" s="130" t="s">
+      <c r="L16" s="111"/>
+      <c r="M16" s="111"/>
+      <c r="N16" s="112"/>
+      <c r="O16" s="52" t="s">
         <v>163</v>
       </c>
-      <c r="P16" s="60"/>
-      <c r="Q16" s="61"/>
+      <c r="P16" s="113"/>
+      <c r="Q16" s="114"/>
     </row>
     <row r="17" spans="1:17">
-      <c r="A17" s="96" t="s">
+      <c r="A17" s="51" t="s">
         <v>164</v>
       </c>
-      <c r="B17" s="75"/>
-      <c r="C17" s="96" t="s">
+      <c r="B17" s="112"/>
+      <c r="C17" s="51" t="s">
         <v>165</v>
       </c>
-      <c r="D17" s="74"/>
-      <c r="E17" s="74"/>
-      <c r="F17" s="74"/>
-      <c r="G17" s="75"/>
-      <c r="H17" s="96" t="s">
+      <c r="D17" s="111"/>
+      <c r="E17" s="111"/>
+      <c r="F17" s="111"/>
+      <c r="G17" s="112"/>
+      <c r="H17" s="51" t="s">
         <v>166</v>
       </c>
-      <c r="I17" s="74"/>
-      <c r="J17" s="75"/>
-      <c r="K17" s="46" t="s">
+      <c r="I17" s="111"/>
+      <c r="J17" s="112"/>
+      <c r="K17" s="40" t="s">
         <v>167</v>
       </c>
-      <c r="L17" s="96" t="s">
+      <c r="L17" s="51" t="s">
         <v>168</v>
       </c>
-      <c r="M17" s="74"/>
-      <c r="N17" s="75"/>
-      <c r="O17" s="65"/>
-      <c r="P17" s="66"/>
-      <c r="Q17" s="67"/>
+      <c r="M17" s="111"/>
+      <c r="N17" s="112"/>
+      <c r="O17" s="115"/>
+      <c r="P17" s="116"/>
+      <c r="Q17" s="117"/>
     </row>
     <row r="18" spans="1:17" ht="15">
-      <c r="A18" s="95"/>
-      <c r="B18" s="74"/>
-      <c r="C18" s="101"/>
-      <c r="D18" s="74"/>
-      <c r="E18" s="74"/>
-      <c r="F18" s="74"/>
-      <c r="G18" s="75"/>
-      <c r="H18" s="97"/>
-      <c r="I18" s="74"/>
-      <c r="J18" s="75"/>
-      <c r="K18" s="47"/>
-      <c r="L18" s="121"/>
-      <c r="M18" s="74"/>
-      <c r="N18" s="75"/>
-      <c r="O18" s="95"/>
-      <c r="P18" s="74"/>
-      <c r="Q18" s="75"/>
+      <c r="A18" s="58"/>
+      <c r="B18" s="111"/>
+      <c r="C18" s="59"/>
+      <c r="D18" s="111"/>
+      <c r="E18" s="111"/>
+      <c r="F18" s="111"/>
+      <c r="G18" s="112"/>
+      <c r="H18" s="60"/>
+      <c r="I18" s="111"/>
+      <c r="J18" s="112"/>
+      <c r="K18" s="41"/>
+      <c r="L18" s="61"/>
+      <c r="M18" s="111"/>
+      <c r="N18" s="112"/>
+      <c r="O18" s="58"/>
+      <c r="P18" s="111"/>
+      <c r="Q18" s="112"/>
     </row>
     <row r="19" spans="1:17" ht="30" customHeight="1">
-      <c r="A19" s="96" t="s">
+      <c r="A19" s="51" t="s">
         <v>180</v>
       </c>
-      <c r="B19" s="74"/>
-      <c r="C19" s="95"/>
-      <c r="D19" s="75"/>
-      <c r="E19" s="104" t="s">
+      <c r="B19" s="111"/>
+      <c r="C19" s="58"/>
+      <c r="D19" s="112"/>
+      <c r="E19" s="66" t="s">
         <v>181</v>
       </c>
-      <c r="F19" s="74"/>
-      <c r="G19" s="95"/>
-      <c r="H19" s="74"/>
-      <c r="I19" s="75"/>
-      <c r="J19" s="104" t="s">
+      <c r="F19" s="111"/>
+      <c r="G19" s="58"/>
+      <c r="H19" s="111"/>
+      <c r="I19" s="112"/>
+      <c r="J19" s="66" t="s">
         <v>182</v>
       </c>
-      <c r="K19" s="74"/>
-      <c r="L19" s="74"/>
-      <c r="M19" s="95"/>
-      <c r="N19" s="75"/>
-      <c r="O19" s="102" t="s">
+      <c r="K19" s="111"/>
+      <c r="L19" s="111"/>
+      <c r="M19" s="58"/>
+      <c r="N19" s="112"/>
+      <c r="O19" s="67" t="s">
         <v>183</v>
       </c>
-      <c r="P19" s="74"/>
-      <c r="Q19" s="49"/>
+      <c r="P19" s="111"/>
+      <c r="Q19" s="43"/>
     </row>
     <row r="20" spans="1:17" ht="34.5" customHeight="1">
-      <c r="A20" s="96" t="s">
+      <c r="A20" s="51" t="s">
         <v>184</v>
       </c>
-      <c r="B20" s="74"/>
-      <c r="C20" s="74"/>
-      <c r="D20" s="75"/>
-      <c r="E20" s="107"/>
-      <c r="F20" s="74"/>
-      <c r="G20" s="75"/>
-      <c r="H20" s="108" t="s">
+      <c r="B20" s="111"/>
+      <c r="C20" s="111"/>
+      <c r="D20" s="112"/>
+      <c r="E20" s="73"/>
+      <c r="F20" s="111"/>
+      <c r="G20" s="112"/>
+      <c r="H20" s="74" t="s">
         <v>185</v>
       </c>
-      <c r="I20" s="66"/>
-      <c r="J20" s="66"/>
-      <c r="K20" s="67"/>
-      <c r="L20" s="107"/>
-      <c r="M20" s="75"/>
-      <c r="N20" s="50" t="s">
+      <c r="I20" s="116"/>
+      <c r="J20" s="116"/>
+      <c r="K20" s="117"/>
+      <c r="L20" s="73"/>
+      <c r="M20" s="112"/>
+      <c r="N20" s="44" t="s">
         <v>169</v>
       </c>
-      <c r="O20" s="95"/>
-      <c r="P20" s="74"/>
-      <c r="Q20" s="75"/>
+      <c r="O20" s="58"/>
+      <c r="P20" s="111"/>
+      <c r="Q20" s="112"/>
     </row>
     <row r="21" spans="1:17" ht="34.5" customHeight="1">
-      <c r="A21" s="96" t="s">
+      <c r="A21" s="51" t="s">
         <v>186</v>
       </c>
-      <c r="B21" s="74"/>
-      <c r="C21" s="97"/>
-      <c r="D21" s="74"/>
-      <c r="E21" s="74"/>
-      <c r="F21" s="75"/>
-      <c r="G21" s="96" t="s">
+      <c r="B21" s="111"/>
+      <c r="C21" s="60"/>
+      <c r="D21" s="111"/>
+      <c r="E21" s="111"/>
+      <c r="F21" s="112"/>
+      <c r="G21" s="51" t="s">
         <v>187</v>
       </c>
-      <c r="H21" s="75"/>
-      <c r="I21" s="85"/>
-      <c r="J21" s="74"/>
-      <c r="K21" s="75"/>
-      <c r="L21" s="48" t="s">
+      <c r="H21" s="112"/>
+      <c r="I21" s="59"/>
+      <c r="J21" s="111"/>
+      <c r="K21" s="112"/>
+      <c r="L21" s="42" t="s">
         <v>188</v>
       </c>
-      <c r="M21" s="98"/>
-      <c r="N21" s="75"/>
-      <c r="O21" s="102" t="s">
+      <c r="M21" s="72"/>
+      <c r="N21" s="112"/>
+      <c r="O21" s="67" t="s">
         <v>189</v>
       </c>
-      <c r="P21" s="74"/>
-      <c r="Q21" s="49"/>
+      <c r="P21" s="111"/>
+      <c r="Q21" s="43"/>
     </row>
     <row r="22" spans="1:17" ht="39" customHeight="1">
-      <c r="A22" s="96" t="s">
+      <c r="A22" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="B22" s="74"/>
-      <c r="C22" s="74"/>
-      <c r="D22" s="74"/>
-      <c r="E22" s="75"/>
-      <c r="F22" s="100"/>
-      <c r="G22" s="74"/>
-      <c r="H22" s="74"/>
-      <c r="I22" s="74"/>
-      <c r="J22" s="96" t="s">
+      <c r="B22" s="111"/>
+      <c r="C22" s="111"/>
+      <c r="D22" s="111"/>
+      <c r="E22" s="112"/>
+      <c r="F22" s="73"/>
+      <c r="G22" s="111"/>
+      <c r="H22" s="111"/>
+      <c r="I22" s="111"/>
+      <c r="J22" s="51" t="s">
         <v>191</v>
       </c>
-      <c r="K22" s="75"/>
-      <c r="L22" s="101"/>
-      <c r="M22" s="74"/>
-      <c r="N22" s="75"/>
-      <c r="O22" s="102" t="s">
+      <c r="K22" s="112"/>
+      <c r="L22" s="59"/>
+      <c r="M22" s="111"/>
+      <c r="N22" s="112"/>
+      <c r="O22" s="67" t="s">
         <v>192</v>
       </c>
-      <c r="P22" s="74"/>
-      <c r="Q22" s="49"/>
-    </row>
-    <row r="23" spans="1:17">
-      <c r="A23" s="103" t="s">
+      <c r="P22" s="111"/>
+      <c r="Q22" s="43"/>
+    </row>
+    <row r="23" spans="1:17" ht="15">
+      <c r="A23" s="118" t="s">
         <v>193</v>
       </c>
-      <c r="B23" s="74"/>
-      <c r="C23" s="74"/>
-      <c r="D23" s="74"/>
-      <c r="E23" s="74"/>
-      <c r="F23" s="74"/>
-      <c r="G23" s="74"/>
-      <c r="H23" s="74"/>
-      <c r="I23" s="74"/>
-      <c r="J23" s="74"/>
-      <c r="K23" s="74"/>
-      <c r="L23" s="74"/>
-      <c r="M23" s="74"/>
-      <c r="N23" s="74"/>
-      <c r="O23" s="74"/>
-      <c r="P23" s="74"/>
-      <c r="Q23" s="75"/>
+      <c r="B23" s="111"/>
+      <c r="C23" s="111"/>
+      <c r="D23" s="111"/>
+      <c r="E23" s="111"/>
+      <c r="F23" s="111"/>
+      <c r="G23" s="111"/>
+      <c r="H23" s="111"/>
+      <c r="I23" s="111"/>
+      <c r="J23" s="111"/>
+      <c r="K23" s="111"/>
+      <c r="L23" s="111"/>
+      <c r="M23" s="111"/>
+      <c r="N23" s="111"/>
+      <c r="O23" s="111"/>
+      <c r="P23" s="111"/>
+      <c r="Q23" s="112"/>
     </row>
     <row r="24" spans="1:17" ht="15">
-      <c r="A24" s="99" t="s">
+      <c r="A24" s="75" t="s">
         <v>194</v>
       </c>
-      <c r="B24" s="74"/>
-      <c r="C24" s="74"/>
-      <c r="D24" s="74"/>
-      <c r="E24" s="74"/>
-      <c r="F24" s="75"/>
-      <c r="G24" s="98"/>
-      <c r="H24" s="74"/>
-      <c r="I24" s="74"/>
-      <c r="J24" s="74"/>
-      <c r="K24" s="75"/>
-      <c r="L24" s="99" t="s">
+      <c r="B24" s="111"/>
+      <c r="C24" s="111"/>
+      <c r="D24" s="111"/>
+      <c r="E24" s="111"/>
+      <c r="F24" s="112"/>
+      <c r="G24" s="72"/>
+      <c r="H24" s="111"/>
+      <c r="I24" s="111"/>
+      <c r="J24" s="111"/>
+      <c r="K24" s="112"/>
+      <c r="L24" s="75" t="s">
         <v>195</v>
       </c>
-      <c r="M24" s="75"/>
-      <c r="N24" s="95"/>
-      <c r="O24" s="74"/>
-      <c r="P24" s="74"/>
-      <c r="Q24" s="75"/>
-    </row>
-    <row r="25" spans="1:17">
-      <c r="A25" s="93" t="s">
+      <c r="M24" s="112"/>
+      <c r="N24" s="58"/>
+      <c r="O24" s="111"/>
+      <c r="P24" s="111"/>
+      <c r="Q24" s="112"/>
+    </row>
+    <row r="25" spans="1:17" ht="12.75">
+      <c r="A25" s="119" t="s">
         <v>196</v>
       </c>
-      <c r="B25" s="82"/>
-      <c r="C25" s="82"/>
-      <c r="D25" s="82"/>
-      <c r="E25" s="82"/>
-      <c r="F25" s="82"/>
-      <c r="G25" s="82"/>
-      <c r="H25" s="82"/>
-      <c r="I25" s="82"/>
-      <c r="J25" s="82"/>
-      <c r="K25" s="82"/>
-      <c r="L25" s="82"/>
-      <c r="M25" s="82"/>
-      <c r="N25" s="82"/>
-      <c r="O25" s="82"/>
-      <c r="P25" s="82"/>
-      <c r="Q25" s="83"/>
-    </row>
-    <row r="26" spans="1:17" ht="134.25" customHeight="1">
-      <c r="A26" s="94"/>
-      <c r="B26" s="66"/>
-      <c r="C26" s="66"/>
-      <c r="D26" s="66"/>
-      <c r="E26" s="66"/>
-      <c r="F26" s="66"/>
-      <c r="G26" s="66"/>
-      <c r="H26" s="66"/>
-      <c r="I26" s="66"/>
-      <c r="J26" s="66"/>
-      <c r="K26" s="66"/>
-      <c r="L26" s="66"/>
-      <c r="M26" s="66"/>
-      <c r="N26" s="66"/>
-      <c r="O26" s="66"/>
-      <c r="P26" s="66"/>
-      <c r="Q26" s="67"/>
-    </row>
-    <row r="27" spans="1:17">
-      <c r="A27" s="93" t="s">
+      <c r="B25" s="101"/>
+      <c r="C25" s="101"/>
+      <c r="D25" s="101"/>
+      <c r="E25" s="101"/>
+      <c r="F25" s="101"/>
+      <c r="G25" s="101"/>
+      <c r="H25" s="101"/>
+      <c r="I25" s="101"/>
+      <c r="J25" s="101"/>
+      <c r="K25" s="101"/>
+      <c r="L25" s="101"/>
+      <c r="M25" s="101"/>
+      <c r="N25" s="101"/>
+      <c r="O25" s="101"/>
+      <c r="P25" s="101"/>
+      <c r="Q25" s="102"/>
+    </row>
+    <row r="26" spans="1:17" ht="225" customHeight="1">
+      <c r="A26" s="120"/>
+      <c r="B26" s="116"/>
+      <c r="C26" s="116"/>
+      <c r="D26" s="116"/>
+      <c r="E26" s="116"/>
+      <c r="F26" s="116"/>
+      <c r="G26" s="116"/>
+      <c r="H26" s="116"/>
+      <c r="I26" s="116"/>
+      <c r="J26" s="116"/>
+      <c r="K26" s="116"/>
+      <c r="L26" s="116"/>
+      <c r="M26" s="116"/>
+      <c r="N26" s="116"/>
+      <c r="O26" s="116"/>
+      <c r="P26" s="116"/>
+      <c r="Q26" s="117"/>
+    </row>
+    <row r="27" spans="1:17" ht="12.75">
+      <c r="A27" s="119" t="s">
         <v>197</v>
       </c>
-      <c r="B27" s="82"/>
-      <c r="C27" s="82"/>
-      <c r="D27" s="82"/>
-      <c r="E27" s="82"/>
-      <c r="F27" s="82"/>
-      <c r="G27" s="82"/>
-      <c r="H27" s="82"/>
-      <c r="I27" s="82"/>
-      <c r="J27" s="82"/>
-      <c r="K27" s="82"/>
-      <c r="L27" s="82"/>
-      <c r="M27" s="82"/>
-      <c r="N27" s="82"/>
-      <c r="O27" s="82"/>
-      <c r="P27" s="82"/>
-      <c r="Q27" s="83"/>
+      <c r="B27" s="101"/>
+      <c r="C27" s="101"/>
+      <c r="D27" s="101"/>
+      <c r="E27" s="101"/>
+      <c r="F27" s="101"/>
+      <c r="G27" s="101"/>
+      <c r="H27" s="101"/>
+      <c r="I27" s="101"/>
+      <c r="J27" s="101"/>
+      <c r="K27" s="101"/>
+      <c r="L27" s="101"/>
+      <c r="M27" s="101"/>
+      <c r="N27" s="101"/>
+      <c r="O27" s="101"/>
+      <c r="P27" s="101"/>
+      <c r="Q27" s="102"/>
     </row>
     <row r="28" spans="1:17" ht="12.75">
-      <c r="A28" s="71" t="s">
+      <c r="A28" s="76" t="s">
         <v>198</v>
       </c>
-      <c r="B28" s="54"/>
-      <c r="C28" s="54"/>
-      <c r="D28" s="54"/>
-      <c r="E28" s="54"/>
-      <c r="F28" s="54"/>
-      <c r="G28" s="54"/>
-      <c r="H28" s="54"/>
-      <c r="I28" s="54"/>
-      <c r="J28" s="54"/>
-      <c r="K28" s="54"/>
-      <c r="L28" s="54"/>
-      <c r="M28" s="54"/>
-      <c r="N28" s="54"/>
-      <c r="O28" s="54"/>
-      <c r="P28" s="54"/>
-      <c r="Q28" s="72"/>
+      <c r="B28" s="105"/>
+      <c r="C28" s="105"/>
+      <c r="D28" s="105"/>
+      <c r="E28" s="105"/>
+      <c r="F28" s="105"/>
+      <c r="G28" s="105"/>
+      <c r="H28" s="105"/>
+      <c r="I28" s="105"/>
+      <c r="J28" s="105"/>
+      <c r="K28" s="105"/>
+      <c r="L28" s="105"/>
+      <c r="M28" s="105"/>
+      <c r="N28" s="105"/>
+      <c r="O28" s="105"/>
+      <c r="P28" s="105"/>
+      <c r="Q28" s="104"/>
     </row>
     <row r="29" spans="1:17" ht="36.75" customHeight="1">
-      <c r="A29" s="53" t="s">
+      <c r="A29" s="77" t="s">
         <v>199</v>
       </c>
-      <c r="B29" s="54"/>
-      <c r="C29" s="54"/>
-      <c r="D29" s="54"/>
-      <c r="E29" s="54"/>
-      <c r="F29" s="54"/>
-      <c r="G29" s="53" t="s">
+      <c r="B29" s="105"/>
+      <c r="C29" s="105"/>
+      <c r="D29" s="105"/>
+      <c r="E29" s="105"/>
+      <c r="F29" s="105"/>
+      <c r="G29" s="77" t="s">
         <v>200</v>
       </c>
-      <c r="H29" s="54"/>
-      <c r="I29" s="54"/>
-      <c r="J29" s="54"/>
-      <c r="K29" s="54"/>
-      <c r="L29" s="53" t="s">
+      <c r="H29" s="105"/>
+      <c r="I29" s="105"/>
+      <c r="J29" s="105"/>
+      <c r="K29" s="105"/>
+      <c r="L29" s="77" t="s">
         <v>201</v>
       </c>
-      <c r="M29" s="54"/>
-      <c r="N29" s="54"/>
-      <c r="O29" s="54"/>
-      <c r="P29" s="54"/>
-      <c r="Q29" s="72"/>
+      <c r="M29" s="105"/>
+      <c r="N29" s="105"/>
+      <c r="O29" s="105"/>
+      <c r="P29" s="105"/>
+      <c r="Q29" s="104"/>
     </row>
     <row r="30" spans="1:17" ht="36" customHeight="1">
-      <c r="A30" s="89" t="s">
+      <c r="A30" s="78" t="s">
         <v>202</v>
       </c>
-      <c r="B30" s="56"/>
-      <c r="C30" s="56"/>
-      <c r="D30" s="56"/>
-      <c r="E30" s="56"/>
-      <c r="F30" s="56"/>
-      <c r="G30" s="59"/>
-      <c r="H30" s="60"/>
-      <c r="I30" s="60"/>
-      <c r="J30" s="60"/>
-      <c r="K30" s="61"/>
-      <c r="L30" s="105"/>
-      <c r="M30" s="74"/>
-      <c r="N30" s="74"/>
-      <c r="O30" s="74"/>
-      <c r="P30" s="74"/>
-      <c r="Q30" s="75"/>
-    </row>
-    <row r="31" spans="1:17">
-      <c r="A31" s="57"/>
-      <c r="B31" s="58"/>
-      <c r="C31" s="58"/>
-      <c r="D31" s="58"/>
-      <c r="E31" s="58"/>
-      <c r="F31" s="58"/>
-      <c r="G31" s="65"/>
-      <c r="H31" s="66"/>
-      <c r="I31" s="66"/>
-      <c r="J31" s="66"/>
-      <c r="K31" s="67"/>
-      <c r="L31" s="51" t="s">
+      <c r="B30" s="89"/>
+      <c r="C30" s="89"/>
+      <c r="D30" s="89"/>
+      <c r="E30" s="89"/>
+      <c r="F30" s="89"/>
+      <c r="G30" s="121"/>
+      <c r="H30" s="113"/>
+      <c r="I30" s="113"/>
+      <c r="J30" s="113"/>
+      <c r="K30" s="114"/>
+      <c r="L30" s="70"/>
+      <c r="M30" s="111"/>
+      <c r="N30" s="111"/>
+      <c r="O30" s="111"/>
+      <c r="P30" s="111"/>
+      <c r="Q30" s="112"/>
+    </row>
+    <row r="31" spans="1:17" ht="45" customHeight="1">
+      <c r="A31" s="94"/>
+      <c r="B31" s="95"/>
+      <c r="C31" s="95"/>
+      <c r="D31" s="95"/>
+      <c r="E31" s="95"/>
+      <c r="F31" s="95"/>
+      <c r="G31" s="115"/>
+      <c r="H31" s="116"/>
+      <c r="I31" s="116"/>
+      <c r="J31" s="116"/>
+      <c r="K31" s="117"/>
+      <c r="L31" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M31" s="77"/>
-      <c r="N31" s="66"/>
-      <c r="O31" s="66"/>
-      <c r="P31" s="66"/>
-      <c r="Q31" s="67"/>
+      <c r="M31" s="69"/>
+      <c r="N31" s="116"/>
+      <c r="O31" s="116"/>
+      <c r="P31" s="116"/>
+      <c r="Q31" s="117"/>
     </row>
     <row r="32" spans="1:17" ht="15">
-      <c r="A32" s="89" t="s">
+      <c r="A32" s="78" t="s">
         <v>203</v>
       </c>
-      <c r="B32" s="56"/>
-      <c r="C32" s="56"/>
-      <c r="D32" s="56"/>
-      <c r="E32" s="56"/>
-      <c r="F32" s="56"/>
-      <c r="G32" s="59"/>
-      <c r="H32" s="60"/>
-      <c r="I32" s="60"/>
-      <c r="J32" s="60"/>
-      <c r="K32" s="61"/>
-      <c r="L32" s="106"/>
-      <c r="M32" s="66"/>
-      <c r="N32" s="66"/>
-      <c r="O32" s="66"/>
-      <c r="P32" s="66"/>
-      <c r="Q32" s="67"/>
-    </row>
-    <row r="33" spans="1:17">
-      <c r="A33" s="57"/>
-      <c r="B33" s="58"/>
-      <c r="C33" s="58"/>
-      <c r="D33" s="58"/>
-      <c r="E33" s="58"/>
-      <c r="F33" s="58"/>
-      <c r="G33" s="65"/>
-      <c r="H33" s="66"/>
-      <c r="I33" s="66"/>
-      <c r="J33" s="66"/>
-      <c r="K33" s="67"/>
-      <c r="L33" s="51" t="s">
+      <c r="B32" s="89"/>
+      <c r="C32" s="89"/>
+      <c r="D32" s="89"/>
+      <c r="E32" s="89"/>
+      <c r="F32" s="89"/>
+      <c r="G32" s="121"/>
+      <c r="H32" s="113"/>
+      <c r="I32" s="113"/>
+      <c r="J32" s="113"/>
+      <c r="K32" s="114"/>
+      <c r="L32" s="71"/>
+      <c r="M32" s="116"/>
+      <c r="N32" s="116"/>
+      <c r="O32" s="116"/>
+      <c r="P32" s="116"/>
+      <c r="Q32" s="117"/>
+    </row>
+    <row r="33" spans="1:17" ht="45" customHeight="1">
+      <c r="A33" s="94"/>
+      <c r="B33" s="95"/>
+      <c r="C33" s="95"/>
+      <c r="D33" s="95"/>
+      <c r="E33" s="95"/>
+      <c r="F33" s="95"/>
+      <c r="G33" s="115"/>
+      <c r="H33" s="116"/>
+      <c r="I33" s="116"/>
+      <c r="J33" s="116"/>
+      <c r="K33" s="117"/>
+      <c r="L33" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M33" s="77"/>
-      <c r="N33" s="66"/>
-      <c r="O33" s="66"/>
-      <c r="P33" s="66"/>
-      <c r="Q33" s="67"/>
+      <c r="M33" s="69"/>
+      <c r="N33" s="116"/>
+      <c r="O33" s="116"/>
+      <c r="P33" s="116"/>
+      <c r="Q33" s="117"/>
     </row>
     <row r="34" spans="1:17" ht="15">
-      <c r="A34" s="55" t="s">
+      <c r="A34" s="79" t="s">
         <v>204</v>
       </c>
-      <c r="B34" s="56"/>
-      <c r="C34" s="56"/>
-      <c r="D34" s="56"/>
-      <c r="E34" s="56"/>
-      <c r="F34" s="56"/>
-      <c r="G34" s="59"/>
-      <c r="H34" s="60"/>
-      <c r="I34" s="60"/>
-      <c r="J34" s="60"/>
-      <c r="K34" s="61"/>
-      <c r="L34" s="76"/>
-      <c r="M34" s="74"/>
-      <c r="N34" s="74"/>
-      <c r="O34" s="74"/>
-      <c r="P34" s="74"/>
-      <c r="Q34" s="75"/>
+      <c r="B34" s="89"/>
+      <c r="C34" s="89"/>
+      <c r="D34" s="89"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="89"/>
+      <c r="G34" s="121"/>
+      <c r="H34" s="113"/>
+      <c r="I34" s="113"/>
+      <c r="J34" s="113"/>
+      <c r="K34" s="114"/>
+      <c r="L34" s="68"/>
+      <c r="M34" s="111"/>
+      <c r="N34" s="111"/>
+      <c r="O34" s="111"/>
+      <c r="P34" s="111"/>
+      <c r="Q34" s="112"/>
     </row>
     <row r="35" spans="1:17" ht="15">
-      <c r="A35" s="57"/>
-      <c r="B35" s="58"/>
-      <c r="C35" s="58"/>
-      <c r="D35" s="58"/>
-      <c r="E35" s="58"/>
-      <c r="F35" s="58"/>
-      <c r="G35" s="62"/>
-      <c r="H35" s="63"/>
-      <c r="I35" s="63"/>
-      <c r="J35" s="63"/>
-      <c r="K35" s="64"/>
-      <c r="L35" s="76"/>
-      <c r="M35" s="74"/>
-      <c r="N35" s="74"/>
-      <c r="O35" s="74"/>
-      <c r="P35" s="74"/>
-      <c r="Q35" s="75"/>
+      <c r="A35" s="94"/>
+      <c r="B35" s="95"/>
+      <c r="C35" s="95"/>
+      <c r="D35" s="95"/>
+      <c r="E35" s="95"/>
+      <c r="F35" s="95"/>
+      <c r="G35" s="122"/>
+      <c r="H35" s="123"/>
+      <c r="I35" s="123"/>
+      <c r="J35" s="123"/>
+      <c r="K35" s="124"/>
+      <c r="L35" s="68"/>
+      <c r="M35" s="111"/>
+      <c r="N35" s="111"/>
+      <c r="O35" s="111"/>
+      <c r="P35" s="111"/>
+      <c r="Q35" s="112"/>
     </row>
     <row r="36" spans="1:17" ht="15">
-      <c r="A36" s="57"/>
-      <c r="B36" s="58"/>
-      <c r="C36" s="58"/>
-      <c r="D36" s="58"/>
-      <c r="E36" s="58"/>
-      <c r="F36" s="58"/>
-      <c r="G36" s="62"/>
-      <c r="H36" s="63"/>
-      <c r="I36" s="63"/>
-      <c r="J36" s="63"/>
-      <c r="K36" s="64"/>
-      <c r="L36" s="76"/>
-      <c r="M36" s="74"/>
-      <c r="N36" s="74"/>
-      <c r="O36" s="74"/>
-      <c r="P36" s="74"/>
-      <c r="Q36" s="75"/>
+      <c r="A36" s="94"/>
+      <c r="B36" s="95"/>
+      <c r="C36" s="95"/>
+      <c r="D36" s="95"/>
+      <c r="E36" s="95"/>
+      <c r="F36" s="95"/>
+      <c r="G36" s="122"/>
+      <c r="H36" s="123"/>
+      <c r="I36" s="123"/>
+      <c r="J36" s="123"/>
+      <c r="K36" s="124"/>
+      <c r="L36" s="68"/>
+      <c r="M36" s="111"/>
+      <c r="N36" s="111"/>
+      <c r="O36" s="111"/>
+      <c r="P36" s="111"/>
+      <c r="Q36" s="112"/>
     </row>
     <row r="37" spans="1:17" ht="15">
-      <c r="A37" s="57"/>
-      <c r="B37" s="58"/>
-      <c r="C37" s="58"/>
-      <c r="D37" s="58"/>
-      <c r="E37" s="58"/>
-      <c r="F37" s="58"/>
-      <c r="G37" s="62"/>
-      <c r="H37" s="63"/>
-      <c r="I37" s="63"/>
-      <c r="J37" s="63"/>
-      <c r="K37" s="64"/>
-      <c r="L37" s="76"/>
-      <c r="M37" s="74"/>
-      <c r="N37" s="74"/>
-      <c r="O37" s="74"/>
-      <c r="P37" s="74"/>
-      <c r="Q37" s="75"/>
-    </row>
-    <row r="38" spans="1:17">
-      <c r="A38" s="57"/>
-      <c r="B38" s="58"/>
-      <c r="C38" s="58"/>
-      <c r="D38" s="58"/>
-      <c r="E38" s="58"/>
-      <c r="F38" s="58"/>
-      <c r="G38" s="65"/>
-      <c r="H38" s="66"/>
-      <c r="I38" s="66"/>
-      <c r="J38" s="66"/>
-      <c r="K38" s="67"/>
-      <c r="L38" s="51" t="s">
+      <c r="A37" s="94"/>
+      <c r="B37" s="95"/>
+      <c r="C37" s="95"/>
+      <c r="D37" s="95"/>
+      <c r="E37" s="95"/>
+      <c r="F37" s="95"/>
+      <c r="G37" s="122"/>
+      <c r="H37" s="123"/>
+      <c r="I37" s="123"/>
+      <c r="J37" s="123"/>
+      <c r="K37" s="124"/>
+      <c r="L37" s="68"/>
+      <c r="M37" s="111"/>
+      <c r="N37" s="111"/>
+      <c r="O37" s="111"/>
+      <c r="P37" s="111"/>
+      <c r="Q37" s="112"/>
+    </row>
+    <row r="38" spans="1:17" ht="45" customHeight="1">
+      <c r="A38" s="94"/>
+      <c r="B38" s="95"/>
+      <c r="C38" s="95"/>
+      <c r="D38" s="95"/>
+      <c r="E38" s="95"/>
+      <c r="F38" s="95"/>
+      <c r="G38" s="115"/>
+      <c r="H38" s="116"/>
+      <c r="I38" s="116"/>
+      <c r="J38" s="116"/>
+      <c r="K38" s="117"/>
+      <c r="L38" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M38" s="77"/>
-      <c r="N38" s="66"/>
-      <c r="O38" s="66"/>
-      <c r="P38" s="66"/>
-      <c r="Q38" s="67"/>
+      <c r="M38" s="69"/>
+      <c r="N38" s="116"/>
+      <c r="O38" s="116"/>
+      <c r="P38" s="116"/>
+      <c r="Q38" s="117"/>
     </row>
     <row r="39" spans="1:17" ht="15">
-      <c r="A39" s="55" t="s">
+      <c r="A39" s="79" t="s">
         <v>205</v>
       </c>
-      <c r="B39" s="56"/>
-      <c r="C39" s="56"/>
-      <c r="D39" s="56"/>
-      <c r="E39" s="56"/>
-      <c r="F39" s="79"/>
-      <c r="G39" s="59"/>
-      <c r="H39" s="60"/>
-      <c r="I39" s="60"/>
-      <c r="J39" s="60"/>
-      <c r="K39" s="61"/>
-      <c r="L39" s="76"/>
-      <c r="M39" s="74"/>
-      <c r="N39" s="74"/>
-      <c r="O39" s="74"/>
-      <c r="P39" s="74"/>
-      <c r="Q39" s="75"/>
+      <c r="B39" s="89"/>
+      <c r="C39" s="89"/>
+      <c r="D39" s="89"/>
+      <c r="E39" s="89"/>
+      <c r="F39" s="90"/>
+      <c r="G39" s="121"/>
+      <c r="H39" s="113"/>
+      <c r="I39" s="113"/>
+      <c r="J39" s="113"/>
+      <c r="K39" s="114"/>
+      <c r="L39" s="68"/>
+      <c r="M39" s="111"/>
+      <c r="N39" s="111"/>
+      <c r="O39" s="111"/>
+      <c r="P39" s="111"/>
+      <c r="Q39" s="112"/>
     </row>
     <row r="40" spans="1:17" ht="15">
-      <c r="A40" s="57"/>
-      <c r="B40" s="58"/>
-      <c r="C40" s="58"/>
-      <c r="D40" s="58"/>
-      <c r="E40" s="58"/>
-      <c r="F40" s="80"/>
-      <c r="G40" s="62"/>
-      <c r="H40" s="63"/>
-      <c r="I40" s="63"/>
-      <c r="J40" s="63"/>
-      <c r="K40" s="64"/>
-      <c r="L40" s="76"/>
-      <c r="M40" s="74"/>
-      <c r="N40" s="74"/>
-      <c r="O40" s="74"/>
-      <c r="P40" s="74"/>
-      <c r="Q40" s="75"/>
+      <c r="A40" s="94"/>
+      <c r="B40" s="95"/>
+      <c r="C40" s="95"/>
+      <c r="D40" s="95"/>
+      <c r="E40" s="95"/>
+      <c r="F40" s="96"/>
+      <c r="G40" s="122"/>
+      <c r="H40" s="123"/>
+      <c r="I40" s="123"/>
+      <c r="J40" s="123"/>
+      <c r="K40" s="124"/>
+      <c r="L40" s="68"/>
+      <c r="M40" s="111"/>
+      <c r="N40" s="111"/>
+      <c r="O40" s="111"/>
+      <c r="P40" s="111"/>
+      <c r="Q40" s="112"/>
     </row>
     <row r="41" spans="1:17" ht="15">
-      <c r="A41" s="57"/>
-      <c r="B41" s="58"/>
-      <c r="C41" s="58"/>
-      <c r="D41" s="58"/>
-      <c r="E41" s="58"/>
-      <c r="F41" s="80"/>
-      <c r="G41" s="62"/>
-      <c r="H41" s="63"/>
-      <c r="I41" s="63"/>
-      <c r="J41" s="63"/>
-      <c r="K41" s="64"/>
-      <c r="L41" s="76"/>
-      <c r="M41" s="74"/>
-      <c r="N41" s="74"/>
-      <c r="O41" s="74"/>
-      <c r="P41" s="74"/>
-      <c r="Q41" s="75"/>
-    </row>
-    <row r="42" spans="1:17">
-      <c r="A42" s="81"/>
-      <c r="B42" s="82"/>
-      <c r="C42" s="82"/>
-      <c r="D42" s="82"/>
-      <c r="E42" s="82"/>
-      <c r="F42" s="83"/>
-      <c r="G42" s="65"/>
-      <c r="H42" s="66"/>
-      <c r="I42" s="66"/>
-      <c r="J42" s="66"/>
-      <c r="K42" s="67"/>
-      <c r="L42" s="51" t="s">
+      <c r="A41" s="94"/>
+      <c r="B41" s="95"/>
+      <c r="C41" s="95"/>
+      <c r="D41" s="95"/>
+      <c r="E41" s="95"/>
+      <c r="F41" s="96"/>
+      <c r="G41" s="122"/>
+      <c r="H41" s="123"/>
+      <c r="I41" s="123"/>
+      <c r="J41" s="123"/>
+      <c r="K41" s="124"/>
+      <c r="L41" s="68"/>
+      <c r="M41" s="111"/>
+      <c r="N41" s="111"/>
+      <c r="O41" s="111"/>
+      <c r="P41" s="111"/>
+      <c r="Q41" s="112"/>
+    </row>
+    <row r="42" spans="1:17" ht="45" customHeight="1">
+      <c r="A42" s="100"/>
+      <c r="B42" s="101"/>
+      <c r="C42" s="101"/>
+      <c r="D42" s="101"/>
+      <c r="E42" s="101"/>
+      <c r="F42" s="102"/>
+      <c r="G42" s="115"/>
+      <c r="H42" s="116"/>
+      <c r="I42" s="116"/>
+      <c r="J42" s="116"/>
+      <c r="K42" s="117"/>
+      <c r="L42" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M42" s="77"/>
-      <c r="N42" s="66"/>
-      <c r="O42" s="66"/>
-      <c r="P42" s="66"/>
-      <c r="Q42" s="67"/>
+      <c r="M42" s="69"/>
+      <c r="N42" s="116"/>
+      <c r="O42" s="116"/>
+      <c r="P42" s="116"/>
+      <c r="Q42" s="117"/>
     </row>
     <row r="43" spans="1:17" ht="12.75">
-      <c r="A43" s="71" t="s">
+      <c r="A43" s="76" t="s">
         <v>206</v>
       </c>
-      <c r="B43" s="54"/>
-      <c r="C43" s="54"/>
-      <c r="D43" s="54"/>
-      <c r="E43" s="54"/>
-      <c r="F43" s="54"/>
-      <c r="G43" s="54"/>
-      <c r="H43" s="54"/>
-      <c r="I43" s="54"/>
-      <c r="J43" s="54"/>
-      <c r="K43" s="54"/>
-      <c r="L43" s="54"/>
-      <c r="M43" s="54"/>
-      <c r="N43" s="54"/>
-      <c r="O43" s="54"/>
-      <c r="P43" s="54"/>
-      <c r="Q43" s="72"/>
+      <c r="B43" s="105"/>
+      <c r="C43" s="105"/>
+      <c r="D43" s="105"/>
+      <c r="E43" s="105"/>
+      <c r="F43" s="105"/>
+      <c r="G43" s="105"/>
+      <c r="H43" s="105"/>
+      <c r="I43" s="105"/>
+      <c r="J43" s="105"/>
+      <c r="K43" s="105"/>
+      <c r="L43" s="105"/>
+      <c r="M43" s="105"/>
+      <c r="N43" s="105"/>
+      <c r="O43" s="105"/>
+      <c r="P43" s="105"/>
+      <c r="Q43" s="104"/>
     </row>
     <row r="44" spans="1:17" ht="30.75" customHeight="1">
-      <c r="A44" s="53" t="s">
+      <c r="A44" s="77" t="s">
         <v>170</v>
       </c>
-      <c r="B44" s="54"/>
-      <c r="C44" s="54"/>
-      <c r="D44" s="54"/>
-      <c r="E44" s="54"/>
-      <c r="F44" s="54"/>
-      <c r="G44" s="53" t="s">
+      <c r="B44" s="105"/>
+      <c r="C44" s="105"/>
+      <c r="D44" s="105"/>
+      <c r="E44" s="105"/>
+      <c r="F44" s="105"/>
+      <c r="G44" s="77" t="s">
         <v>200</v>
       </c>
-      <c r="H44" s="54"/>
-      <c r="I44" s="54"/>
-      <c r="J44" s="54"/>
-      <c r="K44" s="54"/>
-      <c r="L44" s="53" t="s">
+      <c r="H44" s="105"/>
+      <c r="I44" s="105"/>
+      <c r="J44" s="105"/>
+      <c r="K44" s="105"/>
+      <c r="L44" s="77" t="s">
         <v>171</v>
       </c>
-      <c r="M44" s="54"/>
-      <c r="N44" s="54"/>
-      <c r="O44" s="54"/>
-      <c r="P44" s="54"/>
-      <c r="Q44" s="72"/>
+      <c r="M44" s="105"/>
+      <c r="N44" s="105"/>
+      <c r="O44" s="105"/>
+      <c r="P44" s="105"/>
+      <c r="Q44" s="104"/>
     </row>
     <row r="45" spans="1:17" ht="15">
-      <c r="A45" s="70" t="s">
+      <c r="A45" s="79" t="s">
         <v>207</v>
       </c>
-      <c r="B45" s="56"/>
-      <c r="C45" s="56"/>
-      <c r="D45" s="56"/>
-      <c r="E45" s="56"/>
-      <c r="F45" s="56"/>
-      <c r="G45" s="59"/>
-      <c r="H45" s="60"/>
-      <c r="I45" s="60"/>
-      <c r="J45" s="60"/>
-      <c r="K45" s="61"/>
-      <c r="L45" s="76"/>
-      <c r="M45" s="74"/>
-      <c r="N45" s="74"/>
-      <c r="O45" s="74"/>
-      <c r="P45" s="74"/>
-      <c r="Q45" s="75"/>
-    </row>
-    <row r="46" spans="1:17">
-      <c r="A46" s="57"/>
-      <c r="B46" s="58"/>
-      <c r="C46" s="58"/>
-      <c r="D46" s="58"/>
-      <c r="E46" s="58"/>
-      <c r="F46" s="58"/>
-      <c r="G46" s="65"/>
-      <c r="H46" s="66"/>
-      <c r="I46" s="66"/>
-      <c r="J46" s="66"/>
-      <c r="K46" s="67"/>
-      <c r="L46" s="51" t="s">
+      <c r="B45" s="89"/>
+      <c r="C45" s="89"/>
+      <c r="D45" s="89"/>
+      <c r="E45" s="89"/>
+      <c r="F45" s="89"/>
+      <c r="G45" s="121"/>
+      <c r="H45" s="113"/>
+      <c r="I45" s="113"/>
+      <c r="J45" s="113"/>
+      <c r="K45" s="114"/>
+      <c r="L45" s="68"/>
+      <c r="M45" s="111"/>
+      <c r="N45" s="111"/>
+      <c r="O45" s="111"/>
+      <c r="P45" s="111"/>
+      <c r="Q45" s="112"/>
+    </row>
+    <row r="46" spans="1:17" ht="45" customHeight="1">
+      <c r="A46" s="94"/>
+      <c r="B46" s="95"/>
+      <c r="C46" s="95"/>
+      <c r="D46" s="95"/>
+      <c r="E46" s="95"/>
+      <c r="F46" s="95"/>
+      <c r="G46" s="115"/>
+      <c r="H46" s="116"/>
+      <c r="I46" s="116"/>
+      <c r="J46" s="116"/>
+      <c r="K46" s="117"/>
+      <c r="L46" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M46" s="77"/>
-      <c r="N46" s="66"/>
-      <c r="O46" s="66"/>
-      <c r="P46" s="66"/>
-      <c r="Q46" s="67"/>
+      <c r="M46" s="69"/>
+      <c r="N46" s="116"/>
+      <c r="O46" s="116"/>
+      <c r="P46" s="116"/>
+      <c r="Q46" s="117"/>
     </row>
     <row r="47" spans="1:17" ht="15">
-      <c r="A47" s="70" t="s">
+      <c r="A47" s="79" t="s">
         <v>208</v>
       </c>
-      <c r="B47" s="56"/>
-      <c r="C47" s="56"/>
-      <c r="D47" s="56"/>
-      <c r="E47" s="56"/>
-      <c r="F47" s="56"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="60"/>
-      <c r="I47" s="60"/>
-      <c r="J47" s="60"/>
-      <c r="K47" s="61"/>
-      <c r="L47" s="76"/>
-      <c r="M47" s="74"/>
-      <c r="N47" s="74"/>
-      <c r="O47" s="74"/>
-      <c r="P47" s="74"/>
-      <c r="Q47" s="75"/>
-    </row>
-    <row r="48" spans="1:17">
-      <c r="A48" s="57"/>
-      <c r="B48" s="58"/>
-      <c r="C48" s="58"/>
-      <c r="D48" s="58"/>
-      <c r="E48" s="58"/>
-      <c r="F48" s="58"/>
-      <c r="G48" s="65"/>
-      <c r="H48" s="66"/>
-      <c r="I48" s="66"/>
-      <c r="J48" s="66"/>
-      <c r="K48" s="67"/>
-      <c r="L48" s="51" t="s">
+      <c r="B47" s="89"/>
+      <c r="C47" s="89"/>
+      <c r="D47" s="89"/>
+      <c r="E47" s="89"/>
+      <c r="F47" s="89"/>
+      <c r="G47" s="121"/>
+      <c r="H47" s="113"/>
+      <c r="I47" s="113"/>
+      <c r="J47" s="113"/>
+      <c r="K47" s="114"/>
+      <c r="L47" s="68"/>
+      <c r="M47" s="111"/>
+      <c r="N47" s="111"/>
+      <c r="O47" s="111"/>
+      <c r="P47" s="111"/>
+      <c r="Q47" s="112"/>
+    </row>
+    <row r="48" spans="1:17" ht="45" customHeight="1">
+      <c r="A48" s="94"/>
+      <c r="B48" s="95"/>
+      <c r="C48" s="95"/>
+      <c r="D48" s="95"/>
+      <c r="E48" s="95"/>
+      <c r="F48" s="95"/>
+      <c r="G48" s="115"/>
+      <c r="H48" s="116"/>
+      <c r="I48" s="116"/>
+      <c r="J48" s="116"/>
+      <c r="K48" s="117"/>
+      <c r="L48" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M48" s="77"/>
-      <c r="N48" s="66"/>
-      <c r="O48" s="66"/>
-      <c r="P48" s="66"/>
-      <c r="Q48" s="67"/>
+      <c r="M48" s="69"/>
+      <c r="N48" s="116"/>
+      <c r="O48" s="116"/>
+      <c r="P48" s="116"/>
+      <c r="Q48" s="117"/>
     </row>
     <row r="49" spans="1:17" ht="15">
-      <c r="A49" s="70" t="s">
+      <c r="A49" s="79" t="s">
         <v>209</v>
       </c>
-      <c r="B49" s="56"/>
-      <c r="C49" s="56"/>
-      <c r="D49" s="56"/>
-      <c r="E49" s="56"/>
-      <c r="F49" s="56"/>
-      <c r="G49" s="59"/>
-      <c r="H49" s="60"/>
-      <c r="I49" s="60"/>
-      <c r="J49" s="60"/>
-      <c r="K49" s="61"/>
-      <c r="L49" s="76"/>
-      <c r="M49" s="74"/>
-      <c r="N49" s="74"/>
-      <c r="O49" s="74"/>
-      <c r="P49" s="74"/>
-      <c r="Q49" s="75"/>
-    </row>
-    <row r="50" spans="1:17">
-      <c r="A50" s="57"/>
-      <c r="B50" s="58"/>
-      <c r="C50" s="58"/>
-      <c r="D50" s="58"/>
-      <c r="E50" s="58"/>
-      <c r="F50" s="58"/>
-      <c r="G50" s="65"/>
-      <c r="H50" s="66"/>
-      <c r="I50" s="66"/>
-      <c r="J50" s="66"/>
-      <c r="K50" s="67"/>
-      <c r="L50" s="51" t="s">
+      <c r="B49" s="89"/>
+      <c r="C49" s="89"/>
+      <c r="D49" s="89"/>
+      <c r="E49" s="89"/>
+      <c r="F49" s="89"/>
+      <c r="G49" s="121"/>
+      <c r="H49" s="113"/>
+      <c r="I49" s="113"/>
+      <c r="J49" s="113"/>
+      <c r="K49" s="114"/>
+      <c r="L49" s="68"/>
+      <c r="M49" s="111"/>
+      <c r="N49" s="111"/>
+      <c r="O49" s="111"/>
+      <c r="P49" s="111"/>
+      <c r="Q49" s="112"/>
+    </row>
+    <row r="50" spans="1:17" ht="45" customHeight="1">
+      <c r="A50" s="94"/>
+      <c r="B50" s="95"/>
+      <c r="C50" s="95"/>
+      <c r="D50" s="95"/>
+      <c r="E50" s="95"/>
+      <c r="F50" s="95"/>
+      <c r="G50" s="115"/>
+      <c r="H50" s="116"/>
+      <c r="I50" s="116"/>
+      <c r="J50" s="116"/>
+      <c r="K50" s="117"/>
+      <c r="L50" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M50" s="77"/>
-      <c r="N50" s="66"/>
-      <c r="O50" s="66"/>
-      <c r="P50" s="66"/>
-      <c r="Q50" s="67"/>
+      <c r="M50" s="69"/>
+      <c r="N50" s="116"/>
+      <c r="O50" s="116"/>
+      <c r="P50" s="116"/>
+      <c r="Q50" s="117"/>
     </row>
     <row r="51" spans="1:17" ht="15">
-      <c r="A51" s="55" t="s">
+      <c r="A51" s="79" t="s">
         <v>210</v>
       </c>
-      <c r="B51" s="56"/>
-      <c r="C51" s="56"/>
-      <c r="D51" s="56"/>
-      <c r="E51" s="56"/>
-      <c r="F51" s="56"/>
-      <c r="G51" s="59"/>
-      <c r="H51" s="60"/>
-      <c r="I51" s="60"/>
-      <c r="J51" s="60"/>
-      <c r="K51" s="61"/>
-      <c r="L51" s="76"/>
-      <c r="M51" s="74"/>
-      <c r="N51" s="74"/>
-      <c r="O51" s="74"/>
-      <c r="P51" s="74"/>
-      <c r="Q51" s="75"/>
-    </row>
-    <row r="52" spans="1:17">
-      <c r="A52" s="57"/>
-      <c r="B52" s="58"/>
-      <c r="C52" s="58"/>
-      <c r="D52" s="58"/>
-      <c r="E52" s="58"/>
-      <c r="F52" s="58"/>
-      <c r="G52" s="65"/>
-      <c r="H52" s="66"/>
-      <c r="I52" s="66"/>
-      <c r="J52" s="66"/>
-      <c r="K52" s="67"/>
-      <c r="L52" s="51" t="s">
+      <c r="B51" s="89"/>
+      <c r="C51" s="89"/>
+      <c r="D51" s="89"/>
+      <c r="E51" s="89"/>
+      <c r="F51" s="89"/>
+      <c r="G51" s="121"/>
+      <c r="H51" s="113"/>
+      <c r="I51" s="113"/>
+      <c r="J51" s="113"/>
+      <c r="K51" s="114"/>
+      <c r="L51" s="68"/>
+      <c r="M51" s="111"/>
+      <c r="N51" s="111"/>
+      <c r="O51" s="111"/>
+      <c r="P51" s="111"/>
+      <c r="Q51" s="112"/>
+    </row>
+    <row r="52" spans="1:17" ht="45" customHeight="1">
+      <c r="A52" s="94"/>
+      <c r="B52" s="95"/>
+      <c r="C52" s="95"/>
+      <c r="D52" s="95"/>
+      <c r="E52" s="95"/>
+      <c r="F52" s="95"/>
+      <c r="G52" s="115"/>
+      <c r="H52" s="116"/>
+      <c r="I52" s="116"/>
+      <c r="J52" s="116"/>
+      <c r="K52" s="117"/>
+      <c r="L52" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M52" s="77"/>
-      <c r="N52" s="66"/>
-      <c r="O52" s="66"/>
-      <c r="P52" s="66"/>
-      <c r="Q52" s="67"/>
+      <c r="M52" s="69"/>
+      <c r="N52" s="116"/>
+      <c r="O52" s="116"/>
+      <c r="P52" s="116"/>
+      <c r="Q52" s="117"/>
     </row>
     <row r="53" spans="1:17" ht="15">
-      <c r="A53" s="70" t="s">
+      <c r="A53" s="79" t="s">
         <v>211</v>
       </c>
-      <c r="B53" s="56"/>
-      <c r="C53" s="56"/>
-      <c r="D53" s="56"/>
-      <c r="E53" s="56"/>
-      <c r="F53" s="56"/>
-      <c r="G53" s="59"/>
-      <c r="H53" s="60"/>
-      <c r="I53" s="60"/>
-      <c r="J53" s="60"/>
-      <c r="K53" s="61"/>
-      <c r="L53" s="76"/>
-      <c r="M53" s="74"/>
-      <c r="N53" s="74"/>
-      <c r="O53" s="74"/>
-      <c r="P53" s="74"/>
-      <c r="Q53" s="75"/>
-    </row>
-    <row r="54" spans="1:17">
-      <c r="A54" s="57"/>
-      <c r="B54" s="58"/>
-      <c r="C54" s="58"/>
-      <c r="D54" s="58"/>
-      <c r="E54" s="58"/>
-      <c r="F54" s="58"/>
-      <c r="G54" s="65"/>
-      <c r="H54" s="66"/>
-      <c r="I54" s="66"/>
-      <c r="J54" s="66"/>
-      <c r="K54" s="67"/>
-      <c r="L54" s="51" t="s">
+      <c r="B53" s="89"/>
+      <c r="C53" s="89"/>
+      <c r="D53" s="89"/>
+      <c r="E53" s="89"/>
+      <c r="F53" s="89"/>
+      <c r="G53" s="121"/>
+      <c r="H53" s="113"/>
+      <c r="I53" s="113"/>
+      <c r="J53" s="113"/>
+      <c r="K53" s="114"/>
+      <c r="L53" s="68"/>
+      <c r="M53" s="111"/>
+      <c r="N53" s="111"/>
+      <c r="O53" s="111"/>
+      <c r="P53" s="111"/>
+      <c r="Q53" s="112"/>
+    </row>
+    <row r="54" spans="1:17" ht="45" customHeight="1">
+      <c r="A54" s="94"/>
+      <c r="B54" s="95"/>
+      <c r="C54" s="95"/>
+      <c r="D54" s="95"/>
+      <c r="E54" s="95"/>
+      <c r="F54" s="95"/>
+      <c r="G54" s="115"/>
+      <c r="H54" s="116"/>
+      <c r="I54" s="116"/>
+      <c r="J54" s="116"/>
+      <c r="K54" s="117"/>
+      <c r="L54" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M54" s="77"/>
-      <c r="N54" s="66"/>
-      <c r="O54" s="66"/>
-      <c r="P54" s="66"/>
-      <c r="Q54" s="67"/>
+      <c r="M54" s="69"/>
+      <c r="N54" s="116"/>
+      <c r="O54" s="116"/>
+      <c r="P54" s="116"/>
+      <c r="Q54" s="117"/>
     </row>
     <row r="55" spans="1:17" ht="15">
-      <c r="A55" s="70" t="s">
+      <c r="A55" s="79" t="s">
         <v>212</v>
       </c>
-      <c r="B55" s="56"/>
-      <c r="C55" s="56"/>
-      <c r="D55" s="56"/>
-      <c r="E55" s="56"/>
-      <c r="F55" s="56"/>
-      <c r="G55" s="59"/>
-      <c r="H55" s="60"/>
-      <c r="I55" s="60"/>
-      <c r="J55" s="60"/>
-      <c r="K55" s="61"/>
-      <c r="L55" s="76"/>
-      <c r="M55" s="74"/>
-      <c r="N55" s="74"/>
-      <c r="O55" s="74"/>
-      <c r="P55" s="74"/>
-      <c r="Q55" s="75"/>
-    </row>
-    <row r="56" spans="1:17">
-      <c r="A56" s="57"/>
-      <c r="B56" s="58"/>
-      <c r="C56" s="58"/>
-      <c r="D56" s="58"/>
-      <c r="E56" s="58"/>
-      <c r="F56" s="58"/>
-      <c r="G56" s="65"/>
-      <c r="H56" s="66"/>
-      <c r="I56" s="66"/>
-      <c r="J56" s="66"/>
-      <c r="K56" s="67"/>
-      <c r="L56" s="51" t="s">
+      <c r="B55" s="89"/>
+      <c r="C55" s="89"/>
+      <c r="D55" s="89"/>
+      <c r="E55" s="89"/>
+      <c r="F55" s="89"/>
+      <c r="G55" s="121"/>
+      <c r="H55" s="113"/>
+      <c r="I55" s="113"/>
+      <c r="J55" s="113"/>
+      <c r="K55" s="114"/>
+      <c r="L55" s="68"/>
+      <c r="M55" s="111"/>
+      <c r="N55" s="111"/>
+      <c r="O55" s="111"/>
+      <c r="P55" s="111"/>
+      <c r="Q55" s="112"/>
+    </row>
+    <row r="56" spans="1:17" ht="45" customHeight="1">
+      <c r="A56" s="94"/>
+      <c r="B56" s="95"/>
+      <c r="C56" s="95"/>
+      <c r="D56" s="95"/>
+      <c r="E56" s="95"/>
+      <c r="F56" s="95"/>
+      <c r="G56" s="115"/>
+      <c r="H56" s="116"/>
+      <c r="I56" s="116"/>
+      <c r="J56" s="116"/>
+      <c r="K56" s="117"/>
+      <c r="L56" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M56" s="77"/>
-      <c r="N56" s="66"/>
-      <c r="O56" s="66"/>
-      <c r="P56" s="66"/>
-      <c r="Q56" s="67"/>
+      <c r="M56" s="69"/>
+      <c r="N56" s="116"/>
+      <c r="O56" s="116"/>
+      <c r="P56" s="116"/>
+      <c r="Q56" s="117"/>
     </row>
     <row r="57" spans="1:17" ht="12.75">
-      <c r="A57" s="71" t="s">
+      <c r="A57" s="76" t="s">
         <v>213</v>
       </c>
-      <c r="B57" s="54"/>
-      <c r="C57" s="54"/>
-      <c r="D57" s="54"/>
-      <c r="E57" s="54"/>
-      <c r="F57" s="54"/>
-      <c r="G57" s="54"/>
-      <c r="H57" s="54"/>
-      <c r="I57" s="54"/>
-      <c r="J57" s="54"/>
-      <c r="K57" s="54"/>
-      <c r="L57" s="54"/>
-      <c r="M57" s="54"/>
-      <c r="N57" s="54"/>
-      <c r="O57" s="54"/>
-      <c r="P57" s="54"/>
-      <c r="Q57" s="72"/>
+      <c r="B57" s="105"/>
+      <c r="C57" s="105"/>
+      <c r="D57" s="105"/>
+      <c r="E57" s="105"/>
+      <c r="F57" s="105"/>
+      <c r="G57" s="105"/>
+      <c r="H57" s="105"/>
+      <c r="I57" s="105"/>
+      <c r="J57" s="105"/>
+      <c r="K57" s="105"/>
+      <c r="L57" s="105"/>
+      <c r="M57" s="105"/>
+      <c r="N57" s="105"/>
+      <c r="O57" s="105"/>
+      <c r="P57" s="105"/>
+      <c r="Q57" s="104"/>
     </row>
     <row r="58" spans="1:17" ht="27.75" customHeight="1">
-      <c r="A58" s="53" t="s">
+      <c r="A58" s="77" t="s">
         <v>170</v>
       </c>
-      <c r="B58" s="54"/>
-      <c r="C58" s="54"/>
-      <c r="D58" s="54"/>
-      <c r="E58" s="54"/>
-      <c r="F58" s="54"/>
-      <c r="G58" s="73" t="s">
+      <c r="B58" s="105"/>
+      <c r="C58" s="105"/>
+      <c r="D58" s="105"/>
+      <c r="E58" s="105"/>
+      <c r="F58" s="105"/>
+      <c r="G58" s="85" t="s">
         <v>200</v>
       </c>
-      <c r="H58" s="74"/>
-      <c r="I58" s="74"/>
-      <c r="J58" s="74"/>
-      <c r="K58" s="74"/>
-      <c r="L58" s="73" t="s">
+      <c r="H58" s="111"/>
+      <c r="I58" s="111"/>
+      <c r="J58" s="111"/>
+      <c r="K58" s="111"/>
+      <c r="L58" s="85" t="s">
         <v>171</v>
       </c>
-      <c r="M58" s="74"/>
-      <c r="N58" s="74"/>
-      <c r="O58" s="74"/>
-      <c r="P58" s="74"/>
-      <c r="Q58" s="75"/>
+      <c r="M58" s="111"/>
+      <c r="N58" s="111"/>
+      <c r="O58" s="111"/>
+      <c r="P58" s="111"/>
+      <c r="Q58" s="112"/>
     </row>
     <row r="59" spans="1:17" ht="15">
-      <c r="A59" s="55" t="s">
+      <c r="A59" s="79" t="s">
         <v>214</v>
       </c>
-      <c r="B59" s="56"/>
-      <c r="C59" s="56"/>
-      <c r="D59" s="56"/>
-      <c r="E59" s="56"/>
-      <c r="F59" s="56"/>
-      <c r="G59" s="59"/>
-      <c r="H59" s="60"/>
-      <c r="I59" s="60"/>
-      <c r="J59" s="60"/>
-      <c r="K59" s="61"/>
-      <c r="L59" s="76"/>
-      <c r="M59" s="74"/>
-      <c r="N59" s="74"/>
-      <c r="O59" s="74"/>
-      <c r="P59" s="74"/>
-      <c r="Q59" s="75"/>
+      <c r="B59" s="89"/>
+      <c r="C59" s="89"/>
+      <c r="D59" s="89"/>
+      <c r="E59" s="89"/>
+      <c r="F59" s="89"/>
+      <c r="G59" s="121"/>
+      <c r="H59" s="113"/>
+      <c r="I59" s="113"/>
+      <c r="J59" s="113"/>
+      <c r="K59" s="114"/>
+      <c r="L59" s="68"/>
+      <c r="M59" s="111"/>
+      <c r="N59" s="111"/>
+      <c r="O59" s="111"/>
+      <c r="P59" s="111"/>
+      <c r="Q59" s="112"/>
     </row>
     <row r="60" spans="1:17" ht="15">
-      <c r="A60" s="57"/>
-      <c r="B60" s="58"/>
-      <c r="C60" s="58"/>
-      <c r="D60" s="58"/>
-      <c r="E60" s="58"/>
-      <c r="F60" s="58"/>
-      <c r="G60" s="62"/>
-      <c r="H60" s="63"/>
-      <c r="I60" s="63"/>
-      <c r="J60" s="63"/>
-      <c r="K60" s="64"/>
-      <c r="L60" s="76"/>
-      <c r="M60" s="74"/>
-      <c r="N60" s="74"/>
-      <c r="O60" s="74"/>
-      <c r="P60" s="74"/>
-      <c r="Q60" s="75"/>
+      <c r="A60" s="94"/>
+      <c r="B60" s="95"/>
+      <c r="C60" s="95"/>
+      <c r="D60" s="95"/>
+      <c r="E60" s="95"/>
+      <c r="F60" s="95"/>
+      <c r="G60" s="122"/>
+      <c r="H60" s="123"/>
+      <c r="I60" s="123"/>
+      <c r="J60" s="123"/>
+      <c r="K60" s="124"/>
+      <c r="L60" s="68"/>
+      <c r="M60" s="111"/>
+      <c r="N60" s="111"/>
+      <c r="O60" s="111"/>
+      <c r="P60" s="111"/>
+      <c r="Q60" s="112"/>
     </row>
     <row r="61" spans="1:17" ht="15">
-      <c r="A61" s="57"/>
-      <c r="B61" s="58"/>
-      <c r="C61" s="58"/>
-      <c r="D61" s="58"/>
-      <c r="E61" s="58"/>
-      <c r="F61" s="58"/>
-      <c r="G61" s="62"/>
-      <c r="H61" s="63"/>
-      <c r="I61" s="63"/>
-      <c r="J61" s="63"/>
-      <c r="K61" s="64"/>
-      <c r="L61" s="76"/>
-      <c r="M61" s="74"/>
-      <c r="N61" s="74"/>
-      <c r="O61" s="74"/>
-      <c r="P61" s="74"/>
-      <c r="Q61" s="75"/>
+      <c r="A61" s="94"/>
+      <c r="B61" s="95"/>
+      <c r="C61" s="95"/>
+      <c r="D61" s="95"/>
+      <c r="E61" s="95"/>
+      <c r="F61" s="95"/>
+      <c r="G61" s="122"/>
+      <c r="H61" s="123"/>
+      <c r="I61" s="123"/>
+      <c r="J61" s="123"/>
+      <c r="K61" s="124"/>
+      <c r="L61" s="68"/>
+      <c r="M61" s="111"/>
+      <c r="N61" s="111"/>
+      <c r="O61" s="111"/>
+      <c r="P61" s="111"/>
+      <c r="Q61" s="112"/>
     </row>
     <row r="62" spans="1:17" ht="15">
-      <c r="A62" s="57"/>
-      <c r="B62" s="58"/>
-      <c r="C62" s="58"/>
-      <c r="D62" s="58"/>
-      <c r="E62" s="58"/>
-      <c r="F62" s="58"/>
-      <c r="G62" s="62"/>
-      <c r="H62" s="63"/>
-      <c r="I62" s="63"/>
-      <c r="J62" s="63"/>
-      <c r="K62" s="64"/>
-      <c r="L62" s="76"/>
-      <c r="M62" s="74"/>
-      <c r="N62" s="74"/>
-      <c r="O62" s="74"/>
-      <c r="P62" s="74"/>
-      <c r="Q62" s="75"/>
-    </row>
-    <row r="63" spans="1:17">
-      <c r="A63" s="57"/>
-      <c r="B63" s="58"/>
-      <c r="C63" s="58"/>
-      <c r="D63" s="58"/>
-      <c r="E63" s="58"/>
-      <c r="F63" s="58"/>
-      <c r="G63" s="65"/>
-      <c r="H63" s="66"/>
-      <c r="I63" s="66"/>
-      <c r="J63" s="66"/>
-      <c r="K63" s="67"/>
-      <c r="L63" s="51" t="s">
+      <c r="A62" s="94"/>
+      <c r="B62" s="95"/>
+      <c r="C62" s="95"/>
+      <c r="D62" s="95"/>
+      <c r="E62" s="95"/>
+      <c r="F62" s="95"/>
+      <c r="G62" s="122"/>
+      <c r="H62" s="123"/>
+      <c r="I62" s="123"/>
+      <c r="J62" s="123"/>
+      <c r="K62" s="124"/>
+      <c r="L62" s="68"/>
+      <c r="M62" s="111"/>
+      <c r="N62" s="111"/>
+      <c r="O62" s="111"/>
+      <c r="P62" s="111"/>
+      <c r="Q62" s="112"/>
+    </row>
+    <row r="63" spans="1:17" ht="45" customHeight="1">
+      <c r="A63" s="94"/>
+      <c r="B63" s="95"/>
+      <c r="C63" s="95"/>
+      <c r="D63" s="95"/>
+      <c r="E63" s="95"/>
+      <c r="F63" s="95"/>
+      <c r="G63" s="115"/>
+      <c r="H63" s="116"/>
+      <c r="I63" s="116"/>
+      <c r="J63" s="116"/>
+      <c r="K63" s="117"/>
+      <c r="L63" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M63" s="77"/>
-      <c r="N63" s="66"/>
-      <c r="O63" s="66"/>
-      <c r="P63" s="66"/>
-      <c r="Q63" s="67"/>
+      <c r="M63" s="69"/>
+      <c r="N63" s="116"/>
+      <c r="O63" s="116"/>
+      <c r="P63" s="116"/>
+      <c r="Q63" s="117"/>
     </row>
     <row r="64" spans="1:17" ht="15">
-      <c r="A64" s="55" t="s">
+      <c r="A64" s="79" t="s">
         <v>215</v>
       </c>
-      <c r="B64" s="56"/>
-      <c r="C64" s="56"/>
-      <c r="D64" s="56"/>
-      <c r="E64" s="56"/>
-      <c r="F64" s="56"/>
-      <c r="G64" s="59"/>
-      <c r="H64" s="60"/>
-      <c r="I64" s="60"/>
-      <c r="J64" s="60"/>
-      <c r="K64" s="61"/>
-      <c r="L64" s="76"/>
-      <c r="M64" s="74"/>
-      <c r="N64" s="74"/>
-      <c r="O64" s="74"/>
-      <c r="P64" s="74"/>
-      <c r="Q64" s="75"/>
-    </row>
-    <row r="65" spans="1:17">
-      <c r="A65" s="57"/>
-      <c r="B65" s="58"/>
-      <c r="C65" s="58"/>
-      <c r="D65" s="58"/>
-      <c r="E65" s="58"/>
-      <c r="F65" s="58"/>
-      <c r="G65" s="65"/>
-      <c r="H65" s="66"/>
-      <c r="I65" s="66"/>
-      <c r="J65" s="66"/>
-      <c r="K65" s="67"/>
-      <c r="L65" s="51" t="s">
+      <c r="B64" s="89"/>
+      <c r="C64" s="89"/>
+      <c r="D64" s="89"/>
+      <c r="E64" s="89"/>
+      <c r="F64" s="89"/>
+      <c r="G64" s="121"/>
+      <c r="H64" s="113"/>
+      <c r="I64" s="113"/>
+      <c r="J64" s="113"/>
+      <c r="K64" s="114"/>
+      <c r="L64" s="68"/>
+      <c r="M64" s="111"/>
+      <c r="N64" s="111"/>
+      <c r="O64" s="111"/>
+      <c r="P64" s="111"/>
+      <c r="Q64" s="112"/>
+    </row>
+    <row r="65" spans="1:17" ht="45" customHeight="1">
+      <c r="A65" s="94"/>
+      <c r="B65" s="95"/>
+      <c r="C65" s="95"/>
+      <c r="D65" s="95"/>
+      <c r="E65" s="95"/>
+      <c r="F65" s="95"/>
+      <c r="G65" s="115"/>
+      <c r="H65" s="116"/>
+      <c r="I65" s="116"/>
+      <c r="J65" s="116"/>
+      <c r="K65" s="117"/>
+      <c r="L65" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="M65" s="77"/>
-      <c r="N65" s="66"/>
-      <c r="O65" s="66"/>
-      <c r="P65" s="66"/>
-      <c r="Q65" s="67"/>
+      <c r="M65" s="69"/>
+      <c r="N65" s="116"/>
+      <c r="O65" s="116"/>
+      <c r="P65" s="116"/>
+      <c r="Q65" s="117"/>
     </row>
     <row r="66" spans="1:17" ht="33.75" customHeight="1">
-      <c r="A66" s="68" t="s">
+      <c r="A66" s="84" t="s">
         <v>216</v>
       </c>
-      <c r="B66" s="56"/>
-      <c r="C66" s="56"/>
-      <c r="D66" s="56"/>
-      <c r="E66" s="56"/>
-      <c r="F66" s="56"/>
-      <c r="G66" s="69"/>
-      <c r="H66" s="60"/>
-      <c r="I66" s="60"/>
-      <c r="J66" s="60"/>
-      <c r="K66" s="61"/>
-      <c r="L66" s="90"/>
-      <c r="M66" s="74"/>
-      <c r="N66" s="74"/>
-      <c r="O66" s="74"/>
-      <c r="P66" s="74"/>
-      <c r="Q66" s="75"/>
-    </row>
-    <row r="67" spans="1:17" ht="33.75" customHeight="1">
-      <c r="A67" s="57"/>
-      <c r="B67" s="58"/>
-      <c r="C67" s="58"/>
-      <c r="D67" s="58"/>
-      <c r="E67" s="58"/>
-      <c r="F67" s="58"/>
-      <c r="G67" s="65"/>
-      <c r="H67" s="66"/>
-      <c r="I67" s="66"/>
-      <c r="J67" s="66"/>
-      <c r="K67" s="67"/>
-      <c r="L67" s="52" t="s">
+      <c r="B66" s="89"/>
+      <c r="C66" s="89"/>
+      <c r="D66" s="89"/>
+      <c r="E66" s="89"/>
+      <c r="F66" s="89"/>
+      <c r="G66" s="125"/>
+      <c r="H66" s="113"/>
+      <c r="I66" s="113"/>
+      <c r="J66" s="113"/>
+      <c r="K66" s="114"/>
+      <c r="L66" s="80"/>
+      <c r="M66" s="111"/>
+      <c r="N66" s="111"/>
+      <c r="O66" s="111"/>
+      <c r="P66" s="111"/>
+      <c r="Q66" s="112"/>
+    </row>
+    <row r="67" spans="1:17" ht="45" customHeight="1">
+      <c r="A67" s="94"/>
+      <c r="B67" s="95"/>
+      <c r="C67" s="95"/>
+      <c r="D67" s="95"/>
+      <c r="E67" s="95"/>
+      <c r="F67" s="95"/>
+      <c r="G67" s="115"/>
+      <c r="H67" s="116"/>
+      <c r="I67" s="116"/>
+      <c r="J67" s="116"/>
+      <c r="K67" s="117"/>
+      <c r="L67" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="M67" s="91"/>
-      <c r="N67" s="66"/>
-      <c r="O67" s="66"/>
-      <c r="P67" s="66"/>
-      <c r="Q67" s="67"/>
+      <c r="M67" s="81"/>
+      <c r="N67" s="116"/>
+      <c r="O67" s="116"/>
+      <c r="P67" s="116"/>
+      <c r="Q67" s="117"/>
     </row>
     <row r="68" spans="1:17" ht="12.75">
-      <c r="A68" s="92" t="s">
+      <c r="A68" s="82" t="s">
         <v>219</v>
       </c>
-      <c r="B68" s="54"/>
-      <c r="C68" s="54"/>
-      <c r="D68" s="54"/>
-      <c r="E68" s="54"/>
-      <c r="F68" s="54"/>
-      <c r="G68" s="54"/>
-      <c r="H68" s="54"/>
-      <c r="I68" s="54"/>
-      <c r="J68" s="54"/>
-      <c r="K68" s="54"/>
-      <c r="L68" s="54"/>
-      <c r="M68" s="54"/>
-      <c r="N68" s="54"/>
-      <c r="O68" s="54"/>
-      <c r="P68" s="54"/>
-      <c r="Q68" s="72"/>
-    </row>
-    <row r="69" spans="1:17" ht="90" customHeight="1">
-      <c r="A69" s="78"/>
-      <c r="B69" s="74"/>
-      <c r="C69" s="74"/>
-      <c r="D69" s="74"/>
-      <c r="E69" s="74"/>
-      <c r="F69" s="74"/>
-      <c r="G69" s="74"/>
-      <c r="H69" s="74"/>
-      <c r="I69" s="74"/>
-      <c r="J69" s="74"/>
-      <c r="K69" s="74"/>
-      <c r="L69" s="74"/>
-      <c r="M69" s="74"/>
-      <c r="N69" s="74"/>
-      <c r="O69" s="74"/>
-      <c r="P69" s="74"/>
-      <c r="Q69" s="75"/>
+      <c r="B68" s="105"/>
+      <c r="C68" s="105"/>
+      <c r="D68" s="105"/>
+      <c r="E68" s="105"/>
+      <c r="F68" s="105"/>
+      <c r="G68" s="105"/>
+      <c r="H68" s="105"/>
+      <c r="I68" s="105"/>
+      <c r="J68" s="105"/>
+      <c r="K68" s="105"/>
+      <c r="L68" s="105"/>
+      <c r="M68" s="105"/>
+      <c r="N68" s="105"/>
+      <c r="O68" s="105"/>
+      <c r="P68" s="105"/>
+      <c r="Q68" s="104"/>
+    </row>
+    <row r="69" spans="1:17" ht="195" customHeight="1">
+      <c r="A69" s="83"/>
+      <c r="B69" s="111"/>
+      <c r="C69" s="111"/>
+      <c r="D69" s="111"/>
+      <c r="E69" s="111"/>
+      <c r="F69" s="111"/>
+      <c r="G69" s="111"/>
+      <c r="H69" s="111"/>
+      <c r="I69" s="111"/>
+      <c r="J69" s="111"/>
+      <c r="K69" s="111"/>
+      <c r="L69" s="111"/>
+      <c r="M69" s="111"/>
+      <c r="N69" s="111"/>
+      <c r="O69" s="111"/>
+      <c r="P69" s="111"/>
+      <c r="Q69" s="112"/>
     </row>
     <row r="70" spans="1:17" ht="18" customHeight="1">
-      <c r="A70" s="55" t="s">
+      <c r="A70" s="79" t="s">
         <v>217</v>
       </c>
-      <c r="B70" s="56"/>
-      <c r="C70" s="56"/>
-      <c r="D70" s="56"/>
-      <c r="E70" s="56"/>
-      <c r="F70" s="56"/>
-      <c r="G70" s="56"/>
-      <c r="H70" s="56"/>
-      <c r="I70" s="56"/>
-      <c r="J70" s="56"/>
-      <c r="K70" s="56"/>
-      <c r="L70" s="56"/>
-      <c r="M70" s="56"/>
-      <c r="N70" s="56"/>
-      <c r="O70" s="56"/>
-      <c r="P70" s="56"/>
-      <c r="Q70" s="79"/>
+      <c r="B70" s="89"/>
+      <c r="C70" s="89"/>
+      <c r="D70" s="89"/>
+      <c r="E70" s="89"/>
+      <c r="F70" s="89"/>
+      <c r="G70" s="89"/>
+      <c r="H70" s="89"/>
+      <c r="I70" s="89"/>
+      <c r="J70" s="89"/>
+      <c r="K70" s="89"/>
+      <c r="L70" s="89"/>
+      <c r="M70" s="89"/>
+      <c r="N70" s="89"/>
+      <c r="O70" s="89"/>
+      <c r="P70" s="89"/>
+      <c r="Q70" s="90"/>
     </row>
     <row r="71" spans="1:17" ht="18" customHeight="1">
-      <c r="A71" s="57"/>
-      <c r="B71" s="58"/>
-      <c r="C71" s="58"/>
-      <c r="D71" s="58"/>
-      <c r="E71" s="58"/>
-      <c r="F71" s="58"/>
-      <c r="G71" s="58"/>
-      <c r="H71" s="58"/>
-      <c r="I71" s="58"/>
-      <c r="J71" s="58"/>
-      <c r="K71" s="58"/>
-      <c r="L71" s="58"/>
-      <c r="M71" s="58"/>
-      <c r="N71" s="58"/>
-      <c r="O71" s="58"/>
-      <c r="P71" s="58"/>
-      <c r="Q71" s="80"/>
+      <c r="A71" s="94"/>
+      <c r="B71" s="95"/>
+      <c r="C71" s="95"/>
+      <c r="D71" s="95"/>
+      <c r="E71" s="95"/>
+      <c r="F71" s="95"/>
+      <c r="G71" s="95"/>
+      <c r="H71" s="95"/>
+      <c r="I71" s="95"/>
+      <c r="J71" s="95"/>
+      <c r="K71" s="95"/>
+      <c r="L71" s="95"/>
+      <c r="M71" s="95"/>
+      <c r="N71" s="95"/>
+      <c r="O71" s="95"/>
+      <c r="P71" s="95"/>
+      <c r="Q71" s="96"/>
     </row>
     <row r="72" spans="1:17" ht="18" customHeight="1">
-      <c r="A72" s="81"/>
-      <c r="B72" s="82"/>
-      <c r="C72" s="82"/>
-      <c r="D72" s="82"/>
-      <c r="E72" s="82"/>
-      <c r="F72" s="82"/>
-      <c r="G72" s="82"/>
-      <c r="H72" s="82"/>
-      <c r="I72" s="82"/>
-      <c r="J72" s="82"/>
-      <c r="K72" s="82"/>
-      <c r="L72" s="82"/>
-      <c r="M72" s="82"/>
-      <c r="N72" s="82"/>
-      <c r="O72" s="82"/>
-      <c r="P72" s="82"/>
-      <c r="Q72" s="83"/>
-    </row>
-    <row r="73" spans="1:17">
-      <c r="A73" s="87" t="s">
+      <c r="A72" s="100"/>
+      <c r="B72" s="101"/>
+      <c r="C72" s="101"/>
+      <c r="D72" s="101"/>
+      <c r="E72" s="101"/>
+      <c r="F72" s="101"/>
+      <c r="G72" s="101"/>
+      <c r="H72" s="101"/>
+      <c r="I72" s="101"/>
+      <c r="J72" s="101"/>
+      <c r="K72" s="101"/>
+      <c r="L72" s="101"/>
+      <c r="M72" s="101"/>
+      <c r="N72" s="101"/>
+      <c r="O72" s="101"/>
+      <c r="P72" s="101"/>
+      <c r="Q72" s="102"/>
+    </row>
+    <row r="73" spans="1:17" ht="12.75">
+      <c r="A73" s="76" t="s">
         <v>218</v>
       </c>
-      <c r="B73" s="54"/>
-      <c r="C73" s="54"/>
-      <c r="D73" s="54"/>
-      <c r="E73" s="54"/>
-      <c r="F73" s="54"/>
-      <c r="G73" s="54"/>
-      <c r="H73" s="54"/>
-      <c r="I73" s="54"/>
-      <c r="J73" s="54"/>
-      <c r="K73" s="54"/>
-      <c r="L73" s="54"/>
-      <c r="M73" s="54"/>
-      <c r="N73" s="54"/>
-      <c r="O73" s="54"/>
-      <c r="P73" s="54"/>
-      <c r="Q73" s="72"/>
-    </row>
-    <row r="74" spans="1:17" ht="15">
-      <c r="A74" s="84" t="s">
+      <c r="B73" s="105"/>
+      <c r="C73" s="105"/>
+      <c r="D73" s="105"/>
+      <c r="E73" s="105"/>
+      <c r="F73" s="105"/>
+      <c r="G73" s="105"/>
+      <c r="H73" s="105"/>
+      <c r="I73" s="105"/>
+      <c r="J73" s="105"/>
+      <c r="K73" s="105"/>
+      <c r="L73" s="105"/>
+      <c r="M73" s="105"/>
+      <c r="N73" s="105"/>
+      <c r="O73" s="105"/>
+      <c r="P73" s="105"/>
+      <c r="Q73" s="104"/>
+    </row>
+    <row r="74" spans="1:17" ht="30">
+      <c r="A74" s="53" t="s">
         <v>156</v>
       </c>
-      <c r="B74" s="72"/>
-      <c r="C74" s="88"/>
-      <c r="D74" s="74"/>
-      <c r="E74" s="74"/>
-      <c r="F74" s="74"/>
-      <c r="G74" s="74"/>
-      <c r="H74" s="74"/>
-      <c r="I74" s="75"/>
-      <c r="J74" s="40" t="s">
+      <c r="B74" s="104"/>
+      <c r="C74" s="68"/>
+      <c r="D74" s="111"/>
+      <c r="E74" s="111"/>
+      <c r="F74" s="111"/>
+      <c r="G74" s="111"/>
+      <c r="H74" s="111"/>
+      <c r="I74" s="112"/>
+      <c r="J74" s="126" t="s">
         <v>152</v>
       </c>
-      <c r="K74" s="85"/>
-      <c r="L74" s="74"/>
-      <c r="M74" s="74"/>
-      <c r="N74" s="74"/>
-      <c r="O74" s="74"/>
-      <c r="P74" s="74"/>
-      <c r="Q74" s="75"/>
-    </row>
-    <row r="75" spans="1:17" ht="15">
-      <c r="A75" s="84" t="s">
+      <c r="K74" s="59"/>
+      <c r="L74" s="111"/>
+      <c r="M74" s="111"/>
+      <c r="N74" s="111"/>
+      <c r="O74" s="111"/>
+      <c r="P74" s="111"/>
+      <c r="Q74" s="112"/>
+    </row>
+    <row r="75" spans="1:17" ht="30">
+      <c r="A75" s="53" t="s">
         <v>156</v>
       </c>
-      <c r="B75" s="72"/>
-      <c r="C75" s="85"/>
-      <c r="D75" s="74"/>
-      <c r="E75" s="74"/>
-      <c r="F75" s="74"/>
-      <c r="G75" s="74"/>
-      <c r="H75" s="74"/>
-      <c r="I75" s="75"/>
-      <c r="J75" s="40" t="s">
+      <c r="B75" s="104"/>
+      <c r="C75" s="59"/>
+      <c r="D75" s="111"/>
+      <c r="E75" s="111"/>
+      <c r="F75" s="111"/>
+      <c r="G75" s="111"/>
+      <c r="H75" s="111"/>
+      <c r="I75" s="112"/>
+      <c r="J75" s="126" t="s">
         <v>152</v>
       </c>
-      <c r="K75" s="85"/>
-      <c r="L75" s="74"/>
-      <c r="M75" s="74"/>
-      <c r="N75" s="74"/>
-      <c r="O75" s="74"/>
-      <c r="P75" s="74"/>
-      <c r="Q75" s="75"/>
-    </row>
-    <row r="76" spans="1:17" ht="15">
-      <c r="A76" s="84" t="s">
+      <c r="K75" s="59"/>
+      <c r="L75" s="111"/>
+      <c r="M75" s="111"/>
+      <c r="N75" s="111"/>
+      <c r="O75" s="111"/>
+      <c r="P75" s="111"/>
+      <c r="Q75" s="112"/>
+    </row>
+    <row r="76" spans="1:17" ht="30">
+      <c r="A76" s="53" t="s">
         <v>156</v>
       </c>
-      <c r="B76" s="72"/>
-      <c r="C76" s="85"/>
-      <c r="D76" s="74"/>
-      <c r="E76" s="74"/>
-      <c r="F76" s="74"/>
-      <c r="G76" s="74"/>
-      <c r="H76" s="74"/>
-      <c r="I76" s="75"/>
-      <c r="J76" s="40" t="s">
+      <c r="B76" s="104"/>
+      <c r="C76" s="59"/>
+      <c r="D76" s="111"/>
+      <c r="E76" s="111"/>
+      <c r="F76" s="111"/>
+      <c r="G76" s="111"/>
+      <c r="H76" s="111"/>
+      <c r="I76" s="112"/>
+      <c r="J76" s="126" t="s">
         <v>152</v>
       </c>
-      <c r="K76" s="85"/>
-      <c r="L76" s="74"/>
-      <c r="M76" s="74"/>
-      <c r="N76" s="74"/>
-      <c r="O76" s="74"/>
-      <c r="P76" s="74"/>
-      <c r="Q76" s="75"/>
+      <c r="K76" s="59"/>
+      <c r="L76" s="111"/>
+      <c r="M76" s="111"/>
+      <c r="N76" s="111"/>
+      <c r="O76" s="111"/>
+      <c r="P76" s="111"/>
+      <c r="Q76" s="112"/>
     </row>
     <row r="77" spans="1:17" ht="12.75">
-      <c r="A77" s="86" t="s">
+      <c r="A77" s="127" t="s">
         <v>157</v>
       </c>
-      <c r="B77" s="54"/>
-      <c r="C77" s="54"/>
-      <c r="D77" s="54"/>
-      <c r="E77" s="54"/>
-      <c r="F77" s="54"/>
-      <c r="G77" s="54"/>
-      <c r="H77" s="54"/>
-      <c r="I77" s="54"/>
-      <c r="J77" s="54"/>
-      <c r="K77" s="54"/>
-      <c r="L77" s="54"/>
-      <c r="M77" s="54"/>
-      <c r="N77" s="54"/>
-      <c r="O77" s="54"/>
-      <c r="P77" s="54"/>
-      <c r="Q77" s="72"/>
+      <c r="B77" s="105"/>
+      <c r="C77" s="105"/>
+      <c r="D77" s="105"/>
+      <c r="E77" s="105"/>
+      <c r="F77" s="105"/>
+      <c r="G77" s="105"/>
+      <c r="H77" s="105"/>
+      <c r="I77" s="105"/>
+      <c r="J77" s="105"/>
+      <c r="K77" s="105"/>
+      <c r="L77" s="105"/>
+      <c r="M77" s="105"/>
+      <c r="N77" s="105"/>
+      <c r="O77" s="105"/>
+      <c r="P77" s="105"/>
+      <c r="Q77" s="104"/>
     </row>
   </sheetData>
   <mergeCells count="164">
-    <mergeCell ref="L13:Q13"/>
-    <mergeCell ref="A14:Q14"/>
-    <mergeCell ref="A15:Q15"/>
-    <mergeCell ref="A16:J16"/>
-    <mergeCell ref="K16:N16"/>
-    <mergeCell ref="O16:Q17"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="L17:N17"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="D13:I13"/>
-    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A59:F63"/>
+    <mergeCell ref="G59:K63"/>
+    <mergeCell ref="A64:F65"/>
+    <mergeCell ref="G64:K65"/>
+    <mergeCell ref="A66:F67"/>
+    <mergeCell ref="G66:K67"/>
+    <mergeCell ref="A49:F50"/>
+    <mergeCell ref="A51:F52"/>
+    <mergeCell ref="G51:K52"/>
+    <mergeCell ref="A53:F54"/>
+    <mergeCell ref="G53:K54"/>
+    <mergeCell ref="G55:K56"/>
+    <mergeCell ref="A57:Q57"/>
+    <mergeCell ref="G58:K58"/>
+    <mergeCell ref="L58:Q58"/>
+    <mergeCell ref="L59:Q59"/>
+    <mergeCell ref="L60:Q60"/>
+    <mergeCell ref="L61:Q61"/>
+    <mergeCell ref="L62:Q62"/>
+    <mergeCell ref="M63:Q63"/>
+    <mergeCell ref="M52:Q52"/>
+    <mergeCell ref="L53:Q53"/>
+    <mergeCell ref="M54:Q54"/>
+    <mergeCell ref="L55:Q55"/>
+    <mergeCell ref="M56:Q56"/>
+    <mergeCell ref="A47:F48"/>
+    <mergeCell ref="G47:K48"/>
+    <mergeCell ref="L47:Q47"/>
+    <mergeCell ref="M48:Q48"/>
+    <mergeCell ref="G49:K50"/>
+    <mergeCell ref="L49:Q49"/>
+    <mergeCell ref="M50:Q50"/>
+    <mergeCell ref="A55:F56"/>
+    <mergeCell ref="A69:Q69"/>
+    <mergeCell ref="A70:Q72"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="C76:I76"/>
+    <mergeCell ref="K76:Q76"/>
+    <mergeCell ref="A77:Q77"/>
+    <mergeCell ref="A73:Q73"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="C74:I74"/>
+    <mergeCell ref="K74:Q74"/>
+    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="C75:I75"/>
+    <mergeCell ref="K75:Q75"/>
+    <mergeCell ref="A32:F33"/>
+    <mergeCell ref="G32:K33"/>
+    <mergeCell ref="A34:F38"/>
+    <mergeCell ref="G34:K38"/>
+    <mergeCell ref="L64:Q64"/>
+    <mergeCell ref="M65:Q65"/>
+    <mergeCell ref="L66:Q66"/>
+    <mergeCell ref="M67:Q67"/>
+    <mergeCell ref="A68:Q68"/>
+    <mergeCell ref="A39:F42"/>
+    <mergeCell ref="G39:K42"/>
+    <mergeCell ref="L39:Q39"/>
+    <mergeCell ref="L40:Q40"/>
+    <mergeCell ref="L41:Q41"/>
+    <mergeCell ref="M42:Q42"/>
+    <mergeCell ref="A43:Q43"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="L44:Q44"/>
+    <mergeCell ref="A45:F46"/>
+    <mergeCell ref="G45:K46"/>
+    <mergeCell ref="L45:Q45"/>
+    <mergeCell ref="M46:Q46"/>
+    <mergeCell ref="L51:Q51"/>
+    <mergeCell ref="A25:Q25"/>
+    <mergeCell ref="A26:Q26"/>
+    <mergeCell ref="A27:Q27"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="L29:Q29"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:F31"/>
+    <mergeCell ref="G30:K31"/>
+    <mergeCell ref="O20:Q20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="L22:N22"/>
+    <mergeCell ref="O22:P22"/>
+    <mergeCell ref="A23:Q23"/>
+    <mergeCell ref="N24:Q24"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="L37:Q37"/>
+    <mergeCell ref="M38:Q38"/>
+    <mergeCell ref="L30:Q30"/>
+    <mergeCell ref="M31:Q31"/>
+    <mergeCell ref="L32:Q32"/>
+    <mergeCell ref="M33:Q33"/>
+    <mergeCell ref="L34:Q34"/>
+    <mergeCell ref="L35:Q35"/>
+    <mergeCell ref="L36:Q36"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="L10:Q10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:I11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="L12:Q12"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="C18:G18"/>
     <mergeCell ref="H18:J18"/>
@@ -14461,133 +14555,19 @@
     <mergeCell ref="J11:K11"/>
     <mergeCell ref="L11:Q11"/>
     <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:I10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="L10:Q10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:I11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D12:I12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="L12:Q12"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="L37:Q37"/>
-    <mergeCell ref="M38:Q38"/>
-    <mergeCell ref="L30:Q30"/>
-    <mergeCell ref="M31:Q31"/>
-    <mergeCell ref="L32:Q32"/>
-    <mergeCell ref="M33:Q33"/>
-    <mergeCell ref="L34:Q34"/>
-    <mergeCell ref="L35:Q35"/>
-    <mergeCell ref="L36:Q36"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="O20:Q20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="G24:K24"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="F22:I22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="L22:N22"/>
-    <mergeCell ref="O22:P22"/>
-    <mergeCell ref="A23:Q23"/>
-    <mergeCell ref="N24:Q24"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A25:Q25"/>
-    <mergeCell ref="A26:Q26"/>
-    <mergeCell ref="A27:Q27"/>
-    <mergeCell ref="A28:Q28"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="L29:Q29"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A30:F31"/>
-    <mergeCell ref="G30:K31"/>
-    <mergeCell ref="A32:F33"/>
-    <mergeCell ref="G32:K33"/>
-    <mergeCell ref="A34:F38"/>
-    <mergeCell ref="G34:K38"/>
-    <mergeCell ref="L64:Q64"/>
-    <mergeCell ref="M65:Q65"/>
-    <mergeCell ref="L66:Q66"/>
-    <mergeCell ref="M67:Q67"/>
-    <mergeCell ref="A68:Q68"/>
-    <mergeCell ref="A39:F42"/>
-    <mergeCell ref="G39:K42"/>
-    <mergeCell ref="L39:Q39"/>
-    <mergeCell ref="L40:Q40"/>
-    <mergeCell ref="L41:Q41"/>
-    <mergeCell ref="M42:Q42"/>
-    <mergeCell ref="A43:Q43"/>
-    <mergeCell ref="A44:F44"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="L44:Q44"/>
-    <mergeCell ref="A45:F46"/>
-    <mergeCell ref="G45:K46"/>
-    <mergeCell ref="L45:Q45"/>
-    <mergeCell ref="M46:Q46"/>
-    <mergeCell ref="L51:Q51"/>
-    <mergeCell ref="A69:Q69"/>
-    <mergeCell ref="A70:Q72"/>
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="C76:I76"/>
-    <mergeCell ref="K76:Q76"/>
-    <mergeCell ref="A77:Q77"/>
-    <mergeCell ref="A73:Q73"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="C74:I74"/>
-    <mergeCell ref="K74:Q74"/>
-    <mergeCell ref="A75:B75"/>
-    <mergeCell ref="C75:I75"/>
-    <mergeCell ref="K75:Q75"/>
-    <mergeCell ref="L55:Q55"/>
-    <mergeCell ref="M56:Q56"/>
-    <mergeCell ref="A47:F48"/>
-    <mergeCell ref="G47:K48"/>
-    <mergeCell ref="L47:Q47"/>
-    <mergeCell ref="M48:Q48"/>
-    <mergeCell ref="G49:K50"/>
-    <mergeCell ref="L49:Q49"/>
-    <mergeCell ref="M50:Q50"/>
-    <mergeCell ref="A55:F56"/>
-    <mergeCell ref="A58:F58"/>
-    <mergeCell ref="A59:F63"/>
-    <mergeCell ref="G59:K63"/>
-    <mergeCell ref="A64:F65"/>
-    <mergeCell ref="G64:K65"/>
-    <mergeCell ref="A66:F67"/>
-    <mergeCell ref="G66:K67"/>
-    <mergeCell ref="A49:F50"/>
-    <mergeCell ref="A51:F52"/>
-    <mergeCell ref="G51:K52"/>
-    <mergeCell ref="A53:F54"/>
-    <mergeCell ref="G53:K54"/>
-    <mergeCell ref="G55:K56"/>
-    <mergeCell ref="A57:Q57"/>
-    <mergeCell ref="G58:K58"/>
-    <mergeCell ref="L58:Q58"/>
-    <mergeCell ref="L59:Q59"/>
-    <mergeCell ref="L60:Q60"/>
-    <mergeCell ref="L61:Q61"/>
-    <mergeCell ref="L62:Q62"/>
-    <mergeCell ref="M63:Q63"/>
-    <mergeCell ref="M52:Q52"/>
-    <mergeCell ref="L53:Q53"/>
-    <mergeCell ref="M54:Q54"/>
+    <mergeCell ref="L13:Q13"/>
+    <mergeCell ref="A14:Q14"/>
+    <mergeCell ref="A15:Q15"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="K16:N16"/>
+    <mergeCell ref="O16:Q17"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:I13"/>
+    <mergeCell ref="J13:K13"/>
   </mergeCells>
   <dataValidations count="25">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L39" xr:uid="{00000000-0002-0000-0800-000000000000}">
@@ -14667,5 +14647,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>